<commit_message>
Prepare bladder data and parameters
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEC751A0-91DD-5C4A-8C6F-D42A1B6E577C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68D08D95-55D9-6C41-8920-6AF5B6CBDEDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8640" yWindow="760" windowWidth="21600" windowHeight="17760" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="17760" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="37">
   <si>
     <t>target_names</t>
   </si>
@@ -142,6 +142,12 @@
   </si>
   <si>
     <t>Divided by years</t>
+  </si>
+  <si>
+    <t>n_cases_lb</t>
+  </si>
+  <si>
+    <t>n_cases_ub</t>
   </si>
 </sst>
 </file>
@@ -701,15 +707,15 @@
       </c>
       <c r="F5" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A5,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.1</v>
+        <v>5.0435854467200008</v>
       </c>
       <c r="G5" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A5,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>4.7539481057578041E-2</v>
+        <v>0.1</v>
       </c>
       <c r="H5" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A5,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.18231431028870138</v>
+        <v>1.6241209331261943E-3</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>21</v>
@@ -736,15 +742,15 @@
       </c>
       <c r="F6" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A6,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.1</v>
+        <v>5.8673742561799997</v>
       </c>
       <c r="G6" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A6,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>4.9803163272485546E-2</v>
+        <v>0.1</v>
       </c>
       <c r="H6" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A6,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.17318849687090868</v>
+        <v>0</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>21</v>
@@ -770,16 +776,16 @@
         <v>12</v>
       </c>
       <c r="F7" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A7,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>0</v>
       </c>
       <c r="G7" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A7,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
         <v>0</v>
       </c>
       <c r="H7" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A7,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>3.0175692110998593E-2</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.10682882759847878</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>21</v>
@@ -805,16 +811,16 @@
         <v>17</v>
       </c>
       <c r="F8" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A8,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>0.1</v>
       </c>
       <c r="G8" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A8,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>4.8967550470348217E-2</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>1.7013511956265843E-2</v>
       </c>
       <c r="H8" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A8,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.17551503685994646</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.23722104989583823</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>21</v>
@@ -840,16 +846,16 @@
         <v>22</v>
       </c>
       <c r="F9" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A9,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>0.3</v>
       </c>
       <c r="G9" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A9,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.19751025653517687</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>0.1597383882900868</v>
       </c>
       <c r="H9" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A9,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.42651643305256426</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.4874889418786299</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>21</v>
@@ -875,16 +881,16 @@
         <v>27</v>
       </c>
       <c r="F10" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A10,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>0.5</v>
       </c>
       <c r="G10" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A10,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.35526951495750414</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>0.31289158139055295</v>
       </c>
       <c r="H10" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A10,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.68003739631611393</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.73811868911234746</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>21</v>
@@ -910,16 +916,16 @@
         <v>32</v>
       </c>
       <c r="F11" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A11,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>1.1000000000000001</v>
       </c>
       <c r="G11" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A11,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.85790278004408504</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>0.8184299276747744</v>
       </c>
       <c r="H11" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A11,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>1.3738737008883275</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>1.4317978530233426</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>21</v>
@@ -945,16 +951,16 @@
         <v>37</v>
       </c>
       <c r="F12" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A12,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>2.2000000000000002</v>
       </c>
       <c r="G12" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A12,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>1.8524198567476291</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>1.8032433025804822</v>
       </c>
       <c r="H12" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A12,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>2.5875314992726337</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>2.6371938700704867</v>
       </c>
       <c r="I12" s="1" t="s">
         <v>21</v>
@@ -980,16 +986,16 @@
         <v>42</v>
       </c>
       <c r="F13" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A13,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>4.3</v>
       </c>
       <c r="G13" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A13,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>3.8234796326099518</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>3.7766078728748678</v>
       </c>
       <c r="H13" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A13,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>4.8059210133790522</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>4.8583883346410159</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>21</v>
@@ -1015,16 +1021,16 @@
         <v>47</v>
       </c>
       <c r="F14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>9.5</v>
       </c>
       <c r="G14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>8.793324890769302</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>8.7460518806358838</v>
       </c>
       <c r="H14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>10.238774118895414</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>10.289748213803048</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>21</v>
@@ -1050,16 +1056,16 @@
         <v>52</v>
       </c>
       <c r="F15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>18.5</v>
       </c>
       <c r="G15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>17.464539591211235</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>17.419890817649691</v>
       </c>
       <c r="H15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>19.56627052268988</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>19.621383584718842</v>
       </c>
       <c r="I15" s="1" t="s">
         <v>21</v>
@@ -1085,16 +1091,16 @@
         <v>57</v>
       </c>
       <c r="F16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>34.299999999999997</v>
       </c>
       <c r="G16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>32.809192393527404</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>32.767494120937265</v>
       </c>
       <c r="H16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>35.824002291641719</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>35.876275809580278</v>
       </c>
       <c r="I16" s="1" t="s">
         <v>21</v>
@@ -1120,16 +1126,16 @@
         <v>62</v>
       </c>
       <c r="F17" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A17,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>52.9</v>
       </c>
       <c r="G17" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A17,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>50.908689766881942</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>50.860284058021669</v>
       </c>
       <c r="H17" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A17,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>54.933684552221493</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>54.983958159669321</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>21</v>
@@ -1155,16 +1161,16 @@
         <v>67</v>
       </c>
       <c r="F18" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A18,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>82.8</v>
       </c>
       <c r="G18" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A18,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>80.037972220862599</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>79.990143004942581</v>
       </c>
       <c r="H18" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A18,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>85.625368578947473</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>85.674831914507308</v>
       </c>
       <c r="I18" s="1" t="s">
         <v>21</v>
@@ -1190,16 +1196,16 @@
         <v>72</v>
       </c>
       <c r="F19" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A19,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>109.1</v>
       </c>
       <c r="G19" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A19,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>105.49858059568955</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>105.45249909757202</v>
       </c>
       <c r="H19" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A19,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>112.7664147932736</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>112.82992889659357</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>21</v>
@@ -1225,16 +1231,16 @@
         <v>77</v>
       </c>
       <c r="F20" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A20,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>132.19999999999999</v>
       </c>
       <c r="G20" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A20,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>127.49381844285837</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>127.42849266253278</v>
       </c>
       <c r="H20" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A20,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>137.02984726186881</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>137.07498967213519</v>
       </c>
       <c r="I20" s="1" t="s">
         <v>21</v>
@@ -1260,16 +1266,16 @@
         <v>82</v>
       </c>
       <c r="F21" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A21,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>149.30000000000001</v>
       </c>
       <c r="G21" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A21,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>142.80449784276743</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>142.7680888200511</v>
       </c>
       <c r="H21" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A21,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>155.94729853228347</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>156.02337488989809</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>21</v>
@@ -1294,16 +1300,16 @@
         <v>92</v>
       </c>
       <c r="F22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
         <v>141.69999999999999</v>
       </c>
       <c r="G22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>133.9345885509004</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>133.87986472565848</v>
       </c>
       <c r="H22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>149.70149822623048</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>149.75933097441057</v>
       </c>
       <c r="I22" s="1" t="s">
         <v>21</v>
@@ -1803,15 +1809,21 @@
         <v>12</v>
       </c>
       <c r="I23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K23" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="J23" s="1" t="s">
+      <c r="L23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="M23" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="L23" s="1" t="s">
+      <c r="N23" s="1" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1837,27 +1849,35 @@
         <v>84416</v>
       </c>
       <c r="G24" s="1">
-        <f>F24/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" ref="G24:G41" si="13">F24/$B$16*$B$17*($B$19-$B$18+1)</f>
         <v>10087170.893440001</v>
       </c>
       <c r="H24" s="1">
-        <f>I24*G24/$B$20</f>
+        <f>K24*G24/$B$20</f>
         <v>10.087170893440002</v>
       </c>
       <c r="I24" s="1">
+        <f>MAX(0, K24-0.05)*G24/$B$20</f>
+        <v>5.0435854467200008</v>
+      </c>
+      <c r="J24" s="1">
+        <f>(K24+0.05)*G24/$B$20</f>
+        <v>15.130756340160005</v>
+      </c>
+      <c r="K24" s="1">
         <v>0.1</v>
       </c>
-      <c r="J24" s="1">
+      <c r="L24" s="1">
         <f>SUM(H24:H27)/H42</f>
         <v>1.6241209331261943E-3</v>
       </c>
-      <c r="K24" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H24)/$G24*$B$20, 0)</f>
-        <v>4.7539481057578041E-2</v>
-      </c>
-      <c r="L24" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H24+1))/$G24*$B$20, 0)</f>
-        <v>0.18231431028870138</v>
+      <c r="M24" s="1">
+        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*I24)/$G24*$B$20, 0)</f>
+        <v>1.6094566130273689E-2</v>
+      </c>
+      <c r="N24" s="1">
+        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($J24+1))/$G24*$B$20, 0)</f>
+        <v>0.24526419878119815</v>
       </c>
     </row>
     <row r="25" spans="1:24">
@@ -1883,23 +1903,31 @@
         <v>98204</v>
       </c>
       <c r="G25" s="1">
-        <f>F25/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>11734748.512359999</v>
       </c>
       <c r="H25" s="1">
-        <f>I25*G25/$B$20</f>
+        <f>K25*G25/$B$20</f>
         <v>11.734748512359999</v>
       </c>
       <c r="I25" s="1">
+        <f t="shared" ref="I25:I42" si="14">MAX(0, K25-0.05)*G25/$B$20</f>
+        <v>5.8673742561799997</v>
+      </c>
+      <c r="J25" s="1">
+        <f t="shared" ref="J25:J41" si="15">(K25+0.05)*G25/$B$20</f>
+        <v>17.602122768539999</v>
+      </c>
+      <c r="K25" s="1">
         <v>0.1</v>
       </c>
-      <c r="K25" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H25)/$G25*$B$20, 0)</f>
-        <v>4.9803163272485546E-2</v>
-      </c>
-      <c r="L25" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H25+1))/$G25*$B$20, 0)</f>
-        <v>0.17318849687090868</v>
+      <c r="M25" s="1">
+        <f t="shared" ref="M25:M41" si="16">IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*I25)/$G25*$B$20, 0)</f>
+        <v>1.6258329900368296E-2</v>
+      </c>
+      <c r="N25" s="1">
+        <f t="shared" ref="N25:N41" si="17">IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($J25+1))/$G25*$B$20, 0)</f>
+        <v>0.23719286870795328</v>
       </c>
     </row>
     <row r="26" spans="1:24">
@@ -1914,7 +1942,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="1">
-        <f t="shared" ref="D26:D40" si="13">C27</f>
+        <f t="shared" ref="D26:D40" si="18">C27</f>
         <v>15</v>
       </c>
       <c r="E26" s="1">
@@ -1925,23 +1953,31 @@
         <v>102304</v>
       </c>
       <c r="G26" s="1">
-        <f>F26/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>12224672.231360001</v>
       </c>
       <c r="H26" s="1">
-        <f>I26*G26/$B$20</f>
+        <f>K26*G26/$B$20</f>
         <v>0</v>
       </c>
       <c r="I26" s="1">
+        <f t="shared" si="14"/>
         <v>0</v>
       </c>
+      <c r="J26" s="1">
+        <f t="shared" si="15"/>
+        <v>6.1123361156800007</v>
+      </c>
       <c r="K26" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H26)/$G26*$B$20, 0)</f>
         <v>0</v>
       </c>
-      <c r="L26" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H26+1))/$G26*$B$20, 0)</f>
-        <v>3.0175692110998593E-2</v>
+      <c r="M26" s="1">
+        <f t="shared" si="16"/>
+        <v>0</v>
+      </c>
+      <c r="N26" s="1">
+        <f t="shared" si="17"/>
+        <v>0.10682882759847878</v>
       </c>
     </row>
     <row r="27" spans="1:24">
@@ -1956,7 +1992,7 @@
         <v>15</v>
       </c>
       <c r="D27" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>20</v>
       </c>
       <c r="E27" s="1">
@@ -1967,23 +2003,31 @@
         <v>93845</v>
       </c>
       <c r="G27" s="1">
-        <f>F27/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>11213875.95355</v>
       </c>
       <c r="H27" s="1">
-        <f>I27*G27/$B$20</f>
+        <f>K27*G27/$B$20</f>
         <v>11.213875953550001</v>
       </c>
       <c r="I27" s="1">
+        <f t="shared" si="14"/>
+        <v>5.6069379767750007</v>
+      </c>
+      <c r="J27" s="1">
+        <f t="shared" si="15"/>
+        <v>16.820813930325002</v>
+      </c>
+      <c r="K27" s="1">
         <v>0.1</v>
       </c>
-      <c r="K27" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H27)/$G27*$B$20, 0)</f>
-        <v>4.8967550470348217E-2</v>
-      </c>
-      <c r="L27" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H27+1))/$G27*$B$20, 0)</f>
-        <v>0.17551503685994646</v>
+      <c r="M27" s="1">
+        <f t="shared" si="16"/>
+        <v>1.7013511956265843E-2</v>
+      </c>
+      <c r="N27" s="1">
+        <f t="shared" si="17"/>
+        <v>0.23722104989583823</v>
       </c>
     </row>
     <row r="28" spans="1:24">
@@ -1998,7 +2042,7 @@
         <v>20</v>
       </c>
       <c r="D28" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>25</v>
       </c>
       <c r="E28" s="1">
@@ -2009,27 +2053,35 @@
         <v>80561</v>
       </c>
       <c r="G28" s="1">
-        <f>F28/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>9626523.1039899997</v>
       </c>
       <c r="H28" s="1">
-        <f>I28*G28/$B$20</f>
+        <f>K28*G28/$B$20</f>
         <v>28.879569311969998</v>
       </c>
       <c r="I28" s="1">
+        <f t="shared" si="14"/>
+        <v>24.066307759975</v>
+      </c>
+      <c r="J28" s="1">
+        <f t="shared" si="15"/>
+        <v>33.692830863964993</v>
+      </c>
+      <c r="K28" s="1">
         <v>0.3</v>
       </c>
-      <c r="J28" s="1">
+      <c r="L28" s="1">
         <f>SUM(H28:H30)/H42</f>
         <v>7.0026509067945388E-3</v>
       </c>
-      <c r="K28" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H28)/$G28*$B$20, 0)</f>
-        <v>0.19751025653517687</v>
-      </c>
-      <c r="L28" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H28+1))/$G28*$B$20, 0)</f>
-        <v>0.42651643305256426</v>
+      <c r="M28" s="1">
+        <f t="shared" si="16"/>
+        <v>0.1597383882900868</v>
+      </c>
+      <c r="N28" s="1">
+        <f t="shared" si="17"/>
+        <v>0.4874889418786299</v>
       </c>
     </row>
     <row r="29" spans="1:24">
@@ -2044,7 +2096,7 @@
         <v>25</v>
       </c>
       <c r="D29" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>30</v>
       </c>
       <c r="E29" s="1">
@@ -2055,23 +2107,31 @@
         <v>66320</v>
       </c>
       <c r="G29" s="1">
-        <f>F29/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>7924814.8888000008</v>
       </c>
       <c r="H29" s="1">
-        <f>I29*G29/$B$20</f>
+        <f>K29*G29/$B$20</f>
         <v>39.624074444000001</v>
       </c>
       <c r="I29" s="1">
+        <f t="shared" si="14"/>
+        <v>35.661666999600001</v>
+      </c>
+      <c r="J29" s="1">
+        <f t="shared" si="15"/>
+        <v>43.586481888400009</v>
+      </c>
+      <c r="K29" s="1">
         <v>0.5</v>
       </c>
-      <c r="K29" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H29)/$G29*$B$20, 0)</f>
-        <v>0.35526951495750414</v>
-      </c>
-      <c r="L29" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H29+1))/$G29*$B$20, 0)</f>
-        <v>0.68003739631611393</v>
+      <c r="M29" s="1">
+        <f t="shared" si="16"/>
+        <v>0.31289158139055295</v>
+      </c>
+      <c r="N29" s="1">
+        <f t="shared" si="17"/>
+        <v>0.73811868911234746</v>
       </c>
     </row>
     <row r="30" spans="1:24">
@@ -2086,7 +2146,7 @@
         <v>30</v>
       </c>
       <c r="D30" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>35</v>
       </c>
       <c r="E30" s="1">
@@ -2097,23 +2157,31 @@
         <v>56249</v>
       </c>
       <c r="G30" s="1">
-        <f>F30/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>6721394.9439099999</v>
       </c>
       <c r="H30" s="1">
-        <f>I30*G30/$B$20</f>
+        <f>K30*G30/$B$20</f>
         <v>73.935344383010005</v>
       </c>
       <c r="I30" s="1">
+        <f t="shared" si="14"/>
+        <v>70.574646911054998</v>
+      </c>
+      <c r="J30" s="1">
+        <f t="shared" si="15"/>
+        <v>77.296041854965011</v>
+      </c>
+      <c r="K30" s="1">
         <v>1.1000000000000001</v>
       </c>
-      <c r="K30" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H30)/$G30*$B$20, 0)</f>
-        <v>0.85790278004408504</v>
-      </c>
-      <c r="L30" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H30+1))/$G30*$B$20, 0)</f>
-        <v>1.3738737008883275</v>
+      <c r="M30" s="1">
+        <f t="shared" si="16"/>
+        <v>0.8184299276747744</v>
+      </c>
+      <c r="N30" s="1">
+        <f t="shared" si="17"/>
+        <v>1.4317978530233426</v>
       </c>
     </row>
     <row r="31" spans="1:24">
@@ -2128,7 +2196,7 @@
         <v>35</v>
       </c>
       <c r="D31" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>40</v>
       </c>
       <c r="E31" s="1">
@@ -2139,27 +2207,35 @@
         <v>54656</v>
       </c>
       <c r="G31" s="1">
-        <f>F31/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>6531041.6550400006</v>
       </c>
       <c r="H31" s="1">
-        <f>I31*G31/$B$20</f>
+        <f>K31*G31/$B$20</f>
         <v>143.68291641088004</v>
       </c>
       <c r="I31" s="1">
+        <f t="shared" si="14"/>
+        <v>140.41739558336002</v>
+      </c>
+      <c r="J31" s="1">
+        <f t="shared" si="15"/>
+        <v>146.94843723840003</v>
+      </c>
+      <c r="K31" s="1">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J31" s="1">
+      <c r="L31" s="1">
         <f>SUM(H31:H32)/$H$42</f>
         <v>2.1957052888418878E-2</v>
       </c>
-      <c r="K31" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H31)/$G31*$B$20, 0)</f>
-        <v>1.8524198567476291</v>
-      </c>
-      <c r="L31" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H31+1))/$G31*$B$20, 0)</f>
-        <v>2.5875314992726337</v>
+      <c r="M31" s="1">
+        <f t="shared" si="16"/>
+        <v>1.8032433025804822</v>
+      </c>
+      <c r="N31" s="1">
+        <f t="shared" si="17"/>
+        <v>2.6371938700704867</v>
       </c>
     </row>
     <row r="32" spans="1:24">
@@ -2174,7 +2250,7 @@
         <v>40</v>
       </c>
       <c r="D32" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>45</v>
       </c>
       <c r="E32" s="1">
@@ -2185,26 +2261,34 @@
         <v>58958</v>
       </c>
       <c r="G32" s="1">
-        <f>F32/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>7045103.0792200007</v>
       </c>
       <c r="H32" s="1">
-        <f>I32*G32/$B$20</f>
+        <f>K32*G32/$B$20</f>
         <v>302.93943240646001</v>
       </c>
       <c r="I32" s="1">
+        <f t="shared" si="14"/>
+        <v>299.41688086685002</v>
+      </c>
+      <c r="J32" s="1">
+        <f t="shared" si="15"/>
+        <v>306.46198394607001</v>
+      </c>
+      <c r="K32" s="1">
         <v>4.3</v>
       </c>
-      <c r="K32" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H32)/$G32*$B$20, 0)</f>
-        <v>3.8234796326099518</v>
-      </c>
-      <c r="L32" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H32+1))/$G32*$B$20, 0)</f>
-        <v>4.8059210133790522</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12">
+      <c r="M32" s="1">
+        <f t="shared" si="16"/>
+        <v>3.7766078728748678</v>
+      </c>
+      <c r="N32" s="1">
+        <f t="shared" si="17"/>
+        <v>4.8583883346410159</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
       <c r="A33" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_47</v>
@@ -2216,7 +2300,7 @@
         <v>45</v>
       </c>
       <c r="D33" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>50</v>
       </c>
       <c r="E33" s="1">
@@ -2227,30 +2311,38 @@
         <v>59622</v>
       </c>
       <c r="G33" s="1">
-        <f>F33/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>7124446.8229799997</v>
       </c>
       <c r="H33" s="1">
-        <f>I33*G33/$B$20</f>
+        <f>K33*G33/$B$20</f>
         <v>676.82244818309994</v>
       </c>
       <c r="I33" s="1">
+        <f t="shared" si="14"/>
+        <v>673.26022477160996</v>
+      </c>
+      <c r="J33" s="1">
+        <f t="shared" si="15"/>
+        <v>680.38467159458992</v>
+      </c>
+      <c r="K33" s="1">
         <v>9.5</v>
       </c>
-      <c r="J33" s="1">
+      <c r="L33" s="1">
         <f>SUM(H33:H34)/$H$42</f>
         <v>9.2660309853476744E-2</v>
       </c>
-      <c r="K33" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H33)/$G33*$B$20, 0)</f>
-        <v>8.793324890769302</v>
-      </c>
-      <c r="L33" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H33+1))/$G33*$B$20, 0)</f>
-        <v>10.238774118895414</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12">
+      <c r="M33" s="1">
+        <f t="shared" si="16"/>
+        <v>8.7460518806358838</v>
+      </c>
+      <c r="N33" s="1">
+        <f t="shared" si="17"/>
+        <v>10.289748213803048</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
       <c r="A34" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_52</v>
@@ -2262,7 +2354,7 @@
         <v>50</v>
       </c>
       <c r="D34" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>55</v>
       </c>
       <c r="E34" s="1">
@@ -2273,26 +2365,34 @@
         <v>54643</v>
       </c>
       <c r="G34" s="1">
-        <f>F34/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>6529488.2383699995</v>
       </c>
       <c r="H34" s="1">
-        <f>I34*G34/$B$20</f>
+        <f>K34*G34/$B$20</f>
         <v>1207.9553240984499</v>
       </c>
       <c r="I34" s="1">
+        <f t="shared" si="14"/>
+        <v>1204.6905799792648</v>
+      </c>
+      <c r="J34" s="1">
+        <f t="shared" si="15"/>
+        <v>1211.2200682176351</v>
+      </c>
+      <c r="K34" s="1">
         <v>18.5</v>
       </c>
-      <c r="K34" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H34)/$G34*$B$20, 0)</f>
-        <v>17.464539591211235</v>
-      </c>
-      <c r="L34" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H34+1))/$G34*$B$20, 0)</f>
-        <v>19.56627052268988</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12">
+      <c r="M34" s="1">
+        <f t="shared" si="16"/>
+        <v>17.419890817649691</v>
+      </c>
+      <c r="N34" s="1">
+        <f t="shared" si="17"/>
+        <v>19.621383584718842</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
       <c r="A35" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_57</v>
@@ -2304,7 +2404,7 @@
         <v>55</v>
       </c>
       <c r="D35" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>60</v>
       </c>
       <c r="E35" s="1">
@@ -2315,30 +2415,38 @@
         <v>49077</v>
       </c>
       <c r="G35" s="1">
-        <f>F35/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>5864386.9164300002</v>
       </c>
       <c r="H35" s="1">
-        <f>I35*G35/$B$20</f>
+        <f>K35*G35/$B$20</f>
         <v>2011.48471233549</v>
       </c>
       <c r="I35" s="1">
+        <f t="shared" si="14"/>
+        <v>2008.5525188772749</v>
+      </c>
+      <c r="J35" s="1">
+        <f t="shared" si="15"/>
+        <v>2014.4169057937047</v>
+      </c>
+      <c r="K35" s="1">
         <v>34.299999999999997</v>
       </c>
-      <c r="J35" s="1">
+      <c r="L35" s="1">
         <f>SUM(H35:H36)/$H$42</f>
         <v>0.23066375686826504</v>
       </c>
-      <c r="K35" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H35)/$G35*$B$20, 0)</f>
-        <v>32.809192393527404</v>
-      </c>
-      <c r="L35" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H35+1))/$G35*$B$20, 0)</f>
-        <v>35.824002291641719</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12">
+      <c r="M35" s="1">
+        <f t="shared" si="16"/>
+        <v>32.767494120937265</v>
+      </c>
+      <c r="N35" s="1">
+        <f t="shared" si="17"/>
+        <v>35.876275809580278</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_62</v>
@@ -2350,7 +2458,7 @@
         <v>60</v>
       </c>
       <c r="D36" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>65</v>
       </c>
       <c r="E36" s="1">
@@ -2361,26 +2469,34 @@
         <v>42403</v>
       </c>
       <c r="G36" s="1">
-        <f>F36/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>5066886.6967700003</v>
       </c>
       <c r="H36" s="1">
-        <f>I36*G36/$B$20</f>
+        <f>K36*G36/$B$20</f>
         <v>2680.3830625913301</v>
       </c>
       <c r="I36" s="1">
+        <f t="shared" si="14"/>
+        <v>2677.8496192429452</v>
+      </c>
+      <c r="J36" s="1">
+        <f t="shared" si="15"/>
+        <v>2682.9165059397151</v>
+      </c>
+      <c r="K36" s="1">
         <v>52.9</v>
       </c>
-      <c r="K36" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H36)/$G36*$B$20, 0)</f>
-        <v>50.908689766881942</v>
-      </c>
-      <c r="L36" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H36+1))/$G36*$B$20, 0)</f>
-        <v>54.933684552221493</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12">
+      <c r="M36" s="1">
+        <f t="shared" si="16"/>
+        <v>50.860284058021669</v>
+      </c>
+      <c r="N36" s="1">
+        <f t="shared" si="17"/>
+        <v>54.983958159669321</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
       <c r="A37" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_67</v>
@@ -2392,7 +2508,7 @@
         <v>65</v>
       </c>
       <c r="D37" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>70</v>
       </c>
       <c r="E37" s="1">
@@ -2403,30 +2519,38 @@
         <v>34406</v>
       </c>
       <c r="G37" s="1">
-        <f>F37/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>4111296.4575399999</v>
       </c>
       <c r="H37" s="1">
-        <f>I37*G37/$B$20</f>
+        <f>K37*G37/$B$20</f>
         <v>3404.15346684312</v>
       </c>
       <c r="I37" s="1">
+        <f t="shared" si="14"/>
+        <v>3402.0978186143498</v>
+      </c>
+      <c r="J37" s="1">
+        <f t="shared" si="15"/>
+        <v>3406.2091150718898</v>
+      </c>
+      <c r="K37" s="1">
         <v>82.8</v>
       </c>
-      <c r="J37" s="1">
+      <c r="L37" s="1">
         <f>SUM(H37:H38)/$H$42</f>
         <v>0.33905227084581235</v>
       </c>
-      <c r="K37" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H37)/$G37*$B$20, 0)</f>
-        <v>80.037972220862599</v>
-      </c>
-      <c r="L37" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H37+1))/$G37*$B$20, 0)</f>
-        <v>85.625368578947473</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12">
+      <c r="M37" s="1">
+        <f t="shared" si="16"/>
+        <v>79.990143004942581</v>
+      </c>
+      <c r="N37" s="1">
+        <f t="shared" si="17"/>
+        <v>85.674831914507308</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
       <c r="A38" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_72</v>
@@ -2438,7 +2562,7 @@
         <v>70</v>
       </c>
       <c r="D38" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>75</v>
       </c>
       <c r="E38" s="1">
@@ -2449,26 +2573,34 @@
         <v>26789</v>
       </c>
       <c r="G38" s="1">
-        <f>F38/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>3201113.7825100003</v>
       </c>
       <c r="H38" s="1">
-        <f>I38*G38/$B$20</f>
+        <f>K38*G38/$B$20</f>
         <v>3492.4151367184104</v>
       </c>
       <c r="I38" s="1">
+        <f t="shared" si="14"/>
+        <v>3490.8145798271553</v>
+      </c>
+      <c r="J38" s="1">
+        <f t="shared" si="15"/>
+        <v>3494.015693609665</v>
+      </c>
+      <c r="K38" s="1">
         <v>109.1</v>
       </c>
-      <c r="K38" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H38)/$G38*$B$20, 0)</f>
-        <v>105.49858059568955</v>
-      </c>
-      <c r="L38" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H38+1))/$G38*$B$20, 0)</f>
-        <v>112.7664147932736</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12">
+      <c r="M38" s="1">
+        <f t="shared" si="16"/>
+        <v>105.45249909757202</v>
+      </c>
+      <c r="N38" s="1">
+        <f t="shared" si="17"/>
+        <v>112.82992889659357</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
       <c r="A39" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_77</v>
@@ -2480,7 +2612,7 @@
         <v>75</v>
       </c>
       <c r="D39" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>80</v>
       </c>
       <c r="E39" s="1">
@@ -2491,30 +2623,38 @@
         <v>18871</v>
       </c>
       <c r="G39" s="1">
-        <f>F39/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>2254963.5368899996</v>
       </c>
       <c r="H39" s="1">
-        <f>I39*G39/$B$20</f>
+        <f>K39*G39/$B$20</f>
         <v>2981.061795768579</v>
       </c>
       <c r="I39" s="1">
+        <f t="shared" si="14"/>
+        <v>2979.9343140001338</v>
+      </c>
+      <c r="J39" s="1">
+        <f t="shared" si="15"/>
+        <v>2982.1892775370247</v>
+      </c>
+      <c r="K39" s="1">
         <v>132.19999999999999</v>
       </c>
-      <c r="J39" s="1">
+      <c r="L39" s="1">
         <f>SUM(H39:H40)/$H$42</f>
         <v>0.24514861979857369</v>
       </c>
-      <c r="K39" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H39)/$G39*$B$20, 0)</f>
-        <v>127.49381844285837</v>
-      </c>
-      <c r="L39" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H39+1))/$G39*$B$20, 0)</f>
-        <v>137.02984726186881</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12">
+      <c r="M39" s="1">
+        <f t="shared" si="16"/>
+        <v>127.42849266253278</v>
+      </c>
+      <c r="N39" s="1">
+        <f t="shared" si="17"/>
+        <v>137.07498967213519</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_82</v>
@@ -2526,7 +2666,7 @@
         <v>80</v>
       </c>
       <c r="D40" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="18"/>
         <v>85</v>
       </c>
       <c r="E40" s="1">
@@ -2537,26 +2677,34 @@
         <v>11241</v>
       </c>
       <c r="G40" s="1">
-        <f>F40/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>1343227.4451899999</v>
       </c>
       <c r="H40" s="1">
-        <f>I40*G40/$B$20</f>
+        <f>K40*G40/$B$20</f>
         <v>2005.43857566867</v>
       </c>
       <c r="I40" s="1">
+        <f t="shared" si="14"/>
+        <v>2004.7669619460751</v>
+      </c>
+      <c r="J40" s="1">
+        <f t="shared" si="15"/>
+        <v>2006.1101893912653</v>
+      </c>
+      <c r="K40" s="1">
         <v>149.30000000000001</v>
       </c>
-      <c r="K40" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H40)/$G40*$B$20, 0)</f>
-        <v>142.80449784276743</v>
-      </c>
-      <c r="L40" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H40+1))/$G40*$B$20, 0)</f>
-        <v>155.94729853228347</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12">
+      <c r="M40" s="1">
+        <f t="shared" si="16"/>
+        <v>142.7680888200511</v>
+      </c>
+      <c r="N40" s="1">
+        <f t="shared" si="17"/>
+        <v>156.02337488989809</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
       <c r="A41" s="1" t="str">
         <f t="shared" si="11"/>
         <v>incidence_clin_92</v>
@@ -2578,30 +2726,38 @@
         <v>7435</v>
       </c>
       <c r="G41" s="1">
-        <f>F41/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <f t="shared" si="13"/>
         <v>888434.84165000007</v>
       </c>
       <c r="H41" s="1">
-        <f>I41*G41/$B$20</f>
+        <f>K41*G41/$B$20</f>
         <v>1258.9121706180499</v>
       </c>
       <c r="I41" s="1">
+        <f t="shared" si="14"/>
+        <v>1258.4679531972249</v>
+      </c>
+      <c r="J41" s="1">
+        <f t="shared" si="15"/>
+        <v>1259.3563880388751</v>
+      </c>
+      <c r="K41" s="1">
         <v>141.69999999999999</v>
       </c>
-      <c r="J41" s="1">
+      <c r="L41" s="1">
         <f>H41/H42</f>
         <v>6.1891217905532488E-2</v>
       </c>
-      <c r="K41" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*$H41)/$G41*$B$20, 0)</f>
-        <v>133.9345885509004</v>
-      </c>
-      <c r="L41" s="1">
-        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($H41+1))/$G41*$B$20, 0)</f>
-        <v>149.70149822623048</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12">
+      <c r="M41" s="1">
+        <f t="shared" si="16"/>
+        <v>133.87986472565848</v>
+      </c>
+      <c r="N41" s="1">
+        <f t="shared" si="17"/>
+        <v>149.75933097441057</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
       <c r="A42" s="1" t="s">
         <v>30</v>
       </c>
@@ -2618,7 +2774,7 @@
         <v>20340.723825140871</v>
       </c>
     </row>
-    <row r="43" spans="1:12">
+    <row r="43" spans="1:14">
       <c r="A43" s="1" t="s">
         <v>34</v>
       </c>
@@ -2628,10 +2784,10 @@
         <v>23898717.999999996</v>
       </c>
     </row>
-    <row r="44" spans="1:12">
+    <row r="44" spans="1:14">
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="1:12">
+    <row r="45" spans="1:14">
       <c r="F45" s="3"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Calculate starting bounds for bladder IMABC, update SLURM files to R 4.4.2
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68D08D95-55D9-6C41-8920-6AF5B6CBDEDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60E8ADEF-477D-4244-995A-BD49CF75D96B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15120" yWindow="760" windowWidth="15120" windowHeight="17760" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="37">
   <si>
     <t>target_names</t>
   </si>
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -555,7 +555,7 @@
     <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:11">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -572,19 +572,25 @@
         <v>5</v>
       </c>
       <c r="F1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="I1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:11">
       <c r="A2" s="1" t="str">
         <f t="shared" ref="A2:A25" si="0">""&amp;B2&amp;"_"&amp;E2</f>
         <v>prevalence_preclin_71</v>
@@ -604,21 +610,29 @@
       </c>
       <c r="F2" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>5.5248618784530391E-4</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>9.7534036711855159E-5</v>
+        <v>1810</v>
       </c>
       <c r="H2" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>5.5248618784530391E-4</v>
+      </c>
+      <c r="I2" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>9.7534036711855159E-5</v>
+      </c>
+      <c r="J2" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>3.1229562615372915E-3</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:11">
       <c r="A3" s="1" t="str">
         <f t="shared" si="0"/>
         <v>prevalence_preclin_80</v>
@@ -638,21 +652,29 @@
       </c>
       <c r="F3" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>1.530221882172915E-3</v>
+        <v>2</v>
       </c>
       <c r="G3" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>4.1974238437163421E-4</v>
+        <v>1307</v>
       </c>
       <c r="H3" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>1.530221882172915E-3</v>
+      </c>
+      <c r="I3" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>4.1974238437163421E-4</v>
+      </c>
+      <c r="J3" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>5.562261593248006E-3</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:11">
       <c r="A4" s="1" t="str">
         <f t="shared" si="0"/>
         <v>prevalence_preclin_90</v>
@@ -672,21 +694,29 @@
       </c>
       <c r="F4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>1.1961722488038277E-2</v>
+        <v>5</v>
       </c>
       <c r="G4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>5.1198596930172122E-3</v>
+        <v>418</v>
       </c>
       <c r="H4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>1.1961722488038277E-2</v>
+      </c>
+      <c r="I4" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>5.1198596930172122E-3</v>
+      </c>
+      <c r="J4" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>2.7692132896306509E-2</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="K4" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:11">
       <c r="A5" s="1" t="str">
         <f t="shared" ref="A5:A10" si="2">""&amp;B5&amp;"_"&amp;E5</f>
         <v>incidence_clin_2</v>
@@ -706,22 +736,30 @@
         <v>2</v>
       </c>
       <c r="F5" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A5,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>5.0435854467200008</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>10.087170893440002</v>
       </c>
       <c r="G5" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A5,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>10087170.893440001</v>
+      </c>
+      <c r="H5" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
         <v>0.1</v>
       </c>
-      <c r="H5" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A5,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>1.6241209331261943E-3</v>
-      </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.6094566130273689E-2</v>
+      </c>
+      <c r="J5" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.24526419878119815</v>
+      </c>
+      <c r="K5" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:11">
       <c r="A6" s="1" t="str">
         <f t="shared" si="2"/>
         <v>incidence_clin_7</v>
@@ -741,22 +779,30 @@
         <v>7</v>
       </c>
       <c r="F6" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A6,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>5.8673742561799997</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>11.734748512359999</v>
       </c>
       <c r="G6" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A6,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>11734748.512359999</v>
+      </c>
+      <c r="H6" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
         <v>0.1</v>
       </c>
-      <c r="H6" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A6,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0</v>
-      </c>
-      <c r="I6" s="1" t="s">
+      <c r="I6" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.6258329900368296E-2</v>
+      </c>
+      <c r="J6" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.23719286870795328</v>
+      </c>
+      <c r="K6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:11">
       <c r="A7" s="1" t="str">
         <f t="shared" si="2"/>
         <v>incidence_clin_12</v>
@@ -781,17 +827,25 @@
       </c>
       <c r="G7" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>0</v>
+        <v>12224672.231360001</v>
       </c>
       <c r="H7" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.10682882759847878</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:11">
       <c r="A8" s="1" t="str">
         <f t="shared" si="2"/>
         <v>incidence_clin_17</v>
@@ -812,21 +866,29 @@
       </c>
       <c r="F8" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>0.1</v>
+        <v>11.213875953550001</v>
       </c>
       <c r="G8" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>1.7013511956265843E-2</v>
+        <v>11213875.95355</v>
       </c>
       <c r="H8" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.1</v>
+      </c>
+      <c r="I8" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.7013511956265843E-2</v>
+      </c>
+      <c r="J8" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.23722104989583823</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:11">
       <c r="A9" s="1" t="str">
         <f t="shared" si="2"/>
         <v>incidence_clin_22</v>
@@ -847,21 +909,29 @@
       </c>
       <c r="F9" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>0.3</v>
+        <v>28.879569311969998</v>
       </c>
       <c r="G9" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>0.1597383882900868</v>
+        <v>9626523.1039899997</v>
       </c>
       <c r="H9" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.3</v>
+      </c>
+      <c r="I9" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0.1597383882900868</v>
+      </c>
+      <c r="J9" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.4874889418786299</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:11">
       <c r="A10" s="1" t="str">
         <f t="shared" si="2"/>
         <v>incidence_clin_27</v>
@@ -882,21 +952,29 @@
       </c>
       <c r="F10" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>0.5</v>
+        <v>39.624074444000001</v>
       </c>
       <c r="G10" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>0.31289158139055295</v>
+        <v>7924814.8888000008</v>
       </c>
       <c r="H10" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.5</v>
+      </c>
+      <c r="I10" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0.31289158139055295</v>
+      </c>
+      <c r="J10" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.73811868911234746</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="K10" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:11">
       <c r="A11" s="1" t="str">
         <f t="shared" ref="A11:A22" si="5">""&amp;B11&amp;"_"&amp;E11</f>
         <v>incidence_clin_32</v>
@@ -917,21 +995,29 @@
       </c>
       <c r="F11" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>1.1000000000000001</v>
+        <v>73.935344383010005</v>
       </c>
       <c r="G11" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>0.8184299276747744</v>
+        <v>6721394.9439099999</v>
       </c>
       <c r="H11" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="I11" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0.8184299276747744</v>
+      </c>
+      <c r="J11" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>1.4317978530233426</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="K11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:11">
       <c r="A12" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_37</v>
@@ -952,21 +1038,29 @@
       </c>
       <c r="F12" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>2.2000000000000002</v>
+        <v>143.68291641088004</v>
       </c>
       <c r="G12" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>1.8032433025804822</v>
+        <v>6531041.6550400006</v>
       </c>
       <c r="H12" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I12" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.8032433025804822</v>
+      </c>
+      <c r="J12" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>2.6371938700704867</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="K12" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:11">
       <c r="A13" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_42</v>
@@ -987,21 +1081,29 @@
       </c>
       <c r="F13" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>4.3</v>
+        <v>302.93943240646001</v>
       </c>
       <c r="G13" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>3.7766078728748678</v>
+        <v>7045103.0792200007</v>
       </c>
       <c r="H13" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>4.3</v>
+      </c>
+      <c r="I13" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>3.7766078728748678</v>
+      </c>
+      <c r="J13" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>4.8583883346410159</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:11">
       <c r="A14" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_47</v>
@@ -1022,21 +1124,29 @@
       </c>
       <c r="F14" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>9.5</v>
+        <v>676.82244818309994</v>
       </c>
       <c r="G14" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>8.7460518806358838</v>
+        <v>7124446.8229799997</v>
       </c>
       <c r="H14" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>9.5</v>
+      </c>
+      <c r="I14" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>8.7460518806358838</v>
+      </c>
+      <c r="J14" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>10.289748213803048</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="K14" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:11">
       <c r="A15" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_52</v>
@@ -1057,21 +1167,29 @@
       </c>
       <c r="F15" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>18.5</v>
+        <v>1207.9553240984499</v>
       </c>
       <c r="G15" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>17.419890817649691</v>
+        <v>6529488.2383699995</v>
       </c>
       <c r="H15" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>18.5</v>
+      </c>
+      <c r="I15" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>17.419890817649691</v>
+      </c>
+      <c r="J15" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>19.621383584718842</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:11">
       <c r="A16" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_57</v>
@@ -1092,21 +1210,29 @@
       </c>
       <c r="F16" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>34.299999999999997</v>
+        <v>2011.48471233549</v>
       </c>
       <c r="G16" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>32.767494120937265</v>
+        <v>5864386.9164300002</v>
       </c>
       <c r="H16" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>34.299999999999997</v>
+      </c>
+      <c r="I16" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>32.767494120937265</v>
+      </c>
+      <c r="J16" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>35.876275809580278</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="K16" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:11">
       <c r="A17" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_62</v>
@@ -1127,21 +1253,29 @@
       </c>
       <c r="F17" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>52.9</v>
+        <v>2680.3830625913301</v>
       </c>
       <c r="G17" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>50.860284058021669</v>
+        <v>5066886.6967700003</v>
       </c>
       <c r="H17" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>52.9</v>
+      </c>
+      <c r="I17" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>50.860284058021669</v>
+      </c>
+      <c r="J17" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>54.983958159669321</v>
       </c>
-      <c r="I17" s="1" t="s">
+      <c r="K17" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:11">
       <c r="A18" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_67</v>
@@ -1162,21 +1296,29 @@
       </c>
       <c r="F18" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>82.8</v>
+        <v>3404.15346684312</v>
       </c>
       <c r="G18" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>79.990143004942581</v>
+        <v>4111296.4575399999</v>
       </c>
       <c r="H18" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>82.8</v>
+      </c>
+      <c r="I18" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>79.990143004942581</v>
+      </c>
+      <c r="J18" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>85.674831914507308</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:11">
       <c r="A19" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_72</v>
@@ -1197,21 +1339,29 @@
       </c>
       <c r="F19" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>109.1</v>
+        <v>3492.4151367184104</v>
       </c>
       <c r="G19" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>105.45249909757202</v>
+        <v>3201113.7825100003</v>
       </c>
       <c r="H19" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>109.1</v>
+      </c>
+      <c r="I19" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>105.45249909757202</v>
+      </c>
+      <c r="J19" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>112.82992889659357</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="K19" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:11">
       <c r="A20" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_77</v>
@@ -1232,21 +1382,29 @@
       </c>
       <c r="F20" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>132.19999999999999</v>
+        <v>2981.061795768579</v>
       </c>
       <c r="G20" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>127.42849266253278</v>
+        <v>2254963.5368899996</v>
       </c>
       <c r="H20" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>132.19999999999999</v>
+      </c>
+      <c r="I20" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>127.42849266253278</v>
+      </c>
+      <c r="J20" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>137.07498967213519</v>
       </c>
-      <c r="I20" s="1" t="s">
+      <c r="K20" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:11">
       <c r="A21" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_82</v>
@@ -1267,21 +1425,29 @@
       </c>
       <c r="F21" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>149.30000000000001</v>
+        <v>2005.43857566867</v>
       </c>
       <c r="G21" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>142.7680888200511</v>
+        <v>1343227.4451899999</v>
       </c>
       <c r="H21" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>149.30000000000001</v>
+      </c>
+      <c r="I21" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>142.7680888200511</v>
+      </c>
+      <c r="J21" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>156.02337488989809</v>
       </c>
-      <c r="I21" s="1" t="s">
+      <c r="K21" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:11">
       <c r="A22" s="1" t="str">
         <f t="shared" si="5"/>
         <v>incidence_clin_92</v>
@@ -1301,21 +1467,29 @@
       </c>
       <c r="F22" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>141.69999999999999</v>
+        <v>1258.9121706180499</v>
       </c>
       <c r="G22" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>133.87986472565848</v>
+        <v>888434.84165000007</v>
       </c>
       <c r="H22" s="2">
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>141.69999999999999</v>
+      </c>
+      <c r="I22" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>133.87986472565848</v>
+      </c>
+      <c r="J22" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>149.75933097441057</v>
       </c>
-      <c r="I22" s="1" t="s">
+      <c r="K22" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:11">
       <c r="A23" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_1</v>
@@ -1328,21 +1502,29 @@
       </c>
       <c r="F23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.77894736842105272</v>
+        <v>21522.9</v>
       </c>
       <c r="G23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.77401602151958493</v>
+        <v>27630.75</v>
       </c>
       <c r="H23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>0.77894736842105272</v>
+      </c>
+      <c r="I23" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>0.77401602151958493</v>
+      </c>
+      <c r="J23" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>0.78380116289475799</v>
       </c>
-      <c r="I23" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:11">
       <c r="A24" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_2</v>
@@ -1355,21 +1537,29 @@
       </c>
       <c r="F24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>0.18947368421052632</v>
+        <v>5235.3</v>
       </c>
       <c r="G24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>0.18489624853500833</v>
+        <v>27630.75</v>
       </c>
       <c r="H24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>0.18947368421052632</v>
+      </c>
+      <c r="I24" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>0.18489624853500833</v>
+      </c>
+      <c r="J24" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>0.19413745183393108</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="K24" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:11">
       <c r="A25" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_3</v>
@@ -1382,17 +1572,25 @@
       </c>
       <c r="F25" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>3.1578947368421054E-2</v>
+        <v>872.55</v>
       </c>
       <c r="G25" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>2.9581205871892616E-2</v>
+        <v>27630.75</v>
       </c>
       <c r="H25" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>3.1578947368421054E-2</v>
+      </c>
+      <c r="I25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>2.9581205871892616E-2</v>
+      </c>
+      <c r="J25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>3.3706918413456612E-2</v>
       </c>
-      <c r="I25" s="1" t="s">
+      <c r="K25" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1853,7 +2051,7 @@
         <v>10087170.893440001</v>
       </c>
       <c r="H24" s="1">
-        <f>K24*G24/$B$20</f>
+        <f t="shared" ref="H24:H41" si="14">K24*G24/$B$20</f>
         <v>10.087170893440002</v>
       </c>
       <c r="I24" s="1">
@@ -1907,26 +2105,26 @@
         <v>11734748.512359999</v>
       </c>
       <c r="H25" s="1">
-        <f>K25*G25/$B$20</f>
+        <f t="shared" si="14"/>
         <v>11.734748512359999</v>
       </c>
       <c r="I25" s="1">
-        <f t="shared" ref="I25:I42" si="14">MAX(0, K25-0.05)*G25/$B$20</f>
+        <f t="shared" ref="I25:I41" si="15">MAX(0, K25-0.05)*G25/$B$20</f>
         <v>5.8673742561799997</v>
       </c>
       <c r="J25" s="1">
-        <f t="shared" ref="J25:J41" si="15">(K25+0.05)*G25/$B$20</f>
+        <f t="shared" ref="J25:J41" si="16">(K25+0.05)*G25/$B$20</f>
         <v>17.602122768539999</v>
       </c>
       <c r="K25" s="1">
         <v>0.1</v>
       </c>
       <c r="M25" s="1">
-        <f t="shared" ref="M25:M41" si="16">IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*I25)/$G25*$B$20, 0)</f>
+        <f t="shared" ref="M25:M41" si="17">IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*I25)/$G25*$B$20, 0)</f>
         <v>1.6258329900368296E-2</v>
       </c>
       <c r="N25" s="1">
-        <f t="shared" ref="N25:N41" si="17">IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($J25+1))/$G25*$B$20, 0)</f>
+        <f t="shared" ref="N25:N41" si="18">IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($J25+1))/$G25*$B$20, 0)</f>
         <v>0.23719286870795328</v>
       </c>
     </row>
@@ -1942,7 +2140,7 @@
         <v>10</v>
       </c>
       <c r="D26" s="1">
-        <f t="shared" ref="D26:D40" si="18">C27</f>
+        <f t="shared" ref="D26:D40" si="19">C27</f>
         <v>15</v>
       </c>
       <c r="E26" s="1">
@@ -1957,26 +2155,26 @@
         <v>12224672.231360001</v>
       </c>
       <c r="H26" s="1">
-        <f>K26*G26/$B$20</f>
-        <v>0</v>
-      </c>
-      <c r="I26" s="1">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
+      <c r="I26" s="1">
+        <f t="shared" si="15"/>
+        <v>0</v>
+      </c>
       <c r="J26" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>6.1123361156800007</v>
       </c>
       <c r="K26" s="1">
         <v>0</v>
       </c>
       <c r="M26" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="N26" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0.10682882759847878</v>
       </c>
     </row>
@@ -1992,7 +2190,7 @@
         <v>15</v>
       </c>
       <c r="D27" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>20</v>
       </c>
       <c r="E27" s="1">
@@ -2007,26 +2205,26 @@
         <v>11213875.95355</v>
       </c>
       <c r="H27" s="1">
-        <f>K27*G27/$B$20</f>
+        <f t="shared" si="14"/>
         <v>11.213875953550001</v>
       </c>
       <c r="I27" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>5.6069379767750007</v>
       </c>
       <c r="J27" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>16.820813930325002</v>
       </c>
       <c r="K27" s="1">
         <v>0.1</v>
       </c>
       <c r="M27" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1.7013511956265843E-2</v>
       </c>
       <c r="N27" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0.23722104989583823</v>
       </c>
     </row>
@@ -2042,7 +2240,7 @@
         <v>20</v>
       </c>
       <c r="D28" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>25</v>
       </c>
       <c r="E28" s="1">
@@ -2057,15 +2255,15 @@
         <v>9626523.1039899997</v>
       </c>
       <c r="H28" s="1">
-        <f>K28*G28/$B$20</f>
+        <f t="shared" si="14"/>
         <v>28.879569311969998</v>
       </c>
       <c r="I28" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>24.066307759975</v>
       </c>
       <c r="J28" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>33.692830863964993</v>
       </c>
       <c r="K28" s="1">
@@ -2076,11 +2274,11 @@
         <v>7.0026509067945388E-3</v>
       </c>
       <c r="M28" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.1597383882900868</v>
       </c>
       <c r="N28" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0.4874889418786299</v>
       </c>
     </row>
@@ -2096,7 +2294,7 @@
         <v>25</v>
       </c>
       <c r="D29" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>30</v>
       </c>
       <c r="E29" s="1">
@@ -2111,26 +2309,26 @@
         <v>7924814.8888000008</v>
       </c>
       <c r="H29" s="1">
-        <f>K29*G29/$B$20</f>
+        <f t="shared" si="14"/>
         <v>39.624074444000001</v>
       </c>
       <c r="I29" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>35.661666999600001</v>
       </c>
       <c r="J29" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>43.586481888400009</v>
       </c>
       <c r="K29" s="1">
         <v>0.5</v>
       </c>
       <c r="M29" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.31289158139055295</v>
       </c>
       <c r="N29" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>0.73811868911234746</v>
       </c>
     </row>
@@ -2146,7 +2344,7 @@
         <v>30</v>
       </c>
       <c r="D30" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>35</v>
       </c>
       <c r="E30" s="1">
@@ -2161,26 +2359,26 @@
         <v>6721394.9439099999</v>
       </c>
       <c r="H30" s="1">
-        <f>K30*G30/$B$20</f>
+        <f t="shared" si="14"/>
         <v>73.935344383010005</v>
       </c>
       <c r="I30" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>70.574646911054998</v>
       </c>
       <c r="J30" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>77.296041854965011</v>
       </c>
       <c r="K30" s="1">
         <v>1.1000000000000001</v>
       </c>
       <c r="M30" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.8184299276747744</v>
       </c>
       <c r="N30" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>1.4317978530233426</v>
       </c>
     </row>
@@ -2196,7 +2394,7 @@
         <v>35</v>
       </c>
       <c r="D31" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>40</v>
       </c>
       <c r="E31" s="1">
@@ -2211,15 +2409,15 @@
         <v>6531041.6550400006</v>
       </c>
       <c r="H31" s="1">
-        <f>K31*G31/$B$20</f>
+        <f t="shared" si="14"/>
         <v>143.68291641088004</v>
       </c>
       <c r="I31" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>140.41739558336002</v>
       </c>
       <c r="J31" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>146.94843723840003</v>
       </c>
       <c r="K31" s="1">
@@ -2230,11 +2428,11 @@
         <v>2.1957052888418878E-2</v>
       </c>
       <c r="M31" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>1.8032433025804822</v>
       </c>
       <c r="N31" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>2.6371938700704867</v>
       </c>
     </row>
@@ -2250,7 +2448,7 @@
         <v>40</v>
       </c>
       <c r="D32" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>45</v>
       </c>
       <c r="E32" s="1">
@@ -2265,26 +2463,26 @@
         <v>7045103.0792200007</v>
       </c>
       <c r="H32" s="1">
-        <f>K32*G32/$B$20</f>
+        <f t="shared" si="14"/>
         <v>302.93943240646001</v>
       </c>
       <c r="I32" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>299.41688086685002</v>
       </c>
       <c r="J32" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>306.46198394607001</v>
       </c>
       <c r="K32" s="1">
         <v>4.3</v>
       </c>
       <c r="M32" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>3.7766078728748678</v>
       </c>
       <c r="N32" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>4.8583883346410159</v>
       </c>
     </row>
@@ -2300,7 +2498,7 @@
         <v>45</v>
       </c>
       <c r="D33" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>50</v>
       </c>
       <c r="E33" s="1">
@@ -2315,15 +2513,15 @@
         <v>7124446.8229799997</v>
       </c>
       <c r="H33" s="1">
-        <f>K33*G33/$B$20</f>
+        <f t="shared" si="14"/>
         <v>676.82244818309994</v>
       </c>
       <c r="I33" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>673.26022477160996</v>
       </c>
       <c r="J33" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>680.38467159458992</v>
       </c>
       <c r="K33" s="1">
@@ -2334,11 +2532,11 @@
         <v>9.2660309853476744E-2</v>
       </c>
       <c r="M33" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>8.7460518806358838</v>
       </c>
       <c r="N33" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>10.289748213803048</v>
       </c>
     </row>
@@ -2354,7 +2552,7 @@
         <v>50</v>
       </c>
       <c r="D34" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>55</v>
       </c>
       <c r="E34" s="1">
@@ -2369,26 +2567,26 @@
         <v>6529488.2383699995</v>
       </c>
       <c r="H34" s="1">
-        <f>K34*G34/$B$20</f>
+        <f t="shared" si="14"/>
         <v>1207.9553240984499</v>
       </c>
       <c r="I34" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1204.6905799792648</v>
       </c>
       <c r="J34" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1211.2200682176351</v>
       </c>
       <c r="K34" s="1">
         <v>18.5</v>
       </c>
       <c r="M34" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>17.419890817649691</v>
       </c>
       <c r="N34" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>19.621383584718842</v>
       </c>
     </row>
@@ -2404,7 +2602,7 @@
         <v>55</v>
       </c>
       <c r="D35" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>60</v>
       </c>
       <c r="E35" s="1">
@@ -2419,15 +2617,15 @@
         <v>5864386.9164300002</v>
       </c>
       <c r="H35" s="1">
-        <f>K35*G35/$B$20</f>
+        <f t="shared" si="14"/>
         <v>2011.48471233549</v>
       </c>
       <c r="I35" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2008.5525188772749</v>
       </c>
       <c r="J35" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2014.4169057937047</v>
       </c>
       <c r="K35" s="1">
@@ -2438,11 +2636,11 @@
         <v>0.23066375686826504</v>
       </c>
       <c r="M35" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>32.767494120937265</v>
       </c>
       <c r="N35" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>35.876275809580278</v>
       </c>
     </row>
@@ -2458,7 +2656,7 @@
         <v>60</v>
       </c>
       <c r="D36" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>65</v>
       </c>
       <c r="E36" s="1">
@@ -2473,26 +2671,26 @@
         <v>5066886.6967700003</v>
       </c>
       <c r="H36" s="1">
-        <f>K36*G36/$B$20</f>
+        <f t="shared" si="14"/>
         <v>2680.3830625913301</v>
       </c>
       <c r="I36" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2677.8496192429452</v>
       </c>
       <c r="J36" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2682.9165059397151</v>
       </c>
       <c r="K36" s="1">
         <v>52.9</v>
       </c>
       <c r="M36" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>50.860284058021669</v>
       </c>
       <c r="N36" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>54.983958159669321</v>
       </c>
     </row>
@@ -2508,7 +2706,7 @@
         <v>65</v>
       </c>
       <c r="D37" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>70</v>
       </c>
       <c r="E37" s="1">
@@ -2523,15 +2721,15 @@
         <v>4111296.4575399999</v>
       </c>
       <c r="H37" s="1">
-        <f>K37*G37/$B$20</f>
+        <f t="shared" si="14"/>
         <v>3404.15346684312</v>
       </c>
       <c r="I37" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3402.0978186143498</v>
       </c>
       <c r="J37" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>3406.2091150718898</v>
       </c>
       <c r="K37" s="1">
@@ -2542,11 +2740,11 @@
         <v>0.33905227084581235</v>
       </c>
       <c r="M37" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>79.990143004942581</v>
       </c>
       <c r="N37" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>85.674831914507308</v>
       </c>
     </row>
@@ -2562,7 +2760,7 @@
         <v>70</v>
       </c>
       <c r="D38" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>75</v>
       </c>
       <c r="E38" s="1">
@@ -2577,26 +2775,26 @@
         <v>3201113.7825100003</v>
       </c>
       <c r="H38" s="1">
-        <f>K38*G38/$B$20</f>
+        <f t="shared" si="14"/>
         <v>3492.4151367184104</v>
       </c>
       <c r="I38" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3490.8145798271553</v>
       </c>
       <c r="J38" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>3494.015693609665</v>
       </c>
       <c r="K38" s="1">
         <v>109.1</v>
       </c>
       <c r="M38" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>105.45249909757202</v>
       </c>
       <c r="N38" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>112.82992889659357</v>
       </c>
     </row>
@@ -2612,7 +2810,7 @@
         <v>75</v>
       </c>
       <c r="D39" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>80</v>
       </c>
       <c r="E39" s="1">
@@ -2627,15 +2825,15 @@
         <v>2254963.5368899996</v>
       </c>
       <c r="H39" s="1">
-        <f>K39*G39/$B$20</f>
+        <f t="shared" si="14"/>
         <v>2981.061795768579</v>
       </c>
       <c r="I39" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2979.9343140001338</v>
       </c>
       <c r="J39" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2982.1892775370247</v>
       </c>
       <c r="K39" s="1">
@@ -2646,11 +2844,11 @@
         <v>0.24514861979857369</v>
       </c>
       <c r="M39" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>127.42849266253278</v>
       </c>
       <c r="N39" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>137.07498967213519</v>
       </c>
     </row>
@@ -2666,7 +2864,7 @@
         <v>80</v>
       </c>
       <c r="D40" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>85</v>
       </c>
       <c r="E40" s="1">
@@ -2681,26 +2879,26 @@
         <v>1343227.4451899999</v>
       </c>
       <c r="H40" s="1">
-        <f>K40*G40/$B$20</f>
+        <f t="shared" si="14"/>
         <v>2005.43857566867</v>
       </c>
       <c r="I40" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2004.7669619460751</v>
       </c>
       <c r="J40" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2006.1101893912653</v>
       </c>
       <c r="K40" s="1">
         <v>149.30000000000001</v>
       </c>
       <c r="M40" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>142.7680888200511</v>
       </c>
       <c r="N40" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>156.02337488989809</v>
       </c>
     </row>
@@ -2730,15 +2928,15 @@
         <v>888434.84165000007</v>
       </c>
       <c r="H41" s="1">
-        <f>K41*G41/$B$20</f>
+        <f t="shared" si="14"/>
         <v>1258.9121706180499</v>
       </c>
       <c r="I41" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1258.4679531972249</v>
       </c>
       <c r="J41" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1259.3563880388751</v>
       </c>
       <c r="K41" s="1">
@@ -2749,11 +2947,11 @@
         <v>6.1891217905532488E-2</v>
       </c>
       <c r="M41" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>133.87986472565848</v>
       </c>
       <c r="N41" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>149.75933097441057</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert priors, change IMABC number of cores
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B3BFD7F-F004-8045-857B-507258A20D5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AED7BB-E58C-4F48-8EC2-4DFA1A178ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="37">
   <si>
     <t>target_names</t>
   </si>
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -592,7 +592,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1" t="str">
-        <f t="shared" ref="A2:A16" si="0">""&amp;B2&amp;"_"&amp;E2</f>
+        <f t="shared" ref="A2:A25" si="0">""&amp;B2&amp;"_"&amp;E2</f>
         <v>prevalence_preclin_71</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -605,7 +605,7 @@
         <v>76</v>
       </c>
       <c r="E2" s="1">
-        <f t="shared" ref="E2:E13" si="1">FLOOR(AVERAGE(C2,D2), 1)</f>
+        <f t="shared" ref="E2:E22" si="1">FLOOR(AVERAGE(C2,D2), 1)</f>
         <v>71</v>
       </c>
       <c r="F2" s="2">
@@ -718,42 +718,42 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="1" t="str">
-        <f t="shared" ref="A5:A13" si="2">""&amp;B5&amp;"_"&amp;E5</f>
-        <v>incidence_clin_47</v>
+        <f t="shared" ref="A5:A10" si="2">""&amp;B5&amp;"_"&amp;E5</f>
+        <v>incidence_clin_2</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="1">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="D5" s="1">
-        <f t="shared" ref="D5:D12" si="3">C6</f>
-        <v>50</v>
+        <f t="shared" ref="D5" si="3">C6</f>
+        <v>5</v>
       </c>
       <c r="E5" s="1">
         <f t="shared" si="1"/>
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="F5" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A5,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>676.82244818309994</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>10.087170893440002</v>
       </c>
       <c r="G5" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A5,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>7124446.8229799997</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>10087170.893440001</v>
       </c>
       <c r="H5" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A5,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>9.5</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.1</v>
       </c>
       <c r="I5" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A5,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>8.7460518806358838</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.6094566130273689E-2</v>
       </c>
       <c r="J5" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A5,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>10.289748213803048</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.24526419878119815</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>21</v>
@@ -762,41 +762,41 @@
     <row r="6" spans="1:11">
       <c r="A6" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>incidence_clin_52</v>
+        <v>incidence_clin_7</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="1">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="D6" s="1">
-        <f t="shared" si="3"/>
-        <v>55</v>
+        <f>C7</f>
+        <v>10</v>
       </c>
       <c r="E6" s="1">
         <f t="shared" si="1"/>
-        <v>52</v>
+        <v>7</v>
       </c>
       <c r="F6" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A6,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>1207.9553240984499</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>11.734748512359999</v>
       </c>
       <c r="G6" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A6,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>6529488.2383699995</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>11734748.512359999</v>
       </c>
       <c r="H6" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A6,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>18.5</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.1</v>
       </c>
       <c r="I6" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A6,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>17.419890817649691</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.6258329900368296E-2</v>
       </c>
       <c r="J6" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A6,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>19.621383584718842</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.23719286870795328</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>21</v>
@@ -805,41 +805,41 @@
     <row r="7" spans="1:11">
       <c r="A7" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>incidence_clin_57</v>
+        <v>incidence_clin_12</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="1">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1">
-        <f t="shared" si="3"/>
-        <v>60</v>
+        <f t="shared" ref="D7:D21" si="4">C8</f>
+        <v>15</v>
       </c>
       <c r="E7" s="1">
         <f t="shared" si="1"/>
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="F7" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A7,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>2011.48471233549</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>0</v>
       </c>
       <c r="G7" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A7,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>5864386.9164300002</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>12224672.231360001</v>
       </c>
       <c r="H7" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A7,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>34.299999999999997</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0</v>
       </c>
       <c r="I7" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A7,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>32.767494120937265</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0</v>
       </c>
       <c r="J7" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A7,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>35.876275809580278</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.10682882759847878</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>21</v>
@@ -848,41 +848,41 @@
     <row r="8" spans="1:11">
       <c r="A8" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>incidence_clin_62</v>
+        <v>incidence_clin_17</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="1">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="D8" s="1">
-        <f t="shared" si="3"/>
-        <v>65</v>
+        <f t="shared" si="4"/>
+        <v>20</v>
       </c>
       <c r="E8" s="1">
         <f t="shared" si="1"/>
-        <v>62</v>
+        <v>17</v>
       </c>
       <c r="F8" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A8,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>2680.3830625913301</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>11.213875953550001</v>
       </c>
       <c r="G8" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A8,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>5066886.6967700003</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>11213875.95355</v>
       </c>
       <c r="H8" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A8,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>52.9</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.1</v>
       </c>
       <c r="I8" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A8,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>50.860284058021669</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.7013511956265843E-2</v>
       </c>
       <c r="J8" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A8,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>54.983958159669321</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.23722104989583823</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>21</v>
@@ -891,41 +891,41 @@
     <row r="9" spans="1:11">
       <c r="A9" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>incidence_clin_67</v>
+        <v>incidence_clin_22</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="1">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="D9" s="1">
-        <f t="shared" si="3"/>
-        <v>70</v>
+        <f t="shared" si="4"/>
+        <v>25</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="1"/>
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="F9" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A9,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>3404.15346684312</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>28.879569311969998</v>
       </c>
       <c r="G9" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A9,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>4111296.4575399999</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>9626523.1039899997</v>
       </c>
       <c r="H9" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A9,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>82.8</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.3</v>
       </c>
       <c r="I9" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A9,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>79.990143004942581</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0.1597383882900868</v>
       </c>
       <c r="J9" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A9,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>85.674831914507308</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.4874889418786299</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>21</v>
@@ -934,41 +934,41 @@
     <row r="10" spans="1:11">
       <c r="A10" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>incidence_clin_72</v>
+        <v>incidence_clin_27</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="1">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="D10" s="1">
-        <f t="shared" si="3"/>
-        <v>75</v>
+        <f t="shared" si="4"/>
+        <v>30</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" si="1"/>
-        <v>72</v>
+        <v>27</v>
       </c>
       <c r="F10" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A10,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>3492.4151367184104</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>39.624074444000001</v>
       </c>
       <c r="G10" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A10,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>3201113.7825100003</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>7924814.8888000008</v>
       </c>
       <c r="H10" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A10,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>109.1</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>0.5</v>
       </c>
       <c r="I10" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A10,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>105.45249909757202</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0.31289158139055295</v>
       </c>
       <c r="J10" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A10,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>112.82992889659357</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>0.73811868911234746</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>21</v>
@@ -976,42 +976,42 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>incidence_clin_77</v>
+        <f t="shared" ref="A11:A22" si="5">""&amp;B11&amp;"_"&amp;E11</f>
+        <v>incidence_clin_32</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="1">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D11" s="1">
-        <f t="shared" si="3"/>
-        <v>80</v>
+        <f t="shared" si="4"/>
+        <v>35</v>
       </c>
       <c r="E11" s="1">
         <f t="shared" si="1"/>
-        <v>77</v>
+        <v>32</v>
       </c>
       <c r="F11" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A11,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>2981.061795768579</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>73.935344383010005</v>
       </c>
       <c r="G11" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A11,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>2254963.5368899996</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>6721394.9439099999</v>
       </c>
       <c r="H11" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A11,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>132.19999999999999</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I11" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A11,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>127.42849266253278</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>0.8184299276747744</v>
       </c>
       <c r="J11" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A11,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>137.07498967213519</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>1.4317978530233426</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>21</v>
@@ -1019,42 +1019,42 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>incidence_clin_82</v>
+        <f t="shared" si="5"/>
+        <v>incidence_clin_37</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="1">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="D12" s="1">
-        <f t="shared" si="3"/>
-        <v>85</v>
+        <f t="shared" si="4"/>
+        <v>40</v>
       </c>
       <c r="E12" s="1">
         <f t="shared" si="1"/>
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="F12" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A12,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>2005.43857566867</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>143.68291641088004</v>
       </c>
       <c r="G12" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A12,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>1343227.4451899999</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>6531041.6550400006</v>
       </c>
       <c r="H12" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A12,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>149.30000000000001</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>2.2000000000000002</v>
       </c>
       <c r="I12" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A12,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>142.7680888200511</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>1.8032433025804822</v>
       </c>
       <c r="J12" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A12,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>156.02337488989809</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>2.6371938700704867</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>21</v>
@@ -1062,41 +1062,42 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>incidence_clin_92</v>
+        <f t="shared" si="5"/>
+        <v>incidence_clin_42</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="1">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="D13" s="1">
-        <v>100</v>
+        <f t="shared" si="4"/>
+        <v>45</v>
       </c>
       <c r="E13" s="1">
         <f t="shared" si="1"/>
-        <v>92</v>
+        <v>42</v>
       </c>
       <c r="F13" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A13,bounds!$A$23:$A$32,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>1258.9121706180499</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>302.93943240646001</v>
       </c>
       <c r="G13" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A13,bounds!$A$23:$A$32,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>888434.84165000007</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>7045103.0792200007</v>
       </c>
       <c r="H13" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A13,bounds!$A$23:$A$32,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>141.69999999999999</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>4.3</v>
       </c>
       <c r="I13" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A13,bounds!$A$23:$A$32,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>133.87986472565848</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>3.7766078728748678</v>
       </c>
       <c r="J13" s="2">
-        <f>INDEX(bounds!$23:$32,MATCH(targets!$A13,bounds!$A$23:$A$32,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>149.75933097441057</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>4.8583883346410159</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>21</v>
@@ -1104,106 +1105,492 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_47</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="1">
+        <v>45</v>
+      </c>
+      <c r="D14" s="1">
+        <f t="shared" si="4"/>
+        <v>50</v>
+      </c>
+      <c r="E14" s="1">
+        <f t="shared" si="1"/>
+        <v>47</v>
+      </c>
+      <c r="F14" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>676.82244818309994</v>
+      </c>
+      <c r="G14" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>7124446.8229799997</v>
+      </c>
+      <c r="H14" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>9.5</v>
+      </c>
+      <c r="I14" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>8.7460518806358838</v>
+      </c>
+      <c r="J14" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>10.289748213803048</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_52</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="1">
+        <v>50</v>
+      </c>
+      <c r="D15" s="1">
+        <f t="shared" si="4"/>
+        <v>55</v>
+      </c>
+      <c r="E15" s="1">
+        <f t="shared" si="1"/>
+        <v>52</v>
+      </c>
+      <c r="F15" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>1207.9553240984499</v>
+      </c>
+      <c r="G15" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>6529488.2383699995</v>
+      </c>
+      <c r="H15" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>18.5</v>
+      </c>
+      <c r="I15" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>17.419890817649691</v>
+      </c>
+      <c r="J15" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>19.621383584718842</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_57</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="1">
+        <v>55</v>
+      </c>
+      <c r="D16" s="1">
+        <f t="shared" si="4"/>
+        <v>60</v>
+      </c>
+      <c r="E16" s="1">
+        <f t="shared" si="1"/>
+        <v>57</v>
+      </c>
+      <c r="F16" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>2011.48471233549</v>
+      </c>
+      <c r="G16" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>5864386.9164300002</v>
+      </c>
+      <c r="H16" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>34.299999999999997</v>
+      </c>
+      <c r="I16" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>32.767494120937265</v>
+      </c>
+      <c r="J16" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>35.876275809580278</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11">
+      <c r="A17" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_62</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="1">
+        <v>60</v>
+      </c>
+      <c r="D17" s="1">
+        <f t="shared" si="4"/>
+        <v>65</v>
+      </c>
+      <c r="E17" s="1">
+        <f t="shared" si="1"/>
+        <v>62</v>
+      </c>
+      <c r="F17" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>2680.3830625913301</v>
+      </c>
+      <c r="G17" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>5066886.6967700003</v>
+      </c>
+      <c r="H17" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>52.9</v>
+      </c>
+      <c r="I17" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>50.860284058021669</v>
+      </c>
+      <c r="J17" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>54.983958159669321</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11">
+      <c r="A18" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_67</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="1">
+        <v>65</v>
+      </c>
+      <c r="D18" s="1">
+        <f t="shared" si="4"/>
+        <v>70</v>
+      </c>
+      <c r="E18" s="1">
+        <f t="shared" si="1"/>
+        <v>67</v>
+      </c>
+      <c r="F18" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>3404.15346684312</v>
+      </c>
+      <c r="G18" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>4111296.4575399999</v>
+      </c>
+      <c r="H18" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>82.8</v>
+      </c>
+      <c r="I18" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>79.990143004942581</v>
+      </c>
+      <c r="J18" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>85.674831914507308</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11">
+      <c r="A19" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_72</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C19" s="1">
+        <v>70</v>
+      </c>
+      <c r="D19" s="1">
+        <f t="shared" si="4"/>
+        <v>75</v>
+      </c>
+      <c r="E19" s="1">
+        <f t="shared" si="1"/>
+        <v>72</v>
+      </c>
+      <c r="F19" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>3492.4151367184104</v>
+      </c>
+      <c r="G19" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>3201113.7825100003</v>
+      </c>
+      <c r="H19" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>109.1</v>
+      </c>
+      <c r="I19" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>105.45249909757202</v>
+      </c>
+      <c r="J19" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>112.82992889659357</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11">
+      <c r="A20" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_77</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C20" s="1">
+        <v>75</v>
+      </c>
+      <c r="D20" s="1">
+        <f t="shared" si="4"/>
+        <v>80</v>
+      </c>
+      <c r="E20" s="1">
+        <f t="shared" si="1"/>
+        <v>77</v>
+      </c>
+      <c r="F20" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>2981.061795768579</v>
+      </c>
+      <c r="G20" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>2254963.5368899996</v>
+      </c>
+      <c r="H20" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>132.19999999999999</v>
+      </c>
+      <c r="I20" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>127.42849266253278</v>
+      </c>
+      <c r="J20" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>137.07498967213519</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11">
+      <c r="A21" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_82</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="1">
+        <v>80</v>
+      </c>
+      <c r="D21" s="1">
+        <f t="shared" si="4"/>
+        <v>85</v>
+      </c>
+      <c r="E21" s="1">
+        <f t="shared" si="1"/>
+        <v>82</v>
+      </c>
+      <c r="F21" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>2005.43857566867</v>
+      </c>
+      <c r="G21" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>1343227.4451899999</v>
+      </c>
+      <c r="H21" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>149.30000000000001</v>
+      </c>
+      <c r="I21" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>142.7680888200511</v>
+      </c>
+      <c r="J21" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>156.02337488989809</v>
+      </c>
+      <c r="K21" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11">
+      <c r="A22" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v>incidence_clin_92</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C22" s="1">
+        <v>85</v>
+      </c>
+      <c r="D22" s="1">
+        <v>100</v>
+      </c>
+      <c r="E22" s="1">
+        <f t="shared" si="1"/>
+        <v>92</v>
+      </c>
+      <c r="F22" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>1258.9121706180499</v>
+      </c>
+      <c r="G22" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>888434.84165000007</v>
+      </c>
+      <c r="H22" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>141.69999999999999</v>
+      </c>
+      <c r="I22" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>133.87986472565848</v>
+      </c>
+      <c r="J22" s="2">
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>149.75933097441057</v>
+      </c>
+      <c r="K22" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11">
+      <c r="A23" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_1</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E23" s="1">
         <v>1</v>
       </c>
-      <c r="F14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+      <c r="F23" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
         <v>21522.9</v>
       </c>
-      <c r="G14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+      <c r="G23" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
         <v>27630.75</v>
       </c>
-      <c r="H14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+      <c r="H23" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
         <v>0.77894736842105272</v>
       </c>
-      <c r="I14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+      <c r="I23" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
         <v>0.77401602151958493</v>
       </c>
-      <c r="J14" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A14,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
+      <c r="J23" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>0.78380116289475799</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="K23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="1" t="str">
+    <row r="24" spans="1:11">
+      <c r="A24" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_2</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B24" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E24" s="1">
         <v>2</v>
       </c>
-      <c r="F15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+      <c r="F24" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
         <v>5235.3</v>
       </c>
-      <c r="G15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+      <c r="G24" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
         <v>27630.75</v>
       </c>
-      <c r="H15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+      <c r="H24" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
         <v>0.18947368421052632</v>
       </c>
-      <c r="I15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+      <c r="I24" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
         <v>0.18489624853500833</v>
       </c>
-      <c r="J15" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A15,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
+      <c r="J24" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>0.19413745183393108</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="K24" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16" s="1" t="str">
+    <row r="25" spans="1:11">
+      <c r="A25" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_3</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B25" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E25" s="1">
         <v>3</v>
       </c>
-      <c r="F16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+      <c r="F25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
         <v>872.55</v>
       </c>
-      <c r="G16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+      <c r="G25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
         <v>27630.75</v>
       </c>
-      <c r="H16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+      <c r="H25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
         <v>3.1578947368421054E-2</v>
       </c>
-      <c r="I16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+      <c r="I25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
         <v>2.9581205871892616E-2</v>
       </c>
-      <c r="J16" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A16,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
+      <c r="J25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>3.3706918413456612E-2</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="K25" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1215,7 +1602,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79E831A2-898F-7F45-AC2C-D0D6D35A5E8A}">
-  <dimension ref="A1:X36"/>
+  <dimension ref="A1:X45"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="21.33203125" style="1" customWidth="1"/>
@@ -1640,505 +2027,966 @@
     </row>
     <row r="24" spans="1:24">
       <c r="A24" s="1" t="str">
-        <f t="shared" ref="A24:A32" si="11">B24&amp;"_"&amp;E24</f>
-        <v>incidence_clin_47</v>
+        <f t="shared" ref="A24:A41" si="11">B24&amp;"_"&amp;E24</f>
+        <v>incidence_clin_2</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C24" s="1">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="D24" s="1">
-        <f t="shared" ref="D24:D31" si="12">C25</f>
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="E24" s="1">
-        <f t="shared" ref="E24:E32" si="13">FLOOR(AVERAGE(C24,D24), 1)</f>
-        <v>47</v>
+        <f t="shared" ref="E24:E41" si="12">FLOOR(AVERAGE(C24,D24), 1)</f>
+        <v>2</v>
       </c>
       <c r="F24" s="1">
-        <v>59622</v>
+        <v>84416</v>
       </c>
       <c r="G24" s="1">
-        <f t="shared" ref="G24:G32" si="14">F24/$B$16*$B$17*($B$19-$B$18+1)</f>
-        <v>7124446.8229799997</v>
+        <f t="shared" ref="G24:G41" si="13">F24/$B$16*$B$17*($B$19-$B$18+1)</f>
+        <v>10087170.893440001</v>
       </c>
       <c r="H24" s="1">
-        <f t="shared" ref="H24:H32" si="15">K24*G24/$B$20</f>
-        <v>676.82244818309994</v>
+        <f t="shared" ref="H24:H41" si="14">K24*G24/$B$20</f>
+        <v>10.087170893440002</v>
       </c>
       <c r="I24" s="1">
-        <f t="shared" ref="I24:I32" si="16">MAX(0, K24-0.05)*G24/$B$20</f>
-        <v>673.26022477160996</v>
+        <f>MAX(0, K24-0.05)*G24/$B$20</f>
+        <v>5.0435854467200008</v>
       </c>
       <c r="J24" s="1">
-        <f t="shared" ref="J24:J32" si="17">(K24+0.05)*G24/$B$20</f>
-        <v>680.38467159458992</v>
+        <f>(K24+0.05)*G24/$B$20</f>
+        <v>15.130756340160005</v>
       </c>
       <c r="K24" s="1">
-        <v>9.5</v>
+        <v>0.1</v>
       </c>
       <c r="L24" s="1">
-        <f>SUM(H24:H25)/$H$33</f>
-        <v>9.5583622614415803E-2</v>
+        <f>SUM(H24:H27)/H42</f>
+        <v>1.6241209331261943E-3</v>
       </c>
       <c r="M24" s="1">
-        <f t="shared" ref="M24:M32" si="18">IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*I24)/$G24*$B$20, 0)</f>
-        <v>8.7460518806358838</v>
+        <f>IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*I24)/$G24*$B$20, 0)</f>
+        <v>1.6094566130273689E-2</v>
       </c>
       <c r="N24" s="1">
-        <f t="shared" ref="N24:N32" si="19">IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($J24+1))/$G24*$B$20, 0)</f>
-        <v>10.289748213803048</v>
+        <f>IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($J24+1))/$G24*$B$20, 0)</f>
+        <v>0.24526419878119815</v>
       </c>
     </row>
     <row r="25" spans="1:24">
       <c r="A25" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>incidence_clin_52</v>
+        <v>incidence_clin_7</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C25" s="1">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="D25" s="1">
+        <f>C26</f>
+        <v>10</v>
+      </c>
+      <c r="E25" s="1">
         <f t="shared" si="12"/>
-        <v>55</v>
-      </c>
-      <c r="E25" s="1">
+        <v>7</v>
+      </c>
+      <c r="F25" s="1">
+        <v>98204</v>
+      </c>
+      <c r="G25" s="1">
         <f t="shared" si="13"/>
-        <v>52</v>
-      </c>
-      <c r="F25" s="1">
-        <v>54643</v>
-      </c>
-      <c r="G25" s="1">
+        <v>11734748.512359999</v>
+      </c>
+      <c r="H25" s="1">
         <f t="shared" si="14"/>
-        <v>6529488.2383699995</v>
-      </c>
-      <c r="H25" s="1">
-        <f t="shared" si="15"/>
-        <v>1207.9553240984499</v>
+        <v>11.734748512359999</v>
       </c>
       <c r="I25" s="1">
-        <f t="shared" si="16"/>
-        <v>1204.6905799792648</v>
+        <f t="shared" ref="I25:I41" si="15">MAX(0, K25-0.05)*G25/$B$20</f>
+        <v>5.8673742561799997</v>
       </c>
       <c r="J25" s="1">
-        <f t="shared" si="17"/>
-        <v>1211.2200682176351</v>
+        <f t="shared" ref="J25:J41" si="16">(K25+0.05)*G25/$B$20</f>
+        <v>17.602122768539999</v>
       </c>
       <c r="K25" s="1">
-        <v>18.5</v>
+        <v>0.1</v>
       </c>
       <c r="M25" s="1">
-        <f t="shared" si="18"/>
-        <v>17.419890817649691</v>
+        <f t="shared" ref="M25:M41" si="17">IFERROR(0.5*_xlfn.CHISQ.INV($B$3/2,2*I25)/$G25*$B$20, 0)</f>
+        <v>1.6258329900368296E-2</v>
       </c>
       <c r="N25" s="1">
-        <f t="shared" si="19"/>
-        <v>19.621383584718842</v>
+        <f t="shared" ref="N25:N41" si="18">IFERROR(0.5*_xlfn.CHISQ.INV(1-$B$3/2,2*($J25+1))/$G25*$B$20, 0)</f>
+        <v>0.23719286870795328</v>
       </c>
     </row>
     <row r="26" spans="1:24">
       <c r="A26" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>incidence_clin_57</v>
+        <v>incidence_clin_12</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C26" s="1">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="D26" s="1">
+        <f t="shared" ref="D26:D40" si="19">C27</f>
+        <v>15</v>
+      </c>
+      <c r="E26" s="1">
         <f t="shared" si="12"/>
-        <v>60</v>
-      </c>
-      <c r="E26" s="1">
+        <v>12</v>
+      </c>
+      <c r="F26" s="1">
+        <v>102304</v>
+      </c>
+      <c r="G26" s="1">
         <f t="shared" si="13"/>
-        <v>57</v>
-      </c>
-      <c r="F26" s="1">
-        <v>49077</v>
-      </c>
-      <c r="G26" s="1">
+        <v>12224672.231360001</v>
+      </c>
+      <c r="H26" s="1">
         <f t="shared" si="14"/>
-        <v>5864386.9164300002</v>
-      </c>
-      <c r="H26" s="1">
+        <v>0</v>
+      </c>
+      <c r="I26" s="1">
         <f t="shared" si="15"/>
-        <v>2011.48471233549</v>
-      </c>
-      <c r="I26" s="1">
+        <v>0</v>
+      </c>
+      <c r="J26" s="1">
         <f t="shared" si="16"/>
-        <v>2008.5525188772749</v>
-      </c>
-      <c r="J26" s="1">
+        <v>6.1123361156800007</v>
+      </c>
+      <c r="K26" s="1">
+        <v>0</v>
+      </c>
+      <c r="M26" s="1">
         <f t="shared" si="17"/>
-        <v>2014.4169057937047</v>
-      </c>
-      <c r="K26" s="1">
-        <v>34.299999999999997</v>
-      </c>
-      <c r="L26" s="1">
-        <f>SUM(H26:H27)/$H$33</f>
-        <v>0.23794089963851275</v>
-      </c>
-      <c r="M26" s="1">
+        <v>0</v>
+      </c>
+      <c r="N26" s="1">
         <f t="shared" si="18"/>
-        <v>32.767494120937265</v>
-      </c>
-      <c r="N26" s="1">
-        <f t="shared" si="19"/>
-        <v>35.876275809580278</v>
+        <v>0.10682882759847878</v>
       </c>
     </row>
     <row r="27" spans="1:24">
       <c r="A27" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>incidence_clin_62</v>
+        <v>incidence_clin_17</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C27" s="1">
-        <v>60</v>
+        <v>15</v>
       </c>
       <c r="D27" s="1">
+        <f t="shared" si="19"/>
+        <v>20</v>
+      </c>
+      <c r="E27" s="1">
         <f t="shared" si="12"/>
-        <v>65</v>
-      </c>
-      <c r="E27" s="1">
+        <v>17</v>
+      </c>
+      <c r="F27" s="1">
+        <v>93845</v>
+      </c>
+      <c r="G27" s="1">
         <f t="shared" si="13"/>
-        <v>62</v>
-      </c>
-      <c r="F27" s="1">
-        <v>42403</v>
-      </c>
-      <c r="G27" s="1">
+        <v>11213875.95355</v>
+      </c>
+      <c r="H27" s="1">
         <f t="shared" si="14"/>
-        <v>5066886.6967700003</v>
-      </c>
-      <c r="H27" s="1">
+        <v>11.213875953550001</v>
+      </c>
+      <c r="I27" s="1">
         <f t="shared" si="15"/>
-        <v>2680.3830625913301</v>
-      </c>
-      <c r="I27" s="1">
+        <v>5.6069379767750007</v>
+      </c>
+      <c r="J27" s="1">
         <f t="shared" si="16"/>
-        <v>2677.8496192429452</v>
-      </c>
-      <c r="J27" s="1">
+        <v>16.820813930325002</v>
+      </c>
+      <c r="K27" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="M27" s="1">
         <f t="shared" si="17"/>
-        <v>2682.9165059397151</v>
-      </c>
-      <c r="K27" s="1">
-        <v>52.9</v>
-      </c>
-      <c r="M27" s="1">
+        <v>1.7013511956265843E-2</v>
+      </c>
+      <c r="N27" s="1">
         <f t="shared" si="18"/>
-        <v>50.860284058021669</v>
-      </c>
-      <c r="N27" s="1">
-        <f t="shared" si="19"/>
-        <v>54.983958159669321</v>
+        <v>0.23722104989583823</v>
       </c>
     </row>
     <row r="28" spans="1:24">
       <c r="A28" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>incidence_clin_67</v>
+        <v>incidence_clin_22</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C28" s="1">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="D28" s="1">
+        <f t="shared" si="19"/>
+        <v>25</v>
+      </c>
+      <c r="E28" s="1">
         <f t="shared" si="12"/>
-        <v>70</v>
-      </c>
-      <c r="E28" s="1">
+        <v>22</v>
+      </c>
+      <c r="F28" s="1">
+        <v>80561</v>
+      </c>
+      <c r="G28" s="1">
         <f t="shared" si="13"/>
-        <v>67</v>
-      </c>
-      <c r="F28" s="1">
-        <v>34406</v>
-      </c>
-      <c r="G28" s="1">
+        <v>9626523.1039899997</v>
+      </c>
+      <c r="H28" s="1">
         <f t="shared" si="14"/>
-        <v>4111296.4575399999</v>
-      </c>
-      <c r="H28" s="1">
+        <v>28.879569311969998</v>
+      </c>
+      <c r="I28" s="1">
         <f t="shared" si="15"/>
-        <v>3404.15346684312</v>
-      </c>
-      <c r="I28" s="1">
+        <v>24.066307759975</v>
+      </c>
+      <c r="J28" s="1">
         <f t="shared" si="16"/>
-        <v>3402.0978186143498</v>
-      </c>
-      <c r="J28" s="1">
+        <v>33.692830863964993</v>
+      </c>
+      <c r="K28" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="L28" s="1">
+        <f>SUM(H28:H30)/H42</f>
+        <v>7.0026509067945388E-3</v>
+      </c>
+      <c r="M28" s="1">
         <f t="shared" si="17"/>
-        <v>3406.2091150718898</v>
-      </c>
-      <c r="K28" s="1">
-        <v>82.8</v>
-      </c>
-      <c r="L28" s="1">
-        <f>SUM(H28:H29)/$H$33</f>
-        <v>0.34974893084572212</v>
-      </c>
-      <c r="M28" s="1">
+        <v>0.1597383882900868</v>
+      </c>
+      <c r="N28" s="1">
         <f t="shared" si="18"/>
-        <v>79.990143004942581</v>
-      </c>
-      <c r="N28" s="1">
-        <f t="shared" si="19"/>
-        <v>85.674831914507308</v>
+        <v>0.4874889418786299</v>
       </c>
     </row>
     <row r="29" spans="1:24">
       <c r="A29" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>incidence_clin_72</v>
+        <v>incidence_clin_27</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C29" s="1">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="D29" s="1">
+        <f t="shared" si="19"/>
+        <v>30</v>
+      </c>
+      <c r="E29" s="1">
         <f t="shared" si="12"/>
-        <v>75</v>
-      </c>
-      <c r="E29" s="1">
+        <v>27</v>
+      </c>
+      <c r="F29" s="1">
+        <v>66320</v>
+      </c>
+      <c r="G29" s="1">
         <f t="shared" si="13"/>
-        <v>72</v>
-      </c>
-      <c r="F29" s="1">
-        <v>26789</v>
-      </c>
-      <c r="G29" s="1">
+        <v>7924814.8888000008</v>
+      </c>
+      <c r="H29" s="1">
         <f t="shared" si="14"/>
-        <v>3201113.7825100003</v>
-      </c>
-      <c r="H29" s="1">
+        <v>39.624074444000001</v>
+      </c>
+      <c r="I29" s="1">
         <f t="shared" si="15"/>
-        <v>3492.4151367184104</v>
-      </c>
-      <c r="I29" s="1">
+        <v>35.661666999600001</v>
+      </c>
+      <c r="J29" s="1">
         <f t="shared" si="16"/>
-        <v>3490.8145798271553</v>
-      </c>
-      <c r="J29" s="1">
+        <v>43.586481888400009</v>
+      </c>
+      <c r="K29" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M29" s="1">
         <f t="shared" si="17"/>
-        <v>3494.015693609665</v>
-      </c>
-      <c r="K29" s="1">
-        <v>109.1</v>
-      </c>
-      <c r="M29" s="1">
+        <v>0.31289158139055295</v>
+      </c>
+      <c r="N29" s="1">
         <f t="shared" si="18"/>
-        <v>105.45249909757202</v>
-      </c>
-      <c r="N29" s="1">
-        <f t="shared" si="19"/>
-        <v>112.82992889659357</v>
+        <v>0.73811868911234746</v>
       </c>
     </row>
     <row r="30" spans="1:24">
       <c r="A30" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>incidence_clin_77</v>
+        <v>incidence_clin_32</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C30" s="1">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="D30" s="1">
+        <f t="shared" si="19"/>
+        <v>35</v>
+      </c>
+      <c r="E30" s="1">
         <f t="shared" si="12"/>
-        <v>80</v>
-      </c>
-      <c r="E30" s="1">
+        <v>32</v>
+      </c>
+      <c r="F30" s="1">
+        <v>56249</v>
+      </c>
+      <c r="G30" s="1">
         <f t="shared" si="13"/>
-        <v>77</v>
-      </c>
-      <c r="F30" s="1">
-        <v>18871</v>
-      </c>
-      <c r="G30" s="1">
+        <v>6721394.9439099999</v>
+      </c>
+      <c r="H30" s="1">
         <f t="shared" si="14"/>
-        <v>2254963.5368899996</v>
-      </c>
-      <c r="H30" s="1">
+        <v>73.935344383010005</v>
+      </c>
+      <c r="I30" s="1">
         <f t="shared" si="15"/>
-        <v>2981.061795768579</v>
-      </c>
-      <c r="I30" s="1">
+        <v>70.574646911054998</v>
+      </c>
+      <c r="J30" s="1">
         <f t="shared" si="16"/>
-        <v>2979.9343140001338</v>
-      </c>
-      <c r="J30" s="1">
+        <v>77.296041854965011</v>
+      </c>
+      <c r="K30" s="1">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M30" s="1">
         <f t="shared" si="17"/>
-        <v>2982.1892775370247</v>
-      </c>
-      <c r="K30" s="1">
-        <v>132.19999999999999</v>
-      </c>
-      <c r="L30" s="1">
-        <f>SUM(H30:H31)/$H$33</f>
-        <v>0.2528827412332742</v>
-      </c>
-      <c r="M30" s="1">
+        <v>0.8184299276747744</v>
+      </c>
+      <c r="N30" s="1">
         <f t="shared" si="18"/>
-        <v>127.42849266253278</v>
-      </c>
-      <c r="N30" s="1">
-        <f t="shared" si="19"/>
-        <v>137.07498967213519</v>
+        <v>1.4317978530233426</v>
       </c>
     </row>
     <row r="31" spans="1:24">
       <c r="A31" s="1" t="str">
         <f t="shared" si="11"/>
-        <v>incidence_clin_82</v>
+        <v>incidence_clin_37</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C31" s="1">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="D31" s="1">
+        <f t="shared" si="19"/>
+        <v>40</v>
+      </c>
+      <c r="E31" s="1">
         <f t="shared" si="12"/>
-        <v>85</v>
-      </c>
-      <c r="E31" s="1">
+        <v>37</v>
+      </c>
+      <c r="F31" s="1">
+        <v>54656</v>
+      </c>
+      <c r="G31" s="1">
         <f t="shared" si="13"/>
-        <v>82</v>
-      </c>
-      <c r="F31" s="1">
-        <v>11241</v>
-      </c>
-      <c r="G31" s="1">
+        <v>6531041.6550400006</v>
+      </c>
+      <c r="H31" s="1">
         <f t="shared" si="14"/>
-        <v>1343227.4451899999</v>
-      </c>
-      <c r="H31" s="1">
+        <v>143.68291641088004</v>
+      </c>
+      <c r="I31" s="1">
         <f t="shared" si="15"/>
-        <v>2005.43857566867</v>
-      </c>
-      <c r="I31" s="1">
+        <v>140.41739558336002</v>
+      </c>
+      <c r="J31" s="1">
         <f t="shared" si="16"/>
-        <v>2004.7669619460751</v>
-      </c>
-      <c r="J31" s="1">
+        <v>146.94843723840003</v>
+      </c>
+      <c r="K31" s="1">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="L31" s="1">
+        <f>SUM(H31:H32)/$H$42</f>
+        <v>2.1957052888418878E-2</v>
+      </c>
+      <c r="M31" s="1">
         <f t="shared" si="17"/>
-        <v>2006.1101893912653</v>
-      </c>
-      <c r="K31" s="1">
-        <v>149.30000000000001</v>
-      </c>
-      <c r="M31" s="1">
+        <v>1.8032433025804822</v>
+      </c>
+      <c r="N31" s="1">
         <f t="shared" si="18"/>
-        <v>142.7680888200511</v>
-      </c>
-      <c r="N31" s="1">
-        <f t="shared" si="19"/>
-        <v>156.02337488989809</v>
+        <v>2.6371938700704867</v>
       </c>
     </row>
     <row r="32" spans="1:24">
       <c r="A32" s="1" t="str">
         <f t="shared" si="11"/>
+        <v>incidence_clin_42</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C32" s="1">
+        <v>40</v>
+      </c>
+      <c r="D32" s="1">
+        <f t="shared" si="19"/>
+        <v>45</v>
+      </c>
+      <c r="E32" s="1">
+        <f t="shared" si="12"/>
+        <v>42</v>
+      </c>
+      <c r="F32" s="1">
+        <v>58958</v>
+      </c>
+      <c r="G32" s="1">
+        <f t="shared" si="13"/>
+        <v>7045103.0792200007</v>
+      </c>
+      <c r="H32" s="1">
+        <f t="shared" si="14"/>
+        <v>302.93943240646001</v>
+      </c>
+      <c r="I32" s="1">
+        <f t="shared" si="15"/>
+        <v>299.41688086685002</v>
+      </c>
+      <c r="J32" s="1">
+        <f t="shared" si="16"/>
+        <v>306.46198394607001</v>
+      </c>
+      <c r="K32" s="1">
+        <v>4.3</v>
+      </c>
+      <c r="M32" s="1">
+        <f t="shared" si="17"/>
+        <v>3.7766078728748678</v>
+      </c>
+      <c r="N32" s="1">
+        <f t="shared" si="18"/>
+        <v>4.8583883346410159</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
+      <c r="A33" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_47</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="1">
+        <v>45</v>
+      </c>
+      <c r="D33" s="1">
+        <f t="shared" si="19"/>
+        <v>50</v>
+      </c>
+      <c r="E33" s="1">
+        <f t="shared" si="12"/>
+        <v>47</v>
+      </c>
+      <c r="F33" s="1">
+        <v>59622</v>
+      </c>
+      <c r="G33" s="1">
+        <f t="shared" si="13"/>
+        <v>7124446.8229799997</v>
+      </c>
+      <c r="H33" s="1">
+        <f t="shared" si="14"/>
+        <v>676.82244818309994</v>
+      </c>
+      <c r="I33" s="1">
+        <f t="shared" si="15"/>
+        <v>673.26022477160996</v>
+      </c>
+      <c r="J33" s="1">
+        <f t="shared" si="16"/>
+        <v>680.38467159458992</v>
+      </c>
+      <c r="K33" s="1">
+        <v>9.5</v>
+      </c>
+      <c r="L33" s="1">
+        <f>SUM(H33:H34)/$H$42</f>
+        <v>9.2660309853476744E-2</v>
+      </c>
+      <c r="M33" s="1">
+        <f t="shared" si="17"/>
+        <v>8.7460518806358838</v>
+      </c>
+      <c r="N33" s="1">
+        <f t="shared" si="18"/>
+        <v>10.289748213803048</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
+      <c r="A34" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_52</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="1">
+        <v>50</v>
+      </c>
+      <c r="D34" s="1">
+        <f t="shared" si="19"/>
+        <v>55</v>
+      </c>
+      <c r="E34" s="1">
+        <f t="shared" si="12"/>
+        <v>52</v>
+      </c>
+      <c r="F34" s="1">
+        <v>54643</v>
+      </c>
+      <c r="G34" s="1">
+        <f t="shared" si="13"/>
+        <v>6529488.2383699995</v>
+      </c>
+      <c r="H34" s="1">
+        <f t="shared" si="14"/>
+        <v>1207.9553240984499</v>
+      </c>
+      <c r="I34" s="1">
+        <f t="shared" si="15"/>
+        <v>1204.6905799792648</v>
+      </c>
+      <c r="J34" s="1">
+        <f t="shared" si="16"/>
+        <v>1211.2200682176351</v>
+      </c>
+      <c r="K34" s="1">
+        <v>18.5</v>
+      </c>
+      <c r="M34" s="1">
+        <f t="shared" si="17"/>
+        <v>17.419890817649691</v>
+      </c>
+      <c r="N34" s="1">
+        <f t="shared" si="18"/>
+        <v>19.621383584718842</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
+      <c r="A35" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_57</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C35" s="1">
+        <v>55</v>
+      </c>
+      <c r="D35" s="1">
+        <f t="shared" si="19"/>
+        <v>60</v>
+      </c>
+      <c r="E35" s="1">
+        <f t="shared" si="12"/>
+        <v>57</v>
+      </c>
+      <c r="F35" s="1">
+        <v>49077</v>
+      </c>
+      <c r="G35" s="1">
+        <f t="shared" si="13"/>
+        <v>5864386.9164300002</v>
+      </c>
+      <c r="H35" s="1">
+        <f t="shared" si="14"/>
+        <v>2011.48471233549</v>
+      </c>
+      <c r="I35" s="1">
+        <f t="shared" si="15"/>
+        <v>2008.5525188772749</v>
+      </c>
+      <c r="J35" s="1">
+        <f t="shared" si="16"/>
+        <v>2014.4169057937047</v>
+      </c>
+      <c r="K35" s="1">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="L35" s="1">
+        <f>SUM(H35:H36)/$H$42</f>
+        <v>0.23066375686826504</v>
+      </c>
+      <c r="M35" s="1">
+        <f t="shared" si="17"/>
+        <v>32.767494120937265</v>
+      </c>
+      <c r="N35" s="1">
+        <f t="shared" si="18"/>
+        <v>35.876275809580278</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_62</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C36" s="1">
+        <v>60</v>
+      </c>
+      <c r="D36" s="1">
+        <f t="shared" si="19"/>
+        <v>65</v>
+      </c>
+      <c r="E36" s="1">
+        <f t="shared" si="12"/>
+        <v>62</v>
+      </c>
+      <c r="F36" s="1">
+        <v>42403</v>
+      </c>
+      <c r="G36" s="1">
+        <f t="shared" si="13"/>
+        <v>5066886.6967700003</v>
+      </c>
+      <c r="H36" s="1">
+        <f t="shared" si="14"/>
+        <v>2680.3830625913301</v>
+      </c>
+      <c r="I36" s="1">
+        <f t="shared" si="15"/>
+        <v>2677.8496192429452</v>
+      </c>
+      <c r="J36" s="1">
+        <f t="shared" si="16"/>
+        <v>2682.9165059397151</v>
+      </c>
+      <c r="K36" s="1">
+        <v>52.9</v>
+      </c>
+      <c r="M36" s="1">
+        <f t="shared" si="17"/>
+        <v>50.860284058021669</v>
+      </c>
+      <c r="N36" s="1">
+        <f t="shared" si="18"/>
+        <v>54.983958159669321</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
+      <c r="A37" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_67</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" s="1">
+        <v>65</v>
+      </c>
+      <c r="D37" s="1">
+        <f t="shared" si="19"/>
+        <v>70</v>
+      </c>
+      <c r="E37" s="1">
+        <f t="shared" si="12"/>
+        <v>67</v>
+      </c>
+      <c r="F37" s="1">
+        <v>34406</v>
+      </c>
+      <c r="G37" s="1">
+        <f t="shared" si="13"/>
+        <v>4111296.4575399999</v>
+      </c>
+      <c r="H37" s="1">
+        <f t="shared" si="14"/>
+        <v>3404.15346684312</v>
+      </c>
+      <c r="I37" s="1">
+        <f t="shared" si="15"/>
+        <v>3402.0978186143498</v>
+      </c>
+      <c r="J37" s="1">
+        <f t="shared" si="16"/>
+        <v>3406.2091150718898</v>
+      </c>
+      <c r="K37" s="1">
+        <v>82.8</v>
+      </c>
+      <c r="L37" s="1">
+        <f>SUM(H37:H38)/$H$42</f>
+        <v>0.33905227084581235</v>
+      </c>
+      <c r="M37" s="1">
+        <f t="shared" si="17"/>
+        <v>79.990143004942581</v>
+      </c>
+      <c r="N37" s="1">
+        <f t="shared" si="18"/>
+        <v>85.674831914507308</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
+      <c r="A38" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_72</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C38" s="1">
+        <v>70</v>
+      </c>
+      <c r="D38" s="1">
+        <f t="shared" si="19"/>
+        <v>75</v>
+      </c>
+      <c r="E38" s="1">
+        <f t="shared" si="12"/>
+        <v>72</v>
+      </c>
+      <c r="F38" s="1">
+        <v>26789</v>
+      </c>
+      <c r="G38" s="1">
+        <f t="shared" si="13"/>
+        <v>3201113.7825100003</v>
+      </c>
+      <c r="H38" s="1">
+        <f t="shared" si="14"/>
+        <v>3492.4151367184104</v>
+      </c>
+      <c r="I38" s="1">
+        <f t="shared" si="15"/>
+        <v>3490.8145798271553</v>
+      </c>
+      <c r="J38" s="1">
+        <f t="shared" si="16"/>
+        <v>3494.015693609665</v>
+      </c>
+      <c r="K38" s="1">
+        <v>109.1</v>
+      </c>
+      <c r="M38" s="1">
+        <f t="shared" si="17"/>
+        <v>105.45249909757202</v>
+      </c>
+      <c r="N38" s="1">
+        <f t="shared" si="18"/>
+        <v>112.82992889659357</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
+      <c r="A39" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_77</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C39" s="1">
+        <v>75</v>
+      </c>
+      <c r="D39" s="1">
+        <f t="shared" si="19"/>
+        <v>80</v>
+      </c>
+      <c r="E39" s="1">
+        <f t="shared" si="12"/>
+        <v>77</v>
+      </c>
+      <c r="F39" s="1">
+        <v>18871</v>
+      </c>
+      <c r="G39" s="1">
+        <f t="shared" si="13"/>
+        <v>2254963.5368899996</v>
+      </c>
+      <c r="H39" s="1">
+        <f t="shared" si="14"/>
+        <v>2981.061795768579</v>
+      </c>
+      <c r="I39" s="1">
+        <f t="shared" si="15"/>
+        <v>2979.9343140001338</v>
+      </c>
+      <c r="J39" s="1">
+        <f t="shared" si="16"/>
+        <v>2982.1892775370247</v>
+      </c>
+      <c r="K39" s="1">
+        <v>132.19999999999999</v>
+      </c>
+      <c r="L39" s="1">
+        <f>SUM(H39:H40)/$H$42</f>
+        <v>0.24514861979857369</v>
+      </c>
+      <c r="M39" s="1">
+        <f t="shared" si="17"/>
+        <v>127.42849266253278</v>
+      </c>
+      <c r="N39" s="1">
+        <f t="shared" si="18"/>
+        <v>137.07498967213519</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
+      <c r="A40" s="1" t="str">
+        <f t="shared" si="11"/>
+        <v>incidence_clin_82</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C40" s="1">
+        <v>80</v>
+      </c>
+      <c r="D40" s="1">
+        <f t="shared" si="19"/>
+        <v>85</v>
+      </c>
+      <c r="E40" s="1">
+        <f t="shared" si="12"/>
+        <v>82</v>
+      </c>
+      <c r="F40" s="1">
+        <v>11241</v>
+      </c>
+      <c r="G40" s="1">
+        <f t="shared" si="13"/>
+        <v>1343227.4451899999</v>
+      </c>
+      <c r="H40" s="1">
+        <f t="shared" si="14"/>
+        <v>2005.43857566867</v>
+      </c>
+      <c r="I40" s="1">
+        <f t="shared" si="15"/>
+        <v>2004.7669619460751</v>
+      </c>
+      <c r="J40" s="1">
+        <f t="shared" si="16"/>
+        <v>2006.1101893912653</v>
+      </c>
+      <c r="K40" s="1">
+        <v>149.30000000000001</v>
+      </c>
+      <c r="M40" s="1">
+        <f t="shared" si="17"/>
+        <v>142.7680888200511</v>
+      </c>
+      <c r="N40" s="1">
+        <f t="shared" si="18"/>
+        <v>156.02337488989809</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" s="1" t="str">
+        <f t="shared" si="11"/>
         <v>incidence_clin_92</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C32" s="1">
+      <c r="B41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C41" s="1">
         <v>85</v>
       </c>
-      <c r="D32" s="1">
+      <c r="D41" s="1">
         <v>100</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E41" s="1">
+        <f t="shared" si="12"/>
+        <v>92</v>
+      </c>
+      <c r="F41" s="1">
+        <v>7435</v>
+      </c>
+      <c r="G41" s="1">
         <f t="shared" si="13"/>
-        <v>92</v>
-      </c>
-      <c r="F32" s="1">
-        <v>7435</v>
-      </c>
-      <c r="G32" s="1">
+        <v>888434.84165000007</v>
+      </c>
+      <c r="H41" s="1">
         <f t="shared" si="14"/>
-        <v>888434.84165000007</v>
-      </c>
-      <c r="H32" s="1">
+        <v>1258.9121706180499</v>
+      </c>
+      <c r="I41" s="1">
         <f t="shared" si="15"/>
-        <v>1258.9121706180499</v>
-      </c>
-      <c r="I32" s="1">
+        <v>1258.4679531972249</v>
+      </c>
+      <c r="J41" s="1">
         <f t="shared" si="16"/>
-        <v>1258.4679531972249</v>
-      </c>
-      <c r="J32" s="1">
+        <v>1259.3563880388751</v>
+      </c>
+      <c r="K41" s="1">
+        <v>141.69999999999999</v>
+      </c>
+      <c r="L41" s="1">
+        <f>H41/H42</f>
+        <v>6.1891217905532488E-2</v>
+      </c>
+      <c r="M41" s="1">
         <f t="shared" si="17"/>
-        <v>1259.3563880388751</v>
-      </c>
-      <c r="K32" s="1">
-        <v>141.69999999999999</v>
-      </c>
-      <c r="L32" s="1">
-        <f>H32/H33</f>
-        <v>6.3843805668075071E-2</v>
-      </c>
-      <c r="M32" s="1">
+        <v>133.87986472565848</v>
+      </c>
+      <c r="N41" s="1">
         <f t="shared" si="18"/>
-        <v>133.87986472565848</v>
-      </c>
-      <c r="N32" s="1">
-        <f t="shared" si="19"/>
         <v>149.75933097441057</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
-      <c r="A33" s="1" t="s">
+    <row r="42" spans="1:14">
+      <c r="A42" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F33" s="1">
-        <f>SUM(F24:F32)</f>
-        <v>304487</v>
-      </c>
-      <c r="G33" s="1">
-        <f>SUM(G24:G32)</f>
-        <v>36384244.738329999</v>
-      </c>
-      <c r="H33" s="1">
-        <f>SUM(H24:H32)</f>
-        <v>19718.626692825201</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="1" t="s">
+      <c r="F42" s="1">
+        <f>SUM(F24:F41)</f>
+        <v>1000000</v>
+      </c>
+      <c r="G42" s="1">
+        <f>SUM(G24:G41)</f>
+        <v>119493589.99999999</v>
+      </c>
+      <c r="H42" s="1">
+        <f>SUM(H24:H41)</f>
+        <v>20340.723825140871</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
+      <c r="A43" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F34" s="3"/>
-      <c r="G34" s="1">
-        <f>G33/(B19-B18+1)</f>
-        <v>7276848.9476659996</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="F35" s="3"/>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="F36" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="1">
+        <f>G42/(B19-B18+1)</f>
+        <v>23898717.999999996</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
+      <c r="F44" s="3"/>
+    </row>
+    <row r="45" spans="1:14">
+      <c r="F45" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update priors and IMABC parameters for bladder
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00AED7BB-E58C-4F48-8EC2-4DFA1A178ABB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D4A166-D8C2-D548-A369-E9103D12B16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="37">
   <si>
     <t>target_names</t>
   </si>
@@ -547,7 +547,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -592,7 +592,7 @@
     </row>
     <row r="2" spans="1:11">
       <c r="A2" s="1" t="str">
-        <f t="shared" ref="A2:A25" si="0">""&amp;B2&amp;"_"&amp;E2</f>
+        <f t="shared" ref="A2:A24" si="0">""&amp;B2&amp;"_"&amp;E2</f>
         <v>prevalence_preclin_71</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -605,7 +605,7 @@
         <v>76</v>
       </c>
       <c r="E2" s="1">
-        <f t="shared" ref="E2:E22" si="1">FLOOR(AVERAGE(C2,D2), 1)</f>
+        <f t="shared" ref="E2:E21" si="1">FLOOR(AVERAGE(C2,D2), 1)</f>
         <v>71</v>
       </c>
       <c r="F2" s="2">
@@ -814,7 +814,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="1">
-        <f t="shared" ref="D7:D21" si="4">C8</f>
+        <f t="shared" ref="D7:D20" si="4">C8</f>
         <v>15</v>
       </c>
       <c r="E7" s="1">
@@ -976,7 +976,7 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="1" t="str">
-        <f t="shared" ref="A11:A22" si="5">""&amp;B11&amp;"_"&amp;E11</f>
+        <f t="shared" ref="A11:A21" si="5">""&amp;B11&amp;"_"&amp;E11</f>
         <v>incidence_clin_32</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1416,7 +1416,6 @@
         <v>80</v>
       </c>
       <c r="D21" s="1">
-        <f t="shared" si="4"/>
         <v>85</v>
       </c>
       <c r="E21" s="1">
@@ -1449,41 +1448,34 @@
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v>incidence_clin_92</v>
+        <f t="shared" si="0"/>
+        <v>stage_distr_1</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="1">
-        <v>85</v>
-      </c>
-      <c r="D22" s="1">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="E22" s="1">
-        <f t="shared" si="1"/>
-        <v>92</v>
+        <v>1</v>
       </c>
       <c r="F22" s="2">
-        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
-        <v>1258.9121706180499</v>
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <v>21522.9</v>
       </c>
       <c r="G22" s="2">
-        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
-        <v>888434.84165000007</v>
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <v>27630.75</v>
       </c>
       <c r="H22" s="2">
-        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
-        <v>141.69999999999999</v>
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>0.77894736842105272</v>
       </c>
       <c r="I22" s="2">
-        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
-        <v>133.87986472565848</v>
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>0.77401602151958493</v>
       </c>
       <c r="J22" s="2">
-        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
-        <v>149.75933097441057</v>
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
+        <v>0.78380116289475799</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>21</v>
@@ -1492,17 +1484,17 @@
     <row r="23" spans="1:11">
       <c r="A23" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>stage_distr_1</v>
+        <v>stage_distr_2</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E23" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>21522.9</v>
+        <v>5235.3</v>
       </c>
       <c r="G23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
@@ -1510,15 +1502,15 @@
       </c>
       <c r="H23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.77894736842105272</v>
+        <v>0.18947368421052632</v>
       </c>
       <c r="I23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>0.77401602151958493</v>
+        <v>0.18489624853500833</v>
       </c>
       <c r="J23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>0.78380116289475799</v>
+        <v>0.19413745183393108</v>
       </c>
       <c r="K23" s="1" t="s">
         <v>21</v>
@@ -1527,17 +1519,17 @@
     <row r="24" spans="1:11">
       <c r="A24" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>stage_distr_2</v>
+        <v>stage_distr_3</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E24" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>5235.3</v>
+        <v>872.55</v>
       </c>
       <c r="G24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
@@ -1545,52 +1537,17 @@
       </c>
       <c r="H24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.18947368421052632</v>
+        <v>3.1578947368421054E-2</v>
       </c>
       <c r="I24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>0.18489624853500833</v>
+        <v>2.9581205871892616E-2</v>
       </c>
       <c r="J24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>0.19413745183393108</v>
+        <v>3.3706918413456612E-2</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11">
-      <c r="A25" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>stage_distr_3</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E25" s="1">
-        <v>3</v>
-      </c>
-      <c r="F25" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>872.55</v>
-      </c>
-      <c r="G25" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>27630.75</v>
-      </c>
-      <c r="H25" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>3.1578947368421054E-2</v>
-      </c>
-      <c r="I25" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>2.9581205871892616E-2</v>
-      </c>
-      <c r="J25" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>3.3706918413456612E-2</v>
-      </c>
-      <c r="K25" s="1" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update lesion multiplicity calculation, expand target starting bounds for IMABC
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7D4A166-D8C2-D548-A369-E9103D12B16E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF2C031-9D37-C04D-9CA9-CCDE41189EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="39">
   <si>
     <t>target_names</t>
   </si>
@@ -148,6 +148,12 @@
   </si>
   <si>
     <t>n_cases_ub</t>
+  </si>
+  <si>
+    <t>current_lower_bounds</t>
+  </si>
+  <si>
+    <t>current_upper_bounds</t>
   </si>
 </sst>
 </file>
@@ -547,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -555,7 +561,7 @@
     <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:13">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -587,10 +593,16 @@
         <v>10</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:13">
       <c r="A2" s="1" t="str">
         <f t="shared" ref="A2:A24" si="0">""&amp;B2&amp;"_"&amp;E2</f>
         <v>prevalence_preclin_71</v>
@@ -628,11 +640,19 @@
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>3.1229562615372915E-3</v>
       </c>
-      <c r="K2" s="1" t="s">
+      <c r="K2" s="2">
+        <f>IF(H2 - 6*(H2-I2) &lt; 0, 0, H2 - 6*(H2-I2))</f>
+        <v>0</v>
+      </c>
+      <c r="L2" s="2">
+        <f>H2 + 6*(J2-H2)</f>
+        <v>1.597530662999723E-2</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:13">
       <c r="A3" s="1" t="str">
         <f t="shared" si="0"/>
         <v>prevalence_preclin_80</v>
@@ -670,11 +690,19 @@
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>5.562261593248006E-3</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="K3" s="2">
+        <f t="shared" ref="K3:K24" si="2">IF(H3 - 6*(H3-I3) &lt; 0, 0, H3 - 6*(H3-I3))</f>
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <f t="shared" ref="L3:L24" si="3">H3 + 6*(J3-H3)</f>
+        <v>2.572246014862346E-2</v>
+      </c>
+      <c r="M3" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:13">
       <c r="A4" s="1" t="str">
         <f t="shared" si="0"/>
         <v>prevalence_preclin_90</v>
@@ -712,13 +740,21 @@
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>2.7692132896306509E-2</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L4" s="2">
+        <f t="shared" si="3"/>
+        <v>0.10634418493764766</v>
+      </c>
+      <c r="M4" s="1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:13">
       <c r="A5" s="1" t="str">
-        <f t="shared" ref="A5:A10" si="2">""&amp;B5&amp;"_"&amp;E5</f>
+        <f t="shared" ref="A5:A10" si="4">""&amp;B5&amp;"_"&amp;E5</f>
         <v>incidence_clin_2</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -728,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="1">
-        <f t="shared" ref="D5" si="3">C6</f>
+        <f t="shared" ref="D5" si="5">C6</f>
         <v>5</v>
       </c>
       <c r="E5" s="1">
@@ -755,13 +791,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A5,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.24526419878119815</v>
       </c>
-      <c r="K5" s="1" t="s">
+      <c r="K5" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L5" s="2">
+        <f>H5 + 6*(J5-H5)</f>
+        <v>0.9715851926871889</v>
+      </c>
+      <c r="M5" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:13">
       <c r="A6" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>incidence_clin_7</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -798,13 +842,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A6,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.23719286870795328</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="K6" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L6" s="2">
+        <f>H6 + 6*(J6-H6)</f>
+        <v>0.92315721224771963</v>
+      </c>
+      <c r="M6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:13">
       <c r="A7" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>incidence_clin_12</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -814,7 +866,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="1">
-        <f t="shared" ref="D7:D20" si="4">C8</f>
+        <f t="shared" ref="D7:D20" si="6">C8</f>
         <v>15</v>
       </c>
       <c r="E7" s="1">
@@ -841,13 +893,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A7,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.10682882759847878</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L7" s="2">
+        <f t="shared" si="3"/>
+        <v>0.64097296559087269</v>
+      </c>
+      <c r="M7" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:13">
       <c r="A8" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>incidence_clin_17</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -857,7 +917,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>20</v>
       </c>
       <c r="E8" s="1">
@@ -884,13 +944,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A8,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.23722104989583823</v>
       </c>
-      <c r="K8" s="1" t="s">
+      <c r="K8" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L8" s="2">
+        <f t="shared" si="3"/>
+        <v>0.9233262993750293</v>
+      </c>
+      <c r="M8" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:13">
       <c r="A9" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>incidence_clin_22</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -900,7 +968,7 @@
         <v>20</v>
       </c>
       <c r="D9" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>25</v>
       </c>
       <c r="E9" s="1">
@@ -927,13 +995,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A9,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.4874889418786299</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="K9" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L9" s="2">
+        <f t="shared" si="3"/>
+        <v>1.4249336512717796</v>
+      </c>
+      <c r="M9" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:13">
       <c r="A10" s="1" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>incidence_clin_27</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -943,7 +1019,7 @@
         <v>25</v>
       </c>
       <c r="D10" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>30</v>
       </c>
       <c r="E10" s="1">
@@ -970,13 +1046,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A10,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>0.73811868911234746</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="K10" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L10" s="2">
+        <f t="shared" si="3"/>
+        <v>1.9287121346740848</v>
+      </c>
+      <c r="M10" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:13">
       <c r="A11" s="1" t="str">
-        <f t="shared" ref="A11:A21" si="5">""&amp;B11&amp;"_"&amp;E11</f>
+        <f t="shared" ref="A11:A21" si="7">""&amp;B11&amp;"_"&amp;E11</f>
         <v>incidence_clin_32</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -986,7 +1070,7 @@
         <v>30</v>
       </c>
       <c r="D11" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>35</v>
       </c>
       <c r="E11" s="1">
@@ -1013,13 +1097,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A11,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>1.4317978530233426</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="K11" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L11" s="2">
+        <f t="shared" si="3"/>
+        <v>3.0907871181400552</v>
+      </c>
+      <c r="M11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:13">
       <c r="A12" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_37</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1029,7 +1121,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>40</v>
       </c>
       <c r="E12" s="1">
@@ -1056,13 +1148,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A12,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>2.6371938700704867</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="K12" s="2">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="L12" s="2">
+        <f t="shared" si="3"/>
+        <v>4.8231632204229191</v>
+      </c>
+      <c r="M12" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:13">
       <c r="A13" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_42</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -1072,7 +1172,7 @@
         <v>40</v>
       </c>
       <c r="D13" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>45</v>
       </c>
       <c r="E13" s="1">
@@ -1099,13 +1199,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A13,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>4.8583883346410159</v>
       </c>
-      <c r="K13" s="1" t="s">
+      <c r="K13" s="2">
+        <f t="shared" si="2"/>
+        <v>1.1596472372492075</v>
+      </c>
+      <c r="L13" s="2">
+        <f t="shared" si="3"/>
+        <v>7.6503300078460965</v>
+      </c>
+      <c r="M13" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:13">
       <c r="A14" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_47</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1115,7 +1223,7 @@
         <v>45</v>
       </c>
       <c r="D14" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>50</v>
       </c>
       <c r="E14" s="1">
@@ -1142,13 +1250,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A14,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>10.289748213803048</v>
       </c>
-      <c r="K14" s="1" t="s">
+      <c r="K14" s="2">
+        <f t="shared" si="2"/>
+        <v>4.9763112838153027</v>
+      </c>
+      <c r="L14" s="2">
+        <f t="shared" si="3"/>
+        <v>14.238489282818286</v>
+      </c>
+      <c r="M14" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:13">
       <c r="A15" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_52</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1158,7 +1274,7 @@
         <v>50</v>
       </c>
       <c r="D15" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>55</v>
       </c>
       <c r="E15" s="1">
@@ -1185,13 +1301,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A15,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>19.621383584718842</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="K15" s="2">
+        <f t="shared" si="2"/>
+        <v>12.019344905898144</v>
+      </c>
+      <c r="L15" s="2">
+        <f t="shared" si="3"/>
+        <v>25.228301508313052</v>
+      </c>
+      <c r="M15" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:13">
       <c r="A16" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_57</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1201,7 +1325,7 @@
         <v>55</v>
       </c>
       <c r="D16" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>60</v>
       </c>
       <c r="E16" s="1">
@@ -1228,13 +1352,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A16,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>35.876275809580278</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="K16" s="2">
+        <f t="shared" si="2"/>
+        <v>25.104964725623603</v>
+      </c>
+      <c r="L16" s="2">
+        <f t="shared" si="3"/>
+        <v>43.757654857481683</v>
+      </c>
+      <c r="M16" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:13">
       <c r="A17" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_62</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1244,7 +1376,7 @@
         <v>60</v>
       </c>
       <c r="D17" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>65</v>
       </c>
       <c r="E17" s="1">
@@ -1271,13 +1403,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A17,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>54.983958159669321</v>
       </c>
-      <c r="K17" s="1" t="s">
+      <c r="K17" s="2">
+        <f t="shared" si="2"/>
+        <v>40.661704348130023</v>
+      </c>
+      <c r="L17" s="2">
+        <f t="shared" si="3"/>
+        <v>65.403748958015939</v>
+      </c>
+      <c r="M17" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:13">
       <c r="A18" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_67</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1287,7 +1427,7 @@
         <v>65</v>
       </c>
       <c r="D18" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>70</v>
       </c>
       <c r="E18" s="1">
@@ -1314,13 +1454,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A18,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>85.674831914507308</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="K18" s="2">
+        <f t="shared" si="2"/>
+        <v>65.940858029655502</v>
+      </c>
+      <c r="L18" s="2">
+        <f t="shared" si="3"/>
+        <v>100.04899148704386</v>
+      </c>
+      <c r="M18" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:13">
       <c r="A19" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_72</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1330,7 +1478,7 @@
         <v>70</v>
       </c>
       <c r="D19" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>75</v>
       </c>
       <c r="E19" s="1">
@@ -1357,13 +1505,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A19,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>112.82992889659357</v>
       </c>
-      <c r="K19" s="1" t="s">
+      <c r="K19" s="2">
+        <f t="shared" si="2"/>
+        <v>87.214994585432123</v>
+      </c>
+      <c r="L19" s="2">
+        <f t="shared" si="3"/>
+        <v>131.47957337956146</v>
+      </c>
+      <c r="M19" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:13">
       <c r="A20" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_77</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1373,7 +1529,7 @@
         <v>75</v>
       </c>
       <c r="D20" s="1">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>80</v>
       </c>
       <c r="E20" s="1">
@@ -1400,13 +1556,21 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A20,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>137.07498967213519</v>
       </c>
-      <c r="K20" s="1" t="s">
+      <c r="K20" s="2">
+        <f t="shared" si="2"/>
+        <v>103.57095597519671</v>
+      </c>
+      <c r="L20" s="2">
+        <f t="shared" si="3"/>
+        <v>161.44993803281119</v>
+      </c>
+      <c r="M20" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:13">
       <c r="A21" s="1" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>incidence_clin_82</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1442,11 +1606,19 @@
         <f>INDEX(bounds!$23:$41,MATCH(targets!$A21,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
         <v>156.02337488989809</v>
       </c>
-      <c r="K21" s="1" t="s">
+      <c r="K21" s="2">
+        <f t="shared" si="2"/>
+        <v>110.10853292030657</v>
+      </c>
+      <c r="L21" s="2">
+        <f t="shared" si="3"/>
+        <v>189.6402493393885</v>
+      </c>
+      <c r="M21" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:13">
       <c r="A22" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_1</v>
@@ -1477,11 +1649,19 @@
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>0.78380116289475799</v>
       </c>
-      <c r="K22" s="1" t="s">
+      <c r="K22" s="2">
+        <f t="shared" si="2"/>
+        <v>0.74935928701224597</v>
+      </c>
+      <c r="L22" s="2">
+        <f t="shared" si="3"/>
+        <v>0.80807013526328431</v>
+      </c>
+      <c r="M22" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:13">
       <c r="A23" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_2</v>
@@ -1512,11 +1692,19 @@
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>0.19413745183393108</v>
       </c>
-      <c r="K23" s="1" t="s">
+      <c r="K23" s="2">
+        <f t="shared" si="2"/>
+        <v>0.16200907015741836</v>
+      </c>
+      <c r="L23" s="2">
+        <f t="shared" si="3"/>
+        <v>0.21745628995095487</v>
+      </c>
+      <c r="M23" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:13">
       <c r="A24" s="1" t="str">
         <f t="shared" si="0"/>
         <v>stage_distr_3</v>
@@ -1547,7 +1735,15 @@
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
         <v>3.3706918413456612E-2</v>
       </c>
-      <c r="K24" s="1" t="s">
+      <c r="K24" s="2">
+        <f t="shared" si="2"/>
+        <v>1.959249838925043E-2</v>
+      </c>
+      <c r="L24" s="2">
+        <f>H24 + 6*(J24-H24)</f>
+        <v>4.4346773638634401E-2</v>
+      </c>
+      <c r="M24" s="1" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Incorporate fitting log-logistic hazard for bladder priors
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DF2C031-9D37-C04D-9CA9-CCDE41189EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E53BC92-F4DC-A84D-9E08-9B24C8CE92EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
@@ -641,12 +641,12 @@
         <v>3.1229562615372915E-3</v>
       </c>
       <c r="K2" s="2">
-        <f>IF(H2 - 6*(H2-I2) &lt; 0, 0, H2 - 6*(H2-I2))</f>
+        <f>IF(H2 - 10*(H2-I2) &lt; 0, 0, H2 - 10*(H2-I2))</f>
         <v>0</v>
       </c>
       <c r="L2" s="2">
-        <f>H2 + 6*(J2-H2)</f>
-        <v>1.597530662999723E-2</v>
+        <f>H2 + 10*(J2-H2)</f>
+        <v>2.6257186924765179E-2</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>20</v>
@@ -691,12 +691,12 @@
         <v>5.562261593248006E-3</v>
       </c>
       <c r="K3" s="2">
-        <f t="shared" ref="K3:K24" si="2">IF(H3 - 6*(H3-I3) &lt; 0, 0, H3 - 6*(H3-I3))</f>
+        <f t="shared" ref="K3:K24" si="2">IF(H3 - 10*(H3-I3) &lt; 0, 0, H3 - 10*(H3-I3))</f>
         <v>0</v>
       </c>
       <c r="L3" s="2">
-        <f t="shared" ref="L3:L24" si="3">H3 + 6*(J3-H3)</f>
-        <v>2.572246014862346E-2</v>
+        <f t="shared" ref="L3:L24" si="3">H3 + 10*(J3-H3)</f>
+        <v>4.1850618992923819E-2</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>20</v>
@@ -705,7 +705,7 @@
     <row r="4" spans="1:13">
       <c r="A4" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>prevalence_preclin_90</v>
+        <v>prevalence_preclin_92</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>18</v>
@@ -714,11 +714,11 @@
         <v>85</v>
       </c>
       <c r="D4" s="2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E4" s="1">
         <f t="shared" si="1"/>
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
@@ -746,7 +746,7 @@
       </c>
       <c r="L4" s="2">
         <f t="shared" si="3"/>
-        <v>0.10634418493764766</v>
+        <v>0.16926582657072059</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>20</v>
@@ -796,8 +796,8 @@
         <v>0</v>
       </c>
       <c r="L5" s="2">
-        <f>H5 + 6*(J5-H5)</f>
-        <v>0.9715851926871889</v>
+        <f t="shared" si="3"/>
+        <v>1.5526419878119815</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>21</v>
@@ -847,8 +847,8 @@
         <v>0</v>
       </c>
       <c r="L6" s="2">
-        <f>H6 + 6*(J6-H6)</f>
-        <v>0.92315721224771963</v>
+        <f t="shared" si="3"/>
+        <v>1.4719286870795329</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>21</v>
@@ -899,7 +899,7 @@
       </c>
       <c r="L7" s="2">
         <f t="shared" si="3"/>
-        <v>0.64097296559087269</v>
+        <v>1.0682882759847878</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>21</v>
@@ -950,7 +950,7 @@
       </c>
       <c r="L8" s="2">
         <f t="shared" si="3"/>
-        <v>0.9233262993750293</v>
+        <v>1.4722104989583822</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>21</v>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="L9" s="2">
         <f t="shared" si="3"/>
-        <v>1.4249336512717796</v>
+        <v>2.1748894187862988</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>21</v>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="L10" s="2">
         <f t="shared" si="3"/>
-        <v>1.9287121346740848</v>
+        <v>2.8811868911234746</v>
       </c>
       <c r="M10" s="1" t="s">
         <v>21</v>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="L11" s="2">
         <f t="shared" si="3"/>
-        <v>3.0907871181400552</v>
+        <v>4.4179785302334249</v>
       </c>
       <c r="M11" s="1" t="s">
         <v>21</v>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="L12" s="2">
         <f t="shared" si="3"/>
-        <v>4.8231632204229191</v>
+        <v>6.5719387007048651</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>21</v>
@@ -1201,11 +1201,11 @@
       </c>
       <c r="K13" s="2">
         <f t="shared" si="2"/>
-        <v>1.1596472372492075</v>
+        <v>0</v>
       </c>
       <c r="L13" s="2">
         <f t="shared" si="3"/>
-        <v>7.6503300078460965</v>
+        <v>9.8838833464101619</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>21</v>
@@ -1252,11 +1252,11 @@
       </c>
       <c r="K14" s="2">
         <f t="shared" si="2"/>
-        <v>4.9763112838153027</v>
+        <v>1.9605188063588379</v>
       </c>
       <c r="L14" s="2">
         <f t="shared" si="3"/>
-        <v>14.238489282818286</v>
+        <v>17.397482138030476</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>21</v>
@@ -1303,11 +1303,11 @@
       </c>
       <c r="K15" s="2">
         <f t="shared" si="2"/>
-        <v>12.019344905898144</v>
+        <v>7.6989081764969072</v>
       </c>
       <c r="L15" s="2">
         <f t="shared" si="3"/>
-        <v>25.228301508313052</v>
+        <v>29.71383584718842</v>
       </c>
       <c r="M15" s="1" t="s">
         <v>21</v>
@@ -1354,11 +1354,11 @@
       </c>
       <c r="K16" s="2">
         <f t="shared" si="2"/>
-        <v>25.104964725623603</v>
+        <v>18.974941209372673</v>
       </c>
       <c r="L16" s="2">
         <f t="shared" si="3"/>
-        <v>43.757654857481683</v>
+        <v>50.062758095802806</v>
       </c>
       <c r="M16" s="1" t="s">
         <v>21</v>
@@ -1405,11 +1405,11 @@
       </c>
       <c r="K17" s="2">
         <f t="shared" si="2"/>
-        <v>40.661704348130023</v>
+        <v>32.502840580216706</v>
       </c>
       <c r="L17" s="2">
         <f t="shared" si="3"/>
-        <v>65.403748958015939</v>
+        <v>73.739581596693228</v>
       </c>
       <c r="M17" s="1" t="s">
         <v>21</v>
@@ -1456,11 +1456,11 @@
       </c>
       <c r="K18" s="2">
         <f t="shared" si="2"/>
-        <v>65.940858029655502</v>
+        <v>54.701430049425838</v>
       </c>
       <c r="L18" s="2">
         <f t="shared" si="3"/>
-        <v>100.04899148704386</v>
+        <v>111.54831914507311</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>21</v>
@@ -1507,11 +1507,11 @@
       </c>
       <c r="K19" s="2">
         <f t="shared" si="2"/>
-        <v>87.214994585432123</v>
+        <v>72.624990975720209</v>
       </c>
       <c r="L19" s="2">
         <f t="shared" si="3"/>
-        <v>131.47957337956146</v>
+        <v>146.39928896593577</v>
       </c>
       <c r="M19" s="1" t="s">
         <v>21</v>
@@ -1558,11 +1558,11 @@
       </c>
       <c r="K20" s="2">
         <f t="shared" si="2"/>
-        <v>103.57095597519671</v>
+        <v>84.484926625327859</v>
       </c>
       <c r="L20" s="2">
         <f t="shared" si="3"/>
-        <v>161.44993803281119</v>
+        <v>180.94989672135199</v>
       </c>
       <c r="M20" s="1" t="s">
         <v>21</v>
@@ -1608,11 +1608,11 @@
       </c>
       <c r="K21" s="2">
         <f t="shared" si="2"/>
-        <v>110.10853292030657</v>
+        <v>83.980888200510947</v>
       </c>
       <c r="L21" s="2">
         <f t="shared" si="3"/>
-        <v>189.6402493393885</v>
+        <v>216.53374889898083</v>
       </c>
       <c r="M21" s="1" t="s">
         <v>21</v>
@@ -1651,11 +1651,11 @@
       </c>
       <c r="K22" s="2">
         <f t="shared" si="2"/>
-        <v>0.74935928701224597</v>
+        <v>0.7296338994063748</v>
       </c>
       <c r="L22" s="2">
         <f t="shared" si="3"/>
-        <v>0.80807013526328431</v>
+        <v>0.82748531315810536</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>21</v>
@@ -1694,11 +1694,11 @@
       </c>
       <c r="K23" s="2">
         <f t="shared" si="2"/>
-        <v>0.16200907015741836</v>
+        <v>0.14369932745534639</v>
       </c>
       <c r="L23" s="2">
         <f t="shared" si="3"/>
-        <v>0.21745628995095487</v>
+        <v>0.2361113604445739</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>21</v>
@@ -1737,11 +1737,11 @@
       </c>
       <c r="K24" s="2">
         <f t="shared" si="2"/>
-        <v>1.959249838925043E-2</v>
+        <v>1.1601532403136681E-2</v>
       </c>
       <c r="L24" s="2">
-        <f>H24 + 6*(J24-H24)</f>
-        <v>4.4346773638634401E-2</v>
+        <f t="shared" si="3"/>
+        <v>5.2858657818776633E-2</v>
       </c>
       <c r="M24" s="1" t="s">
         <v>21</v>
@@ -1912,7 +1912,7 @@
     <row r="9" spans="1:12">
       <c r="A9" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_90</v>
+        <v>prevalence_preclin_92</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>18</v>
@@ -1921,11 +1921,11 @@
         <v>85</v>
       </c>
       <c r="D9" s="2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="0"/>
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G9" s="1">
         <v>418</v>

</xml_diff>

<commit_message>
Change bladder preclinical cancer prevalence targets to proportion of cancers at death that are incidental
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E53BC92-F4DC-A84D-9E08-9B24C8CE92EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B02930-2B7D-8D49-B2F2-7A6CB1674C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17540" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="-3020" yWindow="-20320" windowWidth="30240" windowHeight="17540" activeTab="1" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -626,19 +626,19 @@
       </c>
       <c r="G2" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>1810</v>
+        <v>12</v>
       </c>
       <c r="H2" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>5.5248618784530391E-4</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="I2" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>9.7534036711855159E-5</v>
+        <v>1.4865094404917123E-2</v>
       </c>
       <c r="J2" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A2,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>3.1229562615372915E-3</v>
+        <v>0.35387991114111689</v>
       </c>
       <c r="K2" s="2">
         <f>IF(H2 - 10*(H2-I2) &lt; 0, 0, H2 - 10*(H2-I2))</f>
@@ -646,7 +646,7 @@
       </c>
       <c r="L2" s="2">
         <f>H2 + 10*(J2-H2)</f>
-        <v>2.6257186924765179E-2</v>
+        <v>2.7887991114111692</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>20</v>
@@ -676,19 +676,19 @@
       </c>
       <c r="G3" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>1307</v>
+        <v>16</v>
       </c>
       <c r="H3" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>1.530221882172915E-3</v>
+        <v>0.125</v>
       </c>
       <c r="I3" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>4.1974238437163421E-4</v>
+        <v>3.4977487743240443E-2</v>
       </c>
       <c r="J3" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A3,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>5.562261593248006E-3</v>
+        <v>0.36022827265758689</v>
       </c>
       <c r="K3" s="2">
         <f t="shared" ref="K3:K24" si="2">IF(H3 - 10*(H3-I3) &lt; 0, 0, H3 - 10*(H3-I3))</f>
@@ -696,7 +696,7 @@
       </c>
       <c r="L3" s="2">
         <f t="shared" ref="L3:L24" si="3">H3 + 10*(J3-H3)</f>
-        <v>4.1850618992923819E-2</v>
+        <v>2.477282726575869</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>20</v>
@@ -722,23 +722,23 @@
       </c>
       <c r="F4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>418</v>
+        <v>8</v>
       </c>
       <c r="H4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>1.1961722488038277E-2</v>
+        <v>0.25</v>
       </c>
       <c r="I4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>5.1198596930172122E-3</v>
+        <v>7.1479212752109056E-2</v>
       </c>
       <c r="J4" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A4,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>2.7692132896306509E-2</v>
+        <v>0.59072456968983111</v>
       </c>
       <c r="K4" s="2">
         <f t="shared" si="2"/>
@@ -746,7 +746,7 @@
       </c>
       <c r="L4" s="2">
         <f t="shared" si="3"/>
-        <v>0.16926582657072059</v>
+        <v>3.6572456968983111</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>20</v>
@@ -1846,26 +1846,26 @@
         <v>71</v>
       </c>
       <c r="G7" s="1">
-        <v>1810</v>
+        <v>12</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="I7" s="1">
         <f>H7/G7</f>
-        <v>5.5248618784530391E-4</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="J7" s="1">
         <f t="shared" ref="J7:J9" si="1">$B$4^2/G7</f>
-        <v>2.1223529396100132E-3</v>
+        <v>0.32012156839117695</v>
       </c>
       <c r="K7" s="1">
         <f t="shared" ref="K7:K9" si="2">(I7+J7/2)/(J7+1)-$B$4/(J7+1)*SQRT(I7*(1-I7)/G7+J7/(4*G7))</f>
-        <v>9.7534036711855159E-5</v>
+        <v>1.4865094404917123E-2</v>
       </c>
       <c r="L7" s="1">
         <f t="shared" ref="L7:L9" si="3">(I7+J7/2)/(J7+1)+$B$4/(J7+1)*SQRT(I7*(1-I7)/G7+J7/(4*G7))</f>
-        <v>3.1229562615372915E-3</v>
+        <v>0.35387991114111689</v>
       </c>
     </row>
     <row r="8" spans="1:12">
@@ -1887,26 +1887,26 @@
         <v>80</v>
       </c>
       <c r="G8" s="1">
-        <v>1307</v>
+        <v>16</v>
       </c>
       <c r="H8" s="1">
         <v>2</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" ref="I8:I9" si="5">H8/G8</f>
-        <v>1.530221882172915E-3</v>
+        <v>0.125</v>
       </c>
       <c r="J8" s="1">
         <f t="shared" si="1"/>
-        <v>2.9391421734461542E-3</v>
+        <v>0.24009117629338272</v>
       </c>
       <c r="K8" s="1">
         <f t="shared" si="2"/>
-        <v>4.1974238437163421E-4</v>
+        <v>3.4977487743240443E-2</v>
       </c>
       <c r="L8" s="1">
         <f t="shared" si="3"/>
-        <v>5.562261593248006E-3</v>
+        <v>0.36022827265758689</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -1928,26 +1928,26 @@
         <v>92</v>
       </c>
       <c r="G9" s="1">
-        <v>418</v>
+        <v>8</v>
       </c>
       <c r="H9" s="1">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="5"/>
-        <v>1.1961722488038277E-2</v>
+        <v>0.25</v>
       </c>
       <c r="J9" s="1">
         <f t="shared" si="1"/>
-        <v>9.1900928724739806E-3</v>
+        <v>0.48018235258676545</v>
       </c>
       <c r="K9" s="1">
         <f t="shared" si="2"/>
-        <v>5.1198596930172122E-3</v>
+        <v>7.1479212752109056E-2</v>
       </c>
       <c r="L9" s="1">
         <f t="shared" si="3"/>
-        <v>2.7692132896306509E-2</v>
+        <v>0.59072456968983111</v>
       </c>
     </row>
     <row r="10" spans="1:12">

</xml_diff>

<commit_message>
Incorporate Weibull cure model for bladder calibration
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14B02930-2B7D-8D49-B2F2-7A6CB1674C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFE6EA9-58CF-5B4E-AE1B-148794989AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3020" yWindow="-20320" windowWidth="30240" windowHeight="17540" activeTab="1" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="39">
   <si>
     <t>target_names</t>
   </si>
@@ -553,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:M24"/>
+  <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -604,7 +604,7 @@
     </row>
     <row r="2" spans="1:13">
       <c r="A2" s="1" t="str">
-        <f t="shared" ref="A2:A24" si="0">""&amp;B2&amp;"_"&amp;E2</f>
+        <f t="shared" ref="A2:A25" si="0">""&amp;B2&amp;"_"&amp;E2</f>
         <v>prevalence_preclin_71</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -691,11 +691,11 @@
         <v>0.36022827265758689</v>
       </c>
       <c r="K3" s="2">
-        <f t="shared" ref="K3:K24" si="2">IF(H3 - 10*(H3-I3) &lt; 0, 0, H3 - 10*(H3-I3))</f>
+        <f t="shared" ref="K3:K25" si="2">IF(H3 - 10*(H3-I3) &lt; 0, 0, H3 - 10*(H3-I3))</f>
         <v>0</v>
       </c>
       <c r="L3" s="2">
-        <f t="shared" ref="L3:L24" si="3">H3 + 10*(J3-H3)</f>
+        <f t="shared" ref="L3:L25" si="3">H3 + 10*(J3-H3)</f>
         <v>2.477282726575869</v>
       </c>
       <c r="M3" s="1" t="s">
@@ -1620,42 +1620,49 @@
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>stage_distr_1</v>
+        <f t="shared" ref="A22" si="8">""&amp;B22&amp;"_"&amp;E22</f>
+        <v>incidence_clin_92</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>8</v>
+        <v>19</v>
+      </c>
+      <c r="C22" s="1">
+        <v>85</v>
+      </c>
+      <c r="D22" s="1">
+        <v>100</v>
       </c>
       <c r="E22" s="1">
-        <v>1</v>
+        <f t="shared" ref="E22" si="9">FLOOR(AVERAGE(C22,D22), 1)</f>
+        <v>92</v>
       </c>
       <c r="F22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>21522.9</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(F$1,bounds!$23:$23,0))</f>
+        <v>1258.9121706180499</v>
       </c>
       <c r="G22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
-        <v>27630.75</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(G$1,bounds!$23:$23,0))</f>
+        <v>888434.84165000007</v>
       </c>
       <c r="H22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.77894736842105272</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(H$1,bounds!$23:$23,0))</f>
+        <v>141.69999999999999</v>
       </c>
       <c r="I22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>0.77401602151958493</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(I$1,bounds!$23:$23,0))</f>
+        <v>133.87986472565848</v>
       </c>
       <c r="J22" s="2">
-        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A22,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>0.78380116289475799</v>
+        <f>INDEX(bounds!$23:$41,MATCH(targets!$A22,bounds!$A$23:$A$41,0), MATCH(J$1,bounds!$23:$23,0))</f>
+        <v>149.75933097441057</v>
       </c>
       <c r="K22" s="2">
-        <f t="shared" si="2"/>
-        <v>0.7296338994063748</v>
+        <f t="shared" ref="K22" si="10">IF(H22 - 10*(H22-I22) &lt; 0, 0, H22 - 10*(H22-I22))</f>
+        <v>63.498647256584889</v>
       </c>
       <c r="L22" s="2">
-        <f t="shared" si="3"/>
-        <v>0.82748531315810536</v>
+        <f t="shared" ref="L22" si="11">H22 + 10*(J22-H22)</f>
+        <v>222.29330974410584</v>
       </c>
       <c r="M22" s="1" t="s">
         <v>21</v>
@@ -1664,17 +1671,17 @@
     <row r="23" spans="1:13">
       <c r="A23" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>stage_distr_2</v>
+        <v>stage_distr_1</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E23" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>5235.3</v>
+        <v>21522.9</v>
       </c>
       <c r="G23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
@@ -1682,23 +1689,23 @@
       </c>
       <c r="H23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>0.18947368421052632</v>
+        <v>0.77894736842105272</v>
       </c>
       <c r="I23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>0.18489624853500833</v>
+        <v>0.77401602151958493</v>
       </c>
       <c r="J23" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A23,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>0.19413745183393108</v>
+        <v>0.78380116289475799</v>
       </c>
       <c r="K23" s="2">
         <f t="shared" si="2"/>
-        <v>0.14369932745534639</v>
+        <v>0.7296338994063748</v>
       </c>
       <c r="L23" s="2">
         <f t="shared" si="3"/>
-        <v>0.2361113604445739</v>
+        <v>0.82748531315810536</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>21</v>
@@ -1707,17 +1714,17 @@
     <row r="24" spans="1:13">
       <c r="A24" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>stage_distr_3</v>
+        <v>stage_distr_2</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>8</v>
       </c>
       <c r="E24" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
-        <v>872.55</v>
+        <v>5235.3</v>
       </c>
       <c r="G24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
@@ -1725,25 +1732,68 @@
       </c>
       <c r="H24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
-        <v>3.1578947368421054E-2</v>
+        <v>0.18947368421052632</v>
       </c>
       <c r="I24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
-        <v>2.9581205871892616E-2</v>
+        <v>0.18489624853500833</v>
       </c>
       <c r="J24" s="2">
         <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A24,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
-        <v>3.3706918413456612E-2</v>
+        <v>0.19413745183393108</v>
       </c>
       <c r="K24" s="2">
         <f t="shared" si="2"/>
-        <v>1.1601532403136681E-2</v>
+        <v>0.14369932745534639</v>
       </c>
       <c r="L24" s="2">
         <f t="shared" si="3"/>
+        <v>0.2361113604445739</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13">
+      <c r="A25" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>stage_distr_3</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E25" s="1">
+        <v>3</v>
+      </c>
+      <c r="F25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(F$1,bounds!$6:$6,0))</f>
+        <v>872.55</v>
+      </c>
+      <c r="G25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(G$1,bounds!$6:$6,0))</f>
+        <v>27630.75</v>
+      </c>
+      <c r="H25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(H$1,bounds!$6:$6,0))</f>
+        <v>3.1578947368421054E-2</v>
+      </c>
+      <c r="I25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(I$1,bounds!$6:$6,0))</f>
+        <v>2.9581205871892616E-2</v>
+      </c>
+      <c r="J25" s="2">
+        <f>INDEX(bounds!$A$6:$L$1048576,MATCH(targets!$A25,bounds!$A$6:$A$1048576,0), MATCH(J$1,bounds!$6:$6,0))</f>
+        <v>3.3706918413456612E-2</v>
+      </c>
+      <c r="K25" s="2">
+        <f t="shared" si="2"/>
+        <v>1.1601532403136681E-2</v>
+      </c>
+      <c r="L25" s="2">
+        <f t="shared" si="3"/>
         <v>5.2858657818776633E-2</v>
       </c>
-      <c r="M24" s="1" t="s">
+      <c r="M25" s="1" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Increase target bounds for bladder
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DFE6EA9-58CF-5B4E-AE1B-148794989AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185535EB-1CEB-024C-923F-A6C399C86CFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="-540" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -645,8 +645,8 @@
         <v>0</v>
       </c>
       <c r="L2" s="2">
-        <f>H2 + 10*(J2-H2)</f>
-        <v>2.7887991114111692</v>
+        <f>H2 + 3*(J2-H2)</f>
+        <v>0.89497306675668409</v>
       </c>
       <c r="M2" s="1" t="s">
         <v>20</v>
@@ -691,12 +691,12 @@
         <v>0.36022827265758689</v>
       </c>
       <c r="K3" s="2">
-        <f t="shared" ref="K3:K25" si="2">IF(H3 - 10*(H3-I3) &lt; 0, 0, H3 - 10*(H3-I3))</f>
+        <f t="shared" ref="K3:K21" si="2">IF(H3 - 10*(H3-I3) &lt; 0, 0, H3 - 10*(H3-I3))</f>
         <v>0</v>
       </c>
       <c r="L3" s="2">
-        <f t="shared" ref="L3:L25" si="3">H3 + 10*(J3-H3)</f>
-        <v>2.477282726575869</v>
+        <f t="shared" ref="L3:L4" si="3">H3 + 3*(J3-H3)</f>
+        <v>0.83068481797276061</v>
       </c>
       <c r="M3" s="1" t="s">
         <v>20</v>
@@ -746,7 +746,7 @@
       </c>
       <c r="L4" s="2">
         <f t="shared" si="3"/>
-        <v>3.6572456968983111</v>
+        <v>1.2721737090694933</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>20</v>
@@ -796,8 +796,8 @@
         <v>0</v>
       </c>
       <c r="L5" s="2">
-        <f t="shared" si="3"/>
-        <v>1.5526419878119815</v>
+        <f>H5 + 20*(J5-H5)</f>
+        <v>3.0052839756239629</v>
       </c>
       <c r="M5" s="1" t="s">
         <v>21</v>
@@ -847,8 +847,8 @@
         <v>0</v>
       </c>
       <c r="L6" s="2">
-        <f t="shared" si="3"/>
-        <v>1.4719286870795329</v>
+        <f t="shared" ref="L6:L13" si="6">H6 + 20*(J6-H6)</f>
+        <v>2.8438573741590658</v>
       </c>
       <c r="M6" s="1" t="s">
         <v>21</v>
@@ -866,7 +866,7 @@
         <v>10</v>
       </c>
       <c r="D7" s="1">
-        <f t="shared" ref="D7:D20" si="6">C8</f>
+        <f t="shared" ref="D7:D20" si="7">C8</f>
         <v>15</v>
       </c>
       <c r="E7" s="1">
@@ -898,8 +898,8 @@
         <v>0</v>
       </c>
       <c r="L7" s="2">
-        <f t="shared" si="3"/>
-        <v>1.0682882759847878</v>
+        <f t="shared" si="6"/>
+        <v>2.1365765519695756</v>
       </c>
       <c r="M7" s="1" t="s">
         <v>21</v>
@@ -917,7 +917,7 @@
         <v>15</v>
       </c>
       <c r="D8" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>20</v>
       </c>
       <c r="E8" s="1">
@@ -949,8 +949,8 @@
         <v>0</v>
       </c>
       <c r="L8" s="2">
-        <f t="shared" si="3"/>
-        <v>1.4722104989583822</v>
+        <f t="shared" si="6"/>
+        <v>2.8444209979167643</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>21</v>
@@ -968,7 +968,7 @@
         <v>20</v>
       </c>
       <c r="D9" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>25</v>
       </c>
       <c r="E9" s="1">
@@ -1000,8 +1000,8 @@
         <v>0</v>
       </c>
       <c r="L9" s="2">
-        <f t="shared" si="3"/>
-        <v>2.1748894187862988</v>
+        <f t="shared" si="6"/>
+        <v>4.0497788375725978</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>21</v>
@@ -1019,7 +1019,7 @@
         <v>25</v>
       </c>
       <c r="D10" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>30</v>
       </c>
       <c r="E10" s="1">
@@ -1051,8 +1051,8 @@
         <v>0</v>
       </c>
       <c r="L10" s="2">
-        <f t="shared" si="3"/>
-        <v>2.8811868911234746</v>
+        <f t="shared" si="6"/>
+        <v>5.2623737822469492</v>
       </c>
       <c r="M10" s="1" t="s">
         <v>21</v>
@@ -1060,7 +1060,7 @@
     </row>
     <row r="11" spans="1:13">
       <c r="A11" s="1" t="str">
-        <f t="shared" ref="A11:A21" si="7">""&amp;B11&amp;"_"&amp;E11</f>
+        <f t="shared" ref="A11:A21" si="8">""&amp;B11&amp;"_"&amp;E11</f>
         <v>incidence_clin_32</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1070,7 +1070,7 @@
         <v>30</v>
       </c>
       <c r="D11" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>35</v>
       </c>
       <c r="E11" s="1">
@@ -1102,8 +1102,8 @@
         <v>0</v>
       </c>
       <c r="L11" s="2">
-        <f t="shared" si="3"/>
-        <v>4.4179785302334249</v>
+        <f t="shared" si="6"/>
+        <v>7.7359570604668502</v>
       </c>
       <c r="M11" s="1" t="s">
         <v>21</v>
@@ -1111,7 +1111,7 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_37</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1121,7 +1121,7 @@
         <v>35</v>
       </c>
       <c r="D12" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>40</v>
       </c>
       <c r="E12" s="1">
@@ -1153,8 +1153,8 @@
         <v>0</v>
       </c>
       <c r="L12" s="2">
-        <f t="shared" si="3"/>
-        <v>6.5719387007048651</v>
+        <f t="shared" si="6"/>
+        <v>10.943877401409729</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>21</v>
@@ -1162,7 +1162,7 @@
     </row>
     <row r="13" spans="1:13">
       <c r="A13" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_42</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -1172,7 +1172,7 @@
         <v>40</v>
       </c>
       <c r="D13" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>45</v>
       </c>
       <c r="E13" s="1">
@@ -1204,8 +1204,8 @@
         <v>0</v>
       </c>
       <c r="L13" s="2">
-        <f t="shared" si="3"/>
-        <v>9.8838833464101619</v>
+        <f t="shared" si="6"/>
+        <v>15.467766692820323</v>
       </c>
       <c r="M13" s="1" t="s">
         <v>21</v>
@@ -1213,7 +1213,7 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_47</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1223,7 +1223,7 @@
         <v>45</v>
       </c>
       <c r="D14" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>50</v>
       </c>
       <c r="E14" s="1">
@@ -1255,7 +1255,7 @@
         <v>1.9605188063588379</v>
       </c>
       <c r="L14" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="L14:L21" si="9">H14 + 10*(J14-H14)</f>
         <v>17.397482138030476</v>
       </c>
       <c r="M14" s="1" t="s">
@@ -1264,7 +1264,7 @@
     </row>
     <row r="15" spans="1:13">
       <c r="A15" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_52</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1274,7 +1274,7 @@
         <v>50</v>
       </c>
       <c r="D15" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>55</v>
       </c>
       <c r="E15" s="1">
@@ -1306,7 +1306,7 @@
         <v>7.6989081764969072</v>
       </c>
       <c r="L15" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>29.71383584718842</v>
       </c>
       <c r="M15" s="1" t="s">
@@ -1315,7 +1315,7 @@
     </row>
     <row r="16" spans="1:13">
       <c r="A16" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_57</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1325,7 +1325,7 @@
         <v>55</v>
       </c>
       <c r="D16" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>60</v>
       </c>
       <c r="E16" s="1">
@@ -1357,7 +1357,7 @@
         <v>18.974941209372673</v>
       </c>
       <c r="L16" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>50.062758095802806</v>
       </c>
       <c r="M16" s="1" t="s">
@@ -1366,7 +1366,7 @@
     </row>
     <row r="17" spans="1:13">
       <c r="A17" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_62</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1376,7 +1376,7 @@
         <v>60</v>
       </c>
       <c r="D17" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>65</v>
       </c>
       <c r="E17" s="1">
@@ -1408,7 +1408,7 @@
         <v>32.502840580216706</v>
       </c>
       <c r="L17" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>73.739581596693228</v>
       </c>
       <c r="M17" s="1" t="s">
@@ -1417,7 +1417,7 @@
     </row>
     <row r="18" spans="1:13">
       <c r="A18" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_67</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1427,7 +1427,7 @@
         <v>65</v>
       </c>
       <c r="D18" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>70</v>
       </c>
       <c r="E18" s="1">
@@ -1459,7 +1459,7 @@
         <v>54.701430049425838</v>
       </c>
       <c r="L18" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>111.54831914507311</v>
       </c>
       <c r="M18" s="1" t="s">
@@ -1468,7 +1468,7 @@
     </row>
     <row r="19" spans="1:13">
       <c r="A19" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_72</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1478,7 +1478,7 @@
         <v>70</v>
       </c>
       <c r="D19" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>75</v>
       </c>
       <c r="E19" s="1">
@@ -1510,7 +1510,7 @@
         <v>72.624990975720209</v>
       </c>
       <c r="L19" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>146.39928896593577</v>
       </c>
       <c r="M19" s="1" t="s">
@@ -1519,7 +1519,7 @@
     </row>
     <row r="20" spans="1:13">
       <c r="A20" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_77</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1529,7 +1529,7 @@
         <v>75</v>
       </c>
       <c r="D20" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>80</v>
       </c>
       <c r="E20" s="1">
@@ -1561,7 +1561,7 @@
         <v>84.484926625327859</v>
       </c>
       <c r="L20" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>180.94989672135199</v>
       </c>
       <c r="M20" s="1" t="s">
@@ -1570,7 +1570,7 @@
     </row>
     <row r="21" spans="1:13">
       <c r="A21" s="1" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>incidence_clin_82</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1611,7 +1611,7 @@
         <v>83.980888200510947</v>
       </c>
       <c r="L21" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="9"/>
         <v>216.53374889898083</v>
       </c>
       <c r="M21" s="1" t="s">
@@ -1620,7 +1620,7 @@
     </row>
     <row r="22" spans="1:13">
       <c r="A22" s="1" t="str">
-        <f t="shared" ref="A22" si="8">""&amp;B22&amp;"_"&amp;E22</f>
+        <f t="shared" ref="A22" si="10">""&amp;B22&amp;"_"&amp;E22</f>
         <v>incidence_clin_92</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1633,7 +1633,7 @@
         <v>100</v>
       </c>
       <c r="E22" s="1">
-        <f t="shared" ref="E22" si="9">FLOOR(AVERAGE(C22,D22), 1)</f>
+        <f t="shared" ref="E22" si="11">FLOOR(AVERAGE(C22,D22), 1)</f>
         <v>92</v>
       </c>
       <c r="F22" s="2">
@@ -1657,11 +1657,11 @@
         <v>149.75933097441057</v>
       </c>
       <c r="K22" s="2">
-        <f t="shared" ref="K22" si="10">IF(H22 - 10*(H22-I22) &lt; 0, 0, H22 - 10*(H22-I22))</f>
+        <f t="shared" ref="K22" si="12">IF(H22 - 10*(H22-I22) &lt; 0, 0, H22 - 10*(H22-I22))</f>
         <v>63.498647256584889</v>
       </c>
       <c r="L22" s="2">
-        <f t="shared" ref="L22" si="11">H22 + 10*(J22-H22)</f>
+        <f t="shared" ref="L22" si="13">H22 + 10*(J22-H22)</f>
         <v>222.29330974410584</v>
       </c>
       <c r="M22" s="1" t="s">
@@ -1700,12 +1700,12 @@
         <v>0.78380116289475799</v>
       </c>
       <c r="K23" s="2">
-        <f t="shared" si="2"/>
-        <v>0.7296338994063748</v>
+        <f>IF(H23 - 20*(H23-I23) &lt; 0, 0, H23 - 20*(H23-I23))</f>
+        <v>0.68032043039169687</v>
       </c>
       <c r="L23" s="2">
-        <f t="shared" si="3"/>
-        <v>0.82748531315810536</v>
+        <f t="shared" ref="L23:L24" si="14">H23 + 20*(J23-H23)</f>
+        <v>0.876023257895158</v>
       </c>
       <c r="M23" s="1" t="s">
         <v>21</v>
@@ -1743,12 +1743,12 @@
         <v>0.19413745183393108</v>
       </c>
       <c r="K24" s="2">
-        <f t="shared" si="2"/>
-        <v>0.14369932745534639</v>
+        <f t="shared" ref="K24:K25" si="15">IF(H24 - 20*(H24-I24) &lt; 0, 0, H24 - 20*(H24-I24))</f>
+        <v>9.7924970700166453E-2</v>
       </c>
       <c r="L24" s="2">
-        <f t="shared" si="3"/>
-        <v>0.2361113604445739</v>
+        <f t="shared" si="14"/>
+        <v>0.2827490366786215</v>
       </c>
       <c r="M24" s="1" t="s">
         <v>21</v>
@@ -1786,12 +1786,12 @@
         <v>3.3706918413456612E-2</v>
       </c>
       <c r="K25" s="2">
-        <f t="shared" si="2"/>
-        <v>1.1601532403136681E-2</v>
+        <f t="shared" si="15"/>
+        <v>0</v>
       </c>
       <c r="L25" s="2">
-        <f t="shared" si="3"/>
-        <v>5.2858657818776633E-2</v>
+        <f>H25 + 20*(J25-H25)</f>
+        <v>7.4138368269132213E-2</v>
       </c>
       <c r="M25" s="1" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Try negative starting bounds for IMABC to account for strictly greater than zero condition
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{185535EB-1CEB-024C-923F-A6C399C86CFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85D0E0BF-1CF0-4940-A01E-672B679797E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-540" yWindow="760" windowWidth="30240" windowHeight="17760" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -641,8 +641,8 @@
         <v>0.35387991114111689</v>
       </c>
       <c r="K2" s="2">
-        <f>IF(H2 - 10*(H2-I2) &lt; 0, 0, H2 - 10*(H2-I2))</f>
-        <v>0</v>
+        <f>IF(H2 - 10*(H2-I2) &lt;= 0, -0.001, H2 - 10*(H2-I2))</f>
+        <v>-1E-3</v>
       </c>
       <c r="L2" s="2">
         <f>H2 + 3*(J2-H2)</f>
@@ -691,8 +691,8 @@
         <v>0.36022827265758689</v>
       </c>
       <c r="K3" s="2">
-        <f t="shared" ref="K3:K21" si="2">IF(H3 - 10*(H3-I3) &lt; 0, 0, H3 - 10*(H3-I3))</f>
-        <v>0</v>
+        <f t="shared" ref="K3:K22" si="2">IF(H3 - 10*(H3-I3) &lt;= 0, -0.001, H3 - 10*(H3-I3))</f>
+        <v>-1E-3</v>
       </c>
       <c r="L3" s="2">
         <f t="shared" ref="L3:L4" si="3">H3 + 3*(J3-H3)</f>
@@ -742,7 +742,7 @@
       </c>
       <c r="K4" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L4" s="2">
         <f t="shared" si="3"/>
@@ -793,7 +793,7 @@
       </c>
       <c r="K5" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L5" s="2">
         <f>H5 + 20*(J5-H5)</f>
@@ -844,7 +844,7 @@
       </c>
       <c r="K6" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L6" s="2">
         <f t="shared" ref="L6:L13" si="6">H6 + 20*(J6-H6)</f>
@@ -895,7 +895,7 @@
       </c>
       <c r="K7" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L7" s="2">
         <f t="shared" si="6"/>
@@ -946,7 +946,7 @@
       </c>
       <c r="K8" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L8" s="2">
         <f t="shared" si="6"/>
@@ -997,7 +997,7 @@
       </c>
       <c r="K9" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L9" s="2">
         <f t="shared" si="6"/>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="K10" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L10" s="2">
         <f t="shared" si="6"/>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="K11" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L11" s="2">
         <f t="shared" si="6"/>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="K12" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L12" s="2">
         <f t="shared" si="6"/>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="K13" s="2">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>-1E-3</v>
       </c>
       <c r="L13" s="2">
         <f t="shared" si="6"/>
@@ -1657,11 +1657,11 @@
         <v>149.75933097441057</v>
       </c>
       <c r="K22" s="2">
-        <f t="shared" ref="K22" si="12">IF(H22 - 10*(H22-I22) &lt; 0, 0, H22 - 10*(H22-I22))</f>
+        <f t="shared" si="2"/>
         <v>63.498647256584889</v>
       </c>
       <c r="L22" s="2">
-        <f t="shared" ref="L22" si="13">H22 + 10*(J22-H22)</f>
+        <f t="shared" ref="L22" si="12">H22 + 10*(J22-H22)</f>
         <v>222.29330974410584</v>
       </c>
       <c r="M22" s="1" t="s">
@@ -1700,11 +1700,11 @@
         <v>0.78380116289475799</v>
       </c>
       <c r="K23" s="2">
-        <f>IF(H23 - 20*(H23-I23) &lt; 0, 0, H23 - 20*(H23-I23))</f>
+        <f>IF(H23 - 20*(H23-I23) &lt;= 0, -0.001, H23 - 20*(H23-I23))</f>
         <v>0.68032043039169687</v>
       </c>
       <c r="L23" s="2">
-        <f t="shared" ref="L23:L24" si="14">H23 + 20*(J23-H23)</f>
+        <f t="shared" ref="L23:L24" si="13">H23 + 20*(J23-H23)</f>
         <v>0.876023257895158</v>
       </c>
       <c r="M23" s="1" t="s">
@@ -1743,11 +1743,11 @@
         <v>0.19413745183393108</v>
       </c>
       <c r="K24" s="2">
-        <f t="shared" ref="K24:K25" si="15">IF(H24 - 20*(H24-I24) &lt; 0, 0, H24 - 20*(H24-I24))</f>
+        <f t="shared" ref="K24:K25" si="14">IF(H24 - 20*(H24-I24) &lt;= 0, -0.001, H24 - 20*(H24-I24))</f>
         <v>9.7924970700166453E-2</v>
       </c>
       <c r="L24" s="2">
-        <f t="shared" si="14"/>
+        <f t="shared" si="13"/>
         <v>0.2827490366786215</v>
       </c>
       <c r="M24" s="1" t="s">
@@ -1786,8 +1786,8 @@
         <v>3.3706918413456612E-2</v>
       </c>
       <c r="K25" s="2">
-        <f t="shared" si="15"/>
-        <v>0</v>
+        <f t="shared" si="14"/>
+        <v>-1E-3</v>
       </c>
       <c r="L25" s="2">
         <f>H25 + 20*(J25-H25)</f>

</xml_diff>

<commit_message>
Consolidate bladder cancer data and rerun with larger IMABC parameters
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder_incidental/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF389104-3CDA-2A4E-A376-E164B702D37B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344F28A2-5AF7-E94E-B86F-FAE3D5F1DCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2740" yWindow="1020" windowWidth="21160" windowHeight="17740" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="2740" yWindow="1020" windowWidth="21160" windowHeight="17740" activeTab="1" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="42">
   <si>
     <t>target_names</t>
   </si>
@@ -97,9 +97,6 @@
   </si>
   <si>
     <t>incidence_clin</t>
-  </si>
-  <si>
-    <t>Suen et al. 1970</t>
   </si>
   <si>
     <t>SEER Cancer Statistics Review 1973-1994</t>
@@ -576,7 +573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -616,13 +613,13 @@
         <v>10</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="L1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="N1" s="2" t="s">
         <v>6</v>
@@ -630,52 +627,53 @@
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="1" t="str">
-        <f t="shared" ref="A2:A25" si="0">""&amp;B2&amp;"_"&amp;E2</f>
-        <v>prevalence_preclin_71</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="2">
-        <v>66</v>
-      </c>
-      <c r="D2" s="2">
-        <v>76</v>
+        <f t="shared" ref="A2:A7" si="0">""&amp;B2&amp;"_"&amp;E2</f>
+        <v>incidence_clin_2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <f t="shared" ref="D2" si="1">C3</f>
+        <v>5</v>
       </c>
       <c r="E2" s="1">
-        <f t="shared" ref="E2:E21" si="1">FLOOR(AVERAGE(C2,D2), 1)</f>
-        <v>71</v>
+        <f t="shared" ref="E2:E18" si="2">FLOOR(AVERAGE(C2,D2), 1)</f>
+        <v>2</v>
       </c>
       <c r="F2" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A2,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
-        <v>1</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A2,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
+        <v>10.087170893440002</v>
       </c>
       <c r="G2" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A2,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
-        <v>12</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A2,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
+        <v>10087170.893440001</v>
       </c>
       <c r="H2" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A2,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
-        <v>8.3333333333333329E-2</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A2,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
+        <v>0.1</v>
       </c>
       <c r="I2" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A2,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
-        <v>1.4865094404917123E-2</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A2,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
+        <v>-1E-3</v>
       </c>
       <c r="J2" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A2,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
-        <v>0.35387991114111689</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A2,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
+        <v>0.36127483158541895</v>
       </c>
       <c r="K2" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2" s="2">
-        <f>IF(H2 - K2*(H2-I2) &lt;= 0, -0.001, H2 - K2*(H2-I2))</f>
+        <f t="shared" ref="L2:L22" si="3">IF(H2 - K2*(H2-I2) &lt;= 0, -0.001, H2 - K2*(H2-I2))</f>
         <v>-1E-3</v>
       </c>
       <c r="M2" s="2">
-        <f>H2 + K2*(J2-H2)</f>
-        <v>0.62442648894890052</v>
+        <f t="shared" ref="M2:M22" si="4">H2 + K2*(J2-H2)</f>
+        <v>0.88382449475625691</v>
       </c>
       <c r="N2" s="1" t="s">
         <v>20</v>
@@ -684,51 +682,52 @@
     <row r="3" spans="1:14">
       <c r="A3" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>prevalence_preclin_80</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="2">
-        <v>76</v>
-      </c>
-      <c r="D3" s="2">
-        <v>85</v>
+        <v>incidence_clin_7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1">
+        <v>5</v>
+      </c>
+      <c r="D3" s="1">
+        <f>C4</f>
+        <v>10</v>
       </c>
       <c r="E3" s="1">
-        <f t="shared" si="1"/>
-        <v>80</v>
+        <f t="shared" si="2"/>
+        <v>7</v>
       </c>
       <c r="F3" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A3,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
-        <v>2</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A3,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
+        <v>11.734748512359999</v>
       </c>
       <c r="G3" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A3,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
-        <v>16</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A3,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
+        <v>11734748.512359999</v>
       </c>
       <c r="H3" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A3,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
-        <v>0.125</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A3,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
+        <v>0.1</v>
       </c>
       <c r="I3" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A3,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
-        <v>3.4977487743240443E-2</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A3,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
+        <v>-1E-3</v>
       </c>
       <c r="J3" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A3,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
-        <v>0.36022827265758689</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A3,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
+        <v>0.34176539057413913</v>
       </c>
       <c r="K3" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L3" s="2">
-        <f t="shared" ref="L3:L25" si="2">IF(H3 - K3*(H3-I3) &lt;= 0, -0.001, H3 - K3*(H3-I3))</f>
+        <f t="shared" si="3"/>
         <v>-1E-3</v>
       </c>
       <c r="M3" s="2">
-        <f t="shared" ref="M3:M25" si="3">H3 + K3*(J3-H3)</f>
-        <v>0.59545654531517378</v>
+        <f t="shared" si="4"/>
+        <v>0.82529617172241732</v>
       </c>
       <c r="N3" s="1" t="s">
         <v>20</v>
@@ -737,51 +736,52 @@
     <row r="4" spans="1:14">
       <c r="A4" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>prevalence_preclin_92</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="2">
-        <v>85</v>
-      </c>
-      <c r="D4" s="2">
-        <v>100</v>
+        <v>incidence_clin_12</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1">
+        <v>10</v>
+      </c>
+      <c r="D4" s="1">
+        <f t="shared" ref="D4:D17" si="5">C5</f>
+        <v>15</v>
       </c>
       <c r="E4" s="1">
-        <f t="shared" si="1"/>
-        <v>92</v>
+        <f t="shared" si="2"/>
+        <v>12</v>
       </c>
       <c r="F4" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A4,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
-        <v>2</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A4,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
+        <v>0</v>
       </c>
       <c r="G4" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A4,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
-        <v>8</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A4,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
+        <v>12224672.231360001</v>
       </c>
       <c r="H4" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A4,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
-        <v>0.25</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A4,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
+        <v>0</v>
       </c>
       <c r="I4" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A4,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
-        <v>7.1479212752109056E-2</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A4,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
+        <v>-1E-3</v>
       </c>
       <c r="J4" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A4,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
-        <v>0.59072456968983111</v>
+        <f>INDEX(bounds!$24:$42,MATCH(targets!$A4,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
+        <v>0.18182240036888692</v>
       </c>
       <c r="K4" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L4" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1E-3</v>
       </c>
       <c r="M4" s="2">
-        <f t="shared" si="3"/>
-        <v>0.93144913937966223</v>
+        <f t="shared" si="4"/>
+        <v>0.5454672011066608</v>
       </c>
       <c r="N4" s="1" t="s">
         <v>20</v>
@@ -789,30 +789,30 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="1" t="str">
-        <f t="shared" ref="A5:A10" si="4">""&amp;B5&amp;"_"&amp;E5</f>
-        <v>incidence_clin_2</v>
+        <f t="shared" si="0"/>
+        <v>incidence_clin_17</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C5" s="1">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D5" s="1">
-        <f t="shared" ref="D5" si="5">C6</f>
-        <v>5</v>
+        <f t="shared" si="5"/>
+        <v>20</v>
       </c>
       <c r="E5" s="1">
-        <f t="shared" si="1"/>
-        <v>2</v>
+        <f t="shared" si="2"/>
+        <v>17</v>
       </c>
       <c r="F5" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A5,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>10.087170893440002</v>
+        <v>11.213875953550001</v>
       </c>
       <c r="G5" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A5,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>10087170.893440001</v>
+        <v>11213875.95355</v>
       </c>
       <c r="H5" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A5,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
@@ -824,53 +824,53 @@
       </c>
       <c r="J5" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A5,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>0.36127483158541895</v>
+        <v>0.34466310103500203</v>
       </c>
       <c r="K5" s="2">
         <v>3</v>
       </c>
       <c r="L5" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1E-3</v>
       </c>
       <c r="M5" s="2">
-        <f t="shared" si="3"/>
-        <v>0.88382449475625691</v>
+        <f t="shared" si="4"/>
+        <v>0.83398930310500607</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:14">
       <c r="A6" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>incidence_clin_7</v>
+        <f t="shared" si="0"/>
+        <v>incidence_clin_22</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C6" s="1">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="D6" s="1">
-        <f>C7</f>
-        <v>10</v>
+        <f t="shared" si="5"/>
+        <v>25</v>
       </c>
       <c r="E6" s="1">
-        <f t="shared" si="1"/>
-        <v>7</v>
+        <f t="shared" si="2"/>
+        <v>22</v>
       </c>
       <c r="F6" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A6,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>11.734748512359999</v>
+        <v>28.879569311969998</v>
       </c>
       <c r="G6" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A6,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>11734748.512359999</v>
+        <v>9626523.1039899997</v>
       </c>
       <c r="H6" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A6,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>0.1</v>
+        <v>0.3</v>
       </c>
       <c r="I6" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A6,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
@@ -878,53 +878,53 @@
       </c>
       <c r="J6" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A6,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>0.34176539057413913</v>
+        <v>0.64601481946145045</v>
       </c>
       <c r="K6" s="2">
         <v>3</v>
       </c>
       <c r="L6" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1E-3</v>
       </c>
       <c r="M6" s="2">
-        <f t="shared" si="3"/>
-        <v>0.82529617172241732</v>
+        <f t="shared" si="4"/>
+        <v>1.3380444583843514</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:14">
       <c r="A7" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>incidence_clin_12</v>
+        <f t="shared" si="0"/>
+        <v>incidence_clin_27</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C7" s="1">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="D7" s="1">
-        <f t="shared" ref="D7:D20" si="6">C8</f>
-        <v>15</v>
+        <f t="shared" si="5"/>
+        <v>30</v>
       </c>
       <c r="E7" s="1">
-        <f t="shared" si="1"/>
-        <v>12</v>
+        <f t="shared" si="2"/>
+        <v>27</v>
       </c>
       <c r="F7" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A7,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>0</v>
+        <v>39.624074444000001</v>
       </c>
       <c r="G7" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A7,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>12224672.231360001</v>
+        <v>7924814.8888000008</v>
       </c>
       <c r="H7" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A7,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I7" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A7,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
@@ -932,53 +932,53 @@
       </c>
       <c r="J7" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A7,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>0.18182240036888692</v>
+        <v>0.94989916767749982</v>
       </c>
       <c r="K7" s="2">
         <v>3</v>
       </c>
       <c r="L7" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1E-3</v>
       </c>
       <c r="M7" s="2">
-        <f t="shared" si="3"/>
-        <v>0.5454672011066608</v>
+        <f t="shared" si="4"/>
+        <v>1.8496975030324996</v>
       </c>
       <c r="N7" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>incidence_clin_17</v>
+        <f t="shared" ref="A8:A18" si="6">""&amp;B8&amp;"_"&amp;E8</f>
+        <v>incidence_clin_32</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="1">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D8" s="1">
-        <f t="shared" si="6"/>
-        <v>20</v>
+        <f t="shared" si="5"/>
+        <v>35</v>
       </c>
       <c r="E8" s="1">
-        <f t="shared" si="1"/>
-        <v>17</v>
+        <f t="shared" si="2"/>
+        <v>32</v>
       </c>
       <c r="F8" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A8,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>11.213875953550001</v>
+        <v>73.935344383010005</v>
       </c>
       <c r="G8" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A8,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>11213875.95355</v>
+        <v>6721394.9439099999</v>
       </c>
       <c r="H8" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A8,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>0.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I8" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A8,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
@@ -986,913 +986,751 @@
       </c>
       <c r="J8" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A8,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>0.34466310103500203</v>
+        <v>1.7431061741782465</v>
       </c>
       <c r="K8" s="2">
         <v>3</v>
       </c>
       <c r="L8" s="2">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>-1E-3</v>
       </c>
       <c r="M8" s="2">
-        <f t="shared" si="3"/>
-        <v>0.83398930310500607</v>
+        <f t="shared" si="4"/>
+        <v>3.0293185225347394</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>incidence_clin_22</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_37</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C9" s="1">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="D9" s="1">
-        <f t="shared" si="6"/>
-        <v>25</v>
+        <f t="shared" si="5"/>
+        <v>40</v>
       </c>
       <c r="E9" s="1">
-        <f t="shared" si="1"/>
-        <v>22</v>
+        <f t="shared" si="2"/>
+        <v>37</v>
       </c>
       <c r="F9" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A9,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>28.879569311969998</v>
+        <v>143.68291641088004</v>
       </c>
       <c r="G9" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A9,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>9626523.1039899997</v>
+        <v>6531041.6550400006</v>
       </c>
       <c r="H9" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A9,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>0.3</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="I9" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A9,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>-1E-3</v>
+        <v>1.5096614770209527</v>
       </c>
       <c r="J9" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A9,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>0.64601481946145045</v>
+        <v>3.0550947154719745</v>
       </c>
       <c r="K9" s="2">
         <v>3</v>
       </c>
       <c r="L9" s="2">
-        <f t="shared" si="2"/>
-        <v>-1E-3</v>
+        <f t="shared" si="3"/>
+        <v>0.1289844310628574</v>
       </c>
       <c r="M9" s="2">
-        <f t="shared" si="3"/>
-        <v>1.3380444583843514</v>
+        <f t="shared" si="4"/>
+        <v>4.7652841464159232</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v>incidence_clin_27</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_42</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="1">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="D10" s="1">
-        <f t="shared" si="6"/>
-        <v>30</v>
+        <f t="shared" si="5"/>
+        <v>45</v>
       </c>
       <c r="E10" s="1">
-        <f t="shared" si="1"/>
-        <v>27</v>
+        <f t="shared" si="2"/>
+        <v>42</v>
       </c>
       <c r="F10" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A10,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>39.624074444000001</v>
+        <v>302.93943240646001</v>
       </c>
       <c r="G10" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A10,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>7924814.8888000008</v>
+        <v>7045103.0792200007</v>
       </c>
       <c r="H10" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A10,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>0.5</v>
+        <v>4.3</v>
       </c>
       <c r="I10" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A10,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>-1E-3</v>
+        <v>3.3552871864818119</v>
       </c>
       <c r="J10" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A10,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>0.94989916767749982</v>
+        <v>5.3927965254376069</v>
       </c>
       <c r="K10" s="2">
         <v>3</v>
       </c>
       <c r="L10" s="2">
-        <f t="shared" si="2"/>
-        <v>-1E-3</v>
+        <f t="shared" si="3"/>
+        <v>1.4658615594454361</v>
       </c>
       <c r="M10" s="2">
-        <f t="shared" si="3"/>
-        <v>1.8496975030324996</v>
+        <f t="shared" si="4"/>
+        <v>7.5783895763128211</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="1" t="str">
-        <f t="shared" ref="A11:A21" si="7">""&amp;B11&amp;"_"&amp;E11</f>
-        <v>incidence_clin_32</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_47</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="1">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="D11" s="1">
-        <f t="shared" si="6"/>
-        <v>35</v>
+        <f t="shared" si="5"/>
+        <v>50</v>
       </c>
       <c r="E11" s="1">
-        <f t="shared" si="1"/>
-        <v>32</v>
+        <f t="shared" si="2"/>
+        <v>47</v>
       </c>
       <c r="F11" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A11,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>73.935344383010005</v>
+        <v>676.82244818309994</v>
       </c>
       <c r="G11" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A11,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>6721394.9439099999</v>
+        <v>7124446.8229799997</v>
       </c>
       <c r="H11" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A11,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>1.1000000000000001</v>
+        <v>9.5</v>
       </c>
       <c r="I11" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A11,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>-1E-3</v>
+        <v>8.0953120007060804</v>
       </c>
       <c r="J11" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A11,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>1.7431061741782465</v>
+        <v>11.050308439923784</v>
       </c>
       <c r="K11" s="2">
         <v>3</v>
       </c>
       <c r="L11" s="2">
-        <f t="shared" si="2"/>
-        <v>-1E-3</v>
+        <f t="shared" si="3"/>
+        <v>5.2859360021182411</v>
       </c>
       <c r="M11" s="2">
-        <f t="shared" si="3"/>
-        <v>3.0293185225347394</v>
+        <f t="shared" si="4"/>
+        <v>14.150925319771352</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_37</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_52</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="1">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="D12" s="1">
-        <f t="shared" si="6"/>
-        <v>40</v>
+        <f t="shared" si="5"/>
+        <v>55</v>
       </c>
       <c r="E12" s="1">
-        <f t="shared" si="1"/>
-        <v>37</v>
+        <f t="shared" si="2"/>
+        <v>52</v>
       </c>
       <c r="F12" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A12,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>143.68291641088004</v>
+        <v>1207.9553240984499</v>
       </c>
       <c r="G12" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A12,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>6531041.6550400006</v>
+        <v>6529488.2383699995</v>
       </c>
       <c r="H12" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A12,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>2.2000000000000002</v>
+        <v>18.5</v>
       </c>
       <c r="I12" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A12,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>1.5096614770209527</v>
+        <v>16.450899786160679</v>
       </c>
       <c r="J12" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A12,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>3.0550947154719745</v>
+        <v>20.708865931030658</v>
       </c>
       <c r="K12" s="2">
         <v>3</v>
       </c>
       <c r="L12" s="2">
-        <f t="shared" si="2"/>
-        <v>0.1289844310628574</v>
+        <f t="shared" si="3"/>
+        <v>12.352699358482038</v>
       </c>
       <c r="M12" s="2">
-        <f t="shared" si="3"/>
-        <v>4.7652841464159232</v>
+        <f t="shared" si="4"/>
+        <v>25.126597793091975</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_42</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_57</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C13" s="1">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="D13" s="1">
-        <f t="shared" si="6"/>
-        <v>45</v>
+        <f t="shared" si="5"/>
+        <v>60</v>
       </c>
       <c r="E13" s="1">
-        <f t="shared" si="1"/>
-        <v>42</v>
+        <f t="shared" si="2"/>
+        <v>57</v>
       </c>
       <c r="F13" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A13,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>302.93943240646001</v>
+        <v>2011.48471233549</v>
       </c>
       <c r="G13" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A13,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>7045103.0792200007</v>
+        <v>5864386.9164300002</v>
       </c>
       <c r="H13" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A13,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>4.3</v>
+        <v>34.299999999999997</v>
       </c>
       <c r="I13" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A13,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>3.3552871864818119</v>
+        <v>31.355881788353273</v>
       </c>
       <c r="J13" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A13,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>5.3927965254376069</v>
+        <v>37.418662813000019</v>
       </c>
       <c r="K13" s="2">
         <v>3</v>
       </c>
       <c r="L13" s="2">
-        <f t="shared" si="2"/>
-        <v>1.4658615594454361</v>
+        <f t="shared" si="3"/>
+        <v>25.467645365059823</v>
       </c>
       <c r="M13" s="2">
-        <f t="shared" si="3"/>
-        <v>7.5783895763128211</v>
+        <f t="shared" si="4"/>
+        <v>43.655988439000062</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_47</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_62</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C14" s="1">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="D14" s="1">
-        <f t="shared" si="6"/>
-        <v>50</v>
+        <f t="shared" si="5"/>
+        <v>65</v>
       </c>
       <c r="E14" s="1">
-        <f t="shared" si="1"/>
-        <v>47</v>
+        <f t="shared" si="2"/>
+        <v>62</v>
       </c>
       <c r="F14" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A14,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>676.82244818309994</v>
+        <v>2680.3830625913301</v>
       </c>
       <c r="G14" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A14,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>7124446.8229799997</v>
+        <v>5066886.6967700003</v>
       </c>
       <c r="H14" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A14,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>9.5</v>
+        <v>52.9</v>
       </c>
       <c r="I14" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A14,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>8.0953120007060804</v>
+        <v>48.962568981583438</v>
       </c>
       <c r="J14" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A14,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>11.050308439923784</v>
+        <v>57.03248272374185</v>
       </c>
       <c r="K14" s="2">
         <v>3</v>
       </c>
       <c r="L14" s="2">
-        <f t="shared" si="2"/>
-        <v>5.2859360021182411</v>
+        <f t="shared" si="3"/>
+        <v>41.087706944750316</v>
       </c>
       <c r="M14" s="2">
-        <f t="shared" si="3"/>
-        <v>14.150925319771352</v>
+        <f t="shared" si="4"/>
+        <v>65.297448171225554</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_52</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_67</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C15" s="1">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="D15" s="1">
-        <f t="shared" si="6"/>
-        <v>55</v>
+        <f t="shared" si="5"/>
+        <v>70</v>
       </c>
       <c r="E15" s="1">
-        <f t="shared" si="1"/>
-        <v>52</v>
+        <f t="shared" si="2"/>
+        <v>67</v>
       </c>
       <c r="F15" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A15,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>1207.9553240984499</v>
+        <v>3404.15346684312</v>
       </c>
       <c r="G15" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A15,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>6529488.2383699995</v>
+        <v>4111296.4575399999</v>
       </c>
       <c r="H15" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A15,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>18.5</v>
+        <v>82.8</v>
       </c>
       <c r="I15" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A15,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>16.450899786160679</v>
+        <v>77.342309223810418</v>
       </c>
       <c r="J15" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A15,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>20.708865931030658</v>
+        <v>88.507822558360061</v>
       </c>
       <c r="K15" s="2">
         <v>3</v>
       </c>
       <c r="L15" s="2">
-        <f t="shared" si="2"/>
-        <v>12.352699358482038</v>
+        <f t="shared" si="3"/>
+        <v>66.426927671431258</v>
       </c>
       <c r="M15" s="2">
-        <f t="shared" si="3"/>
-        <v>25.126597793091975</v>
+        <f t="shared" si="4"/>
+        <v>99.92346767508019</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_57</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_72</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C16" s="1">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="D16" s="1">
-        <f t="shared" si="6"/>
-        <v>60</v>
+        <f t="shared" si="5"/>
+        <v>75</v>
       </c>
       <c r="E16" s="1">
-        <f t="shared" si="1"/>
-        <v>57</v>
+        <f t="shared" si="2"/>
+        <v>72</v>
       </c>
       <c r="F16" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A16,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>2011.48471233549</v>
+        <v>3492.4151367184104</v>
       </c>
       <c r="G16" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A16,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>5864386.9164300002</v>
+        <v>3201113.7825100003</v>
       </c>
       <c r="H16" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A16,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>34.299999999999997</v>
+        <v>109.1</v>
       </c>
       <c r="I16" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A16,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>31.355881788353273</v>
+        <v>102.00634410001473</v>
       </c>
       <c r="J16" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A16,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>37.418662813000019</v>
+        <v>116.51359947428682</v>
       </c>
       <c r="K16" s="2">
         <v>3</v>
       </c>
       <c r="L16" s="2">
-        <f t="shared" si="2"/>
-        <v>25.467645365059823</v>
+        <f t="shared" si="3"/>
+        <v>87.819032300044199</v>
       </c>
       <c r="M16" s="2">
-        <f t="shared" si="3"/>
-        <v>43.655988439000062</v>
+        <f t="shared" si="4"/>
+        <v>131.34079842286047</v>
       </c>
       <c r="N16" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:14">
       <c r="A17" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_62</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_77</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C17" s="1">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="D17" s="1">
-        <f t="shared" si="6"/>
-        <v>65</v>
+        <f t="shared" si="5"/>
+        <v>80</v>
       </c>
       <c r="E17" s="1">
-        <f t="shared" si="1"/>
-        <v>62</v>
+        <f t="shared" si="2"/>
+        <v>77</v>
       </c>
       <c r="F17" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A17,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>2680.3830625913301</v>
+        <v>2981.061795768579</v>
       </c>
       <c r="G17" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A17,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>5066886.6967700003</v>
+        <v>2254963.5368899996</v>
       </c>
       <c r="H17" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A17,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>52.9</v>
+        <v>132.19999999999999</v>
       </c>
       <c r="I17" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A17,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>48.962568981583438</v>
+        <v>122.92121750008623</v>
       </c>
       <c r="J17" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A17,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>57.03248272374185</v>
+        <v>141.91891919184286</v>
       </c>
       <c r="K17" s="2">
         <v>3</v>
       </c>
       <c r="L17" s="2">
-        <f t="shared" si="2"/>
-        <v>41.087706944750316</v>
+        <f t="shared" si="3"/>
+        <v>104.36365250025871</v>
       </c>
       <c r="M17" s="2">
-        <f t="shared" si="3"/>
-        <v>65.297448171225554</v>
+        <f t="shared" si="4"/>
+        <v>161.3567575755286</v>
       </c>
       <c r="N17" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_67</v>
+        <f t="shared" si="6"/>
+        <v>incidence_clin_82</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C18" s="1">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D18" s="1">
-        <f t="shared" si="6"/>
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="E18" s="1">
-        <f t="shared" si="1"/>
-        <v>67</v>
+        <f t="shared" si="2"/>
+        <v>82</v>
       </c>
       <c r="F18" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A18,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>3404.15346684312</v>
+        <v>2005.43857566867</v>
       </c>
       <c r="G18" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A18,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>4111296.4575399999</v>
+        <v>1343227.4451899999</v>
       </c>
       <c r="H18" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A18,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>82.8</v>
+        <v>149.30000000000001</v>
       </c>
       <c r="I18" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A18,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>77.342309223810418</v>
+        <v>136.61155641874043</v>
       </c>
       <c r="J18" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A18,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>88.507822558360061</v>
+        <v>162.74445396561978</v>
       </c>
       <c r="K18" s="2">
         <v>3</v>
       </c>
       <c r="L18" s="2">
-        <f t="shared" si="2"/>
-        <v>66.426927671431258</v>
+        <f t="shared" si="3"/>
+        <v>111.23466925622128</v>
       </c>
       <c r="M18" s="2">
-        <f t="shared" si="3"/>
-        <v>99.92346767508019</v>
+        <f t="shared" si="4"/>
+        <v>189.63336189685933</v>
       </c>
       <c r="N18" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_72</v>
+        <f t="shared" ref="A19" si="7">""&amp;B19&amp;"_"&amp;E19</f>
+        <v>incidence_clin_92</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C19" s="1">
-        <v>70</v>
+        <v>85</v>
       </c>
       <c r="D19" s="1">
-        <f t="shared" si="6"/>
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="E19" s="1">
-        <f t="shared" si="1"/>
-        <v>72</v>
+        <f t="shared" ref="E19" si="8">FLOOR(AVERAGE(C19,D19), 1)</f>
+        <v>92</v>
       </c>
       <c r="F19" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A19,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>3492.4151367184104</v>
+        <v>1258.9121706180499</v>
       </c>
       <c r="G19" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A19,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>3201113.7825100003</v>
+        <v>888434.84165000007</v>
       </c>
       <c r="H19" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A19,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>109.1</v>
+        <v>141.69999999999999</v>
       </c>
       <c r="I19" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A19,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>102.00634410001473</v>
+        <v>126.59273939334641</v>
       </c>
       <c r="J19" s="2">
         <f>INDEX(bounds!$24:$42,MATCH(targets!$A19,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>116.51359947428682</v>
+        <v>157.89999500379088</v>
       </c>
       <c r="K19" s="2">
         <v>3</v>
       </c>
       <c r="L19" s="2">
-        <f t="shared" si="2"/>
-        <v>87.819032300044199</v>
+        <f t="shared" si="3"/>
+        <v>96.378218180039241</v>
       </c>
       <c r="M19" s="2">
-        <f t="shared" si="3"/>
-        <v>131.34079842286047</v>
+        <f t="shared" si="4"/>
+        <v>190.29998501137266</v>
       </c>
       <c r="N19" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_77</v>
+        <f t="shared" ref="A20:A22" si="9">""&amp;B20&amp;"_"&amp;E20</f>
+        <v>stage_distr_1</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="1">
-        <v>75</v>
-      </c>
-      <c r="D20" s="1">
-        <f t="shared" si="6"/>
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="E20" s="1">
-        <f t="shared" si="1"/>
-        <v>77</v>
+        <v>1</v>
       </c>
       <c r="F20" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A20,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>2981.061795768579</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A20,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
+        <v>21522.9</v>
       </c>
       <c r="G20" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A20,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>2254963.5368899996</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A20,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
+        <v>27630.75</v>
       </c>
       <c r="H20" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A20,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>132.19999999999999</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A20,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
+        <v>0.77894736842105272</v>
       </c>
       <c r="I20" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A20,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>122.92121750008623</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A20,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
+        <v>0.769196681186881</v>
       </c>
       <c r="J20" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A20,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>141.91891919184286</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A20,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
+        <v>0.78862050322746191</v>
       </c>
       <c r="K20" s="2">
         <v>3</v>
       </c>
       <c r="L20" s="2">
-        <f t="shared" si="2"/>
-        <v>104.36365250025871</v>
+        <f t="shared" si="3"/>
+        <v>0.74969530671853757</v>
       </c>
       <c r="M20" s="2">
-        <f t="shared" si="3"/>
-        <v>161.3567575755286</v>
+        <f t="shared" si="4"/>
+        <v>0.80796677284028029</v>
       </c>
       <c r="N20" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="1" t="str">
-        <f t="shared" si="7"/>
-        <v>incidence_clin_82</v>
+        <f t="shared" si="9"/>
+        <v>stage_distr_2</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C21" s="1">
-        <v>80</v>
-      </c>
-      <c r="D21" s="1">
-        <v>85</v>
+        <v>8</v>
       </c>
       <c r="E21" s="1">
-        <f t="shared" si="1"/>
-        <v>82</v>
+        <v>2</v>
       </c>
       <c r="F21" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A21,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>2005.43857566867</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A21,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
+        <v>5235.3</v>
       </c>
       <c r="G21" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A21,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>1343227.4451899999</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A21,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
+        <v>27630.75</v>
       </c>
       <c r="H21" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A21,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>149.30000000000001</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A21,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
+        <v>0.18947368421052632</v>
       </c>
       <c r="I21" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A21,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>136.61155641874043</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A21,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
+        <v>0.18034480649920773</v>
       </c>
       <c r="J21" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A21,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>162.74445396561978</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A21,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
+        <v>0.19868889386973168</v>
       </c>
       <c r="K21" s="2">
         <v>3</v>
       </c>
       <c r="L21" s="2">
-        <f t="shared" si="2"/>
-        <v>111.23466925622128</v>
+        <f t="shared" si="3"/>
+        <v>0.16208705107657054</v>
       </c>
       <c r="M21" s="2">
-        <f t="shared" si="3"/>
-        <v>189.63336189685933</v>
+        <f t="shared" si="4"/>
+        <v>0.2171193131881424</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="1" t="str">
-        <f t="shared" ref="A22" si="8">""&amp;B22&amp;"_"&amp;E22</f>
-        <v>incidence_clin_92</v>
+        <f t="shared" si="9"/>
+        <v>stage_distr_3</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C22" s="1">
-        <v>85</v>
-      </c>
-      <c r="D22" s="1">
-        <v>100</v>
+        <v>8</v>
       </c>
       <c r="E22" s="1">
-        <f t="shared" ref="E22" si="9">FLOOR(AVERAGE(C22,D22), 1)</f>
-        <v>92</v>
+        <v>3</v>
       </c>
       <c r="F22" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A22,bounds!$A$24:$A$42,0), MATCH(F$1,bounds!$24:$24,0))</f>
-        <v>1258.9121706180499</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A22,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
+        <v>872.55</v>
       </c>
       <c r="G22" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A22,bounds!$A$24:$A$42,0), MATCH(G$1,bounds!$24:$24,0))</f>
-        <v>888434.84165000007</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A22,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
+        <v>27630.75</v>
       </c>
       <c r="H22" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A22,bounds!$A$24:$A$42,0), MATCH(H$1,bounds!$24:$24,0))</f>
-        <v>141.69999999999999</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A22,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
+        <v>3.1578947368421054E-2</v>
       </c>
       <c r="I22" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A22,bounds!$A$24:$A$42,0), MATCH(I$1,bounds!$24:$24,0))</f>
-        <v>126.59273939334641</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A22,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
+        <v>2.7549225740961719E-2</v>
       </c>
       <c r="J22" s="2">
-        <f>INDEX(bounds!$24:$42,MATCH(targets!$A22,bounds!$A$24:$A$42,0), MATCH(J$1,bounds!$24:$24,0))</f>
-        <v>157.89999500379088</v>
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A22,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
+        <v>3.5738898544387512E-2</v>
       </c>
       <c r="K22" s="2">
         <v>3</v>
       </c>
       <c r="L22" s="2">
-        <f t="shared" si="2"/>
-        <v>96.378218180039241</v>
+        <f t="shared" si="3"/>
+        <v>1.948978248604305E-2</v>
       </c>
       <c r="M22" s="2">
-        <f t="shared" si="3"/>
-        <v>190.29998501137266</v>
+        <f t="shared" si="4"/>
+        <v>4.405880089632043E-2</v>
       </c>
       <c r="N22" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14">
-      <c r="A23" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>stage_distr_1</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="1">
-        <v>1</v>
-      </c>
-      <c r="F23" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
-        <v>21522.9</v>
-      </c>
-      <c r="G23" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
-        <v>27630.75</v>
-      </c>
-      <c r="H23" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
-        <v>0.77894736842105272</v>
-      </c>
-      <c r="I23" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
-        <v>0.769196681186881</v>
-      </c>
-      <c r="J23" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
-        <v>0.78862050322746191</v>
-      </c>
-      <c r="K23" s="2">
-        <v>3</v>
-      </c>
-      <c r="L23" s="2">
-        <f t="shared" si="2"/>
-        <v>0.74969530671853757</v>
-      </c>
-      <c r="M23" s="2">
-        <f t="shared" si="3"/>
-        <v>0.80796677284028029</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14">
-      <c r="A24" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>stage_distr_2</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E24" s="1">
-        <v>2</v>
-      </c>
-      <c r="F24" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
-        <v>5235.3</v>
-      </c>
-      <c r="G24" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
-        <v>27630.75</v>
-      </c>
-      <c r="H24" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
-        <v>0.18947368421052632</v>
-      </c>
-      <c r="I24" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
-        <v>0.18034480649920773</v>
-      </c>
-      <c r="J24" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
-        <v>0.19868889386973168</v>
-      </c>
-      <c r="K24" s="2">
-        <v>3</v>
-      </c>
-      <c r="L24" s="2">
-        <f t="shared" si="2"/>
-        <v>0.16208705107657054</v>
-      </c>
-      <c r="M24" s="2">
-        <f t="shared" si="3"/>
-        <v>0.2171193131881424</v>
-      </c>
-      <c r="N24" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14">
-      <c r="A25" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>stage_distr_3</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E25" s="1">
-        <v>3</v>
-      </c>
-      <c r="F25" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
-        <v>872.55</v>
-      </c>
-      <c r="G25" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
-        <v>27630.75</v>
-      </c>
-      <c r="H25" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
-        <v>3.1578947368421054E-2</v>
-      </c>
-      <c r="I25" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
-        <v>2.7549225740961719E-2</v>
-      </c>
-      <c r="J25" s="2">
-        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
-        <v>3.5738898544387512E-2</v>
-      </c>
-      <c r="K25" s="2">
-        <v>3</v>
-      </c>
-      <c r="L25" s="2">
-        <f t="shared" si="2"/>
-        <v>1.948978248604305E-2</v>
-      </c>
-      <c r="M25" s="2">
-        <f t="shared" si="3"/>
-        <v>4.405880089632043E-2</v>
-      </c>
-      <c r="N25" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -2009,26 +1847,26 @@
         <v>71</v>
       </c>
       <c r="G8" s="1">
-        <v>12</v>
+        <v>1810</v>
       </c>
       <c r="H8" s="1">
         <v>1</v>
       </c>
       <c r="I8" s="1">
         <f>H8/G8</f>
-        <v>8.3333333333333329E-2</v>
+        <v>5.5248618784530391E-4</v>
       </c>
       <c r="J8" s="1">
         <f t="shared" ref="J8:J10" si="1">$B$5^2/G8</f>
-        <v>0.32012156839117695</v>
+        <v>2.1223529396100132E-3</v>
       </c>
       <c r="K8" s="1">
         <f t="shared" ref="K8:K10" si="2">(I8+J8/2)/(J8+1)-$B$5/(J8+1)*SQRT(I8*(1-I8)/G8+J8/(4*G8))</f>
-        <v>1.4865094404917123E-2</v>
+        <v>9.7534036711855159E-5</v>
       </c>
       <c r="L8" s="1">
         <f t="shared" ref="L8:L10" si="3">(I8+J8/2)/(J8+1)+$B$5/(J8+1)*SQRT(I8*(1-I8)/G8+J8/(4*G8))</f>
-        <v>0.35387991114111689</v>
+        <v>3.1229562615372915E-3</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -2050,26 +1888,26 @@
         <v>80</v>
       </c>
       <c r="G9" s="1">
-        <v>16</v>
+        <v>1307</v>
       </c>
       <c r="H9" s="1">
         <v>2</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" ref="I9:I10" si="5">H9/G9</f>
-        <v>0.125</v>
+        <v>1.530221882172915E-3</v>
       </c>
       <c r="J9" s="1">
         <f t="shared" si="1"/>
-        <v>0.24009117629338272</v>
+        <v>2.9391421734461542E-3</v>
       </c>
       <c r="K9" s="1">
         <f t="shared" si="2"/>
-        <v>3.4977487743240443E-2</v>
+        <v>4.1974238437163421E-4</v>
       </c>
       <c r="L9" s="1">
         <f t="shared" si="3"/>
-        <v>0.36022827265758689</v>
+        <v>5.562261593248006E-3</v>
       </c>
     </row>
     <row r="10" spans="1:12">
@@ -2091,26 +1929,26 @@
         <v>92</v>
       </c>
       <c r="G10" s="1">
-        <v>8</v>
+        <v>418</v>
       </c>
       <c r="H10" s="1">
         <v>2</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" si="5"/>
-        <v>0.25</v>
+        <v>4.7846889952153108E-3</v>
       </c>
       <c r="J10" s="1">
         <f t="shared" si="1"/>
-        <v>0.48018235258676545</v>
+        <v>9.1900928724739806E-3</v>
       </c>
       <c r="K10" s="1">
         <f t="shared" si="2"/>
-        <v>7.1479212752109056E-2</v>
+        <v>1.313116453381476E-3</v>
       </c>
       <c r="L10" s="1">
         <f t="shared" si="3"/>
-        <v>0.59072456968983111</v>
+        <v>1.7275523085785241E-2</v>
       </c>
     </row>
     <row r="11" spans="1:12">
@@ -2223,17 +2061,17 @@
     </row>
     <row r="15" spans="1:12">
       <c r="A15" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:12">
       <c r="A16" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:24">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B17" s="1">
         <v>1000000</v>
@@ -2241,7 +2079,7 @@
     </row>
     <row r="18" spans="1:24">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B18" s="1">
         <v>23898718</v>
@@ -2249,7 +2087,7 @@
     </row>
     <row r="19" spans="1:24">
       <c r="A19" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B19" s="1">
         <v>1989</v>
@@ -2259,7 +2097,7 @@
     </row>
     <row r="20" spans="1:24">
       <c r="A20" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B20" s="1">
         <v>1993</v>
@@ -2269,7 +2107,7 @@
     </row>
     <row r="21" spans="1:24">
       <c r="A21" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" s="1">
         <v>100000</v>
@@ -2279,7 +2117,7 @@
     </row>
     <row r="22" spans="1:24">
       <c r="A22" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" s="5">
         <v>22682</v>
@@ -2289,10 +2127,10 @@
     </row>
     <row r="23" spans="1:24">
       <c r="D23" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="W23" s="4"/>
       <c r="X23" s="5"/>
@@ -2314,7 +2152,7 @@
         <v>5</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>11</v>
@@ -2323,19 +2161,19 @@
         <v>12</v>
       </c>
       <c r="I24" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J24" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="J24" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="K24" s="1" t="s">
         <v>2</v>
       </c>
       <c r="L24" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M24" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="N24" s="1" t="s">
         <v>9</v>
@@ -2344,10 +2182,10 @@
         <v>10</v>
       </c>
       <c r="Q24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R24" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="R24" s="1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:24">
@@ -3498,7 +3336,7 @@
     </row>
     <row r="43" spans="1:18">
       <c r="A43" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F43" s="1">
         <f>SUM(F25:F42)</f>
@@ -3515,7 +3353,7 @@
     </row>
     <row r="44" spans="1:18">
       <c r="A44" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F44" s="3"/>
       <c r="G44" s="1">

</xml_diff>

<commit_message>
Regenerate bladder cancer model parameters with incidental cancer data
</commit_message>
<xml_diff>
--- a/data/bladder/targets.xlsx
+++ b/data/bladder/targets.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10921"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder_incidental/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/selinapi/Repositories/tutorial_cancer_modeling_des/data/bladder/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344F28A2-5AF7-E94E-B86F-FAE3D5F1DCFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A7F395-6CFE-8043-837E-9805B62E6986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2740" yWindow="1020" windowWidth="21160" windowHeight="17740" activeTab="1" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
+    <workbookView xWindow="4000" yWindow="760" windowWidth="26240" windowHeight="17740" xr2:uid="{A45334B4-46D3-3441-9F0C-EDD51E1C869C}"/>
   </bookViews>
   <sheets>
     <sheet name="targets" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="45">
   <si>
     <t>target_names</t>
   </si>
@@ -163,6 +163,15 @@
   </si>
   <si>
     <t>cumulative proportion of cases</t>
+  </si>
+  <si>
+    <t>prevalence_incidental</t>
+  </si>
+  <si>
+    <t>Suen 1974</t>
+  </si>
+  <si>
+    <t>include_target</t>
   </si>
 </sst>
 </file>
@@ -573,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B407C086-A524-D44D-8D0D-4CA59B33056E}">
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="25.33203125" style="1" customWidth="1"/>
@@ -581,7 +590,7 @@
     <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -624,8 +633,11 @@
       <c r="N1" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15">
       <c r="A2" s="1" t="str">
         <f t="shared" ref="A2:A7" si="0">""&amp;B2&amp;"_"&amp;E2</f>
         <v>incidence_clin_2</v>
@@ -678,8 +690,11 @@
       <c r="N2" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="3" spans="1:14">
+      <c r="O2" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15">
       <c r="A3" s="1" t="str">
         <f t="shared" si="0"/>
         <v>incidence_clin_7</v>
@@ -732,8 +747,11 @@
       <c r="N3" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:14">
+      <c r="O3" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15">
       <c r="A4" s="1" t="str">
         <f t="shared" si="0"/>
         <v>incidence_clin_12</v>
@@ -786,8 +804,11 @@
       <c r="N4" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:14">
+      <c r="O4" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15">
       <c r="A5" s="1" t="str">
         <f t="shared" si="0"/>
         <v>incidence_clin_17</v>
@@ -840,8 +861,11 @@
       <c r="N5" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:14">
+      <c r="O5" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15">
       <c r="A6" s="1" t="str">
         <f t="shared" si="0"/>
         <v>incidence_clin_22</v>
@@ -894,8 +918,11 @@
       <c r="N6" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="7" spans="1:14">
+      <c r="O6" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15">
       <c r="A7" s="1" t="str">
         <f t="shared" si="0"/>
         <v>incidence_clin_27</v>
@@ -948,8 +975,11 @@
       <c r="N7" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="8" spans="1:14">
+      <c r="O7" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15">
       <c r="A8" s="1" t="str">
         <f t="shared" ref="A8:A18" si="6">""&amp;B8&amp;"_"&amp;E8</f>
         <v>incidence_clin_32</v>
@@ -1002,8 +1032,11 @@
       <c r="N8" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:14">
+      <c r="O8" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
       <c r="A9" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_37</v>
@@ -1056,8 +1089,11 @@
       <c r="N9" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="10" spans="1:14">
+      <c r="O9" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15">
       <c r="A10" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_42</v>
@@ -1110,8 +1146,11 @@
       <c r="N10" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:14">
+      <c r="O10" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15">
       <c r="A11" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_47</v>
@@ -1164,8 +1203,11 @@
       <c r="N11" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="12" spans="1:14">
+      <c r="O11" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
       <c r="A12" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_52</v>
@@ -1218,8 +1260,11 @@
       <c r="N12" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:14">
+      <c r="O12" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15">
       <c r="A13" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_57</v>
@@ -1272,8 +1317,11 @@
       <c r="N13" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="14" spans="1:14">
+      <c r="O13" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15">
       <c r="A14" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_62</v>
@@ -1326,8 +1374,11 @@
       <c r="N14" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="15" spans="1:14">
+      <c r="O14" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15">
       <c r="A15" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_67</v>
@@ -1380,8 +1431,11 @@
       <c r="N15" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="16" spans="1:14">
+      <c r="O15" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15">
       <c r="A16" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_72</v>
@@ -1434,8 +1488,11 @@
       <c r="N16" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="17" spans="1:14">
+      <c r="O16" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15">
       <c r="A17" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_77</v>
@@ -1488,8 +1545,11 @@
       <c r="N17" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="1:14">
+      <c r="O17" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15">
       <c r="A18" s="1" t="str">
         <f t="shared" si="6"/>
         <v>incidence_clin_82</v>
@@ -1541,8 +1601,11 @@
       <c r="N18" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="19" spans="1:14">
+      <c r="O18" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15">
       <c r="A19" s="1" t="str">
         <f t="shared" ref="A19" si="7">""&amp;B19&amp;"_"&amp;E19</f>
         <v>incidence_clin_92</v>
@@ -1594,10 +1657,13 @@
       <c r="N19" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:14">
+      <c r="O19" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15">
       <c r="A20" s="1" t="str">
-        <f t="shared" ref="A20:A22" si="9">""&amp;B20&amp;"_"&amp;E20</f>
+        <f t="shared" ref="A20:A23" si="9">""&amp;B20&amp;"_"&amp;E20</f>
         <v>stage_distr_1</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1640,8 +1706,11 @@
       <c r="N20" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="21" spans="1:14">
+      <c r="O20" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15">
       <c r="A21" s="1" t="str">
         <f t="shared" si="9"/>
         <v>stage_distr_2</v>
@@ -1686,8 +1755,11 @@
       <c r="N21" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:14">
+      <c r="O21" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15">
       <c r="A22" s="1" t="str">
         <f t="shared" si="9"/>
         <v>stage_distr_3</v>
@@ -1731,6 +1803,180 @@
       </c>
       <c r="N22" s="1" t="s">
         <v>20</v>
+      </c>
+      <c r="O22" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15">
+      <c r="A23" s="1" t="str">
+        <f t="shared" si="9"/>
+        <v>prevalence_incidental_71</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C23" s="1">
+        <v>66</v>
+      </c>
+      <c r="D23" s="1">
+        <f>C23+10</f>
+        <v>76</v>
+      </c>
+      <c r="E23" s="1">
+        <f t="shared" ref="E23:E25" si="10">FLOOR(AVERAGE(C23,D23), 1)</f>
+        <v>71</v>
+      </c>
+      <c r="F23" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
+        <v>1</v>
+      </c>
+      <c r="G23" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
+        <v>1810</v>
+      </c>
+      <c r="H23" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
+        <v>5.5248618784530391E-4</v>
+      </c>
+      <c r="I23" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
+        <v>9.7534036711855159E-5</v>
+      </c>
+      <c r="J23" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A23,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
+        <v>3.1229562615372915E-3</v>
+      </c>
+      <c r="K23" s="2">
+        <v>3</v>
+      </c>
+      <c r="L23" s="2">
+        <f t="shared" ref="L23:L25" si="11">IF(H23 - K23*(H23-I23) &lt;= 0, -0.001, H23 - K23*(H23-I23))</f>
+        <v>-1E-3</v>
+      </c>
+      <c r="M23" s="2">
+        <f t="shared" ref="M23:M25" si="12">H23 + K23*(J23-H23)</f>
+        <v>8.2638964089212664E-3</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="O23" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15">
+      <c r="A24" s="1" t="str">
+        <f t="shared" ref="A24:A25" si="13">""&amp;B24&amp;"_"&amp;E24</f>
+        <v>prevalence_incidental_81</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C24" s="1">
+        <v>76</v>
+      </c>
+      <c r="D24" s="1">
+        <f t="shared" ref="D24:D25" si="14">C24+10</f>
+        <v>86</v>
+      </c>
+      <c r="E24" s="1">
+        <f t="shared" si="10"/>
+        <v>81</v>
+      </c>
+      <c r="F24" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
+        <v>2</v>
+      </c>
+      <c r="G24" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
+        <v>1307</v>
+      </c>
+      <c r="H24" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
+        <v>1.530221882172915E-3</v>
+      </c>
+      <c r="I24" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
+        <v>4.1974238437163421E-4</v>
+      </c>
+      <c r="J24" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A24,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
+        <v>5.562261593248006E-3</v>
+      </c>
+      <c r="K24" s="2">
+        <v>3</v>
+      </c>
+      <c r="L24" s="2">
+        <f t="shared" si="11"/>
+        <v>-1E-3</v>
+      </c>
+      <c r="M24" s="2">
+        <f t="shared" si="12"/>
+        <v>1.3626341015398186E-2</v>
+      </c>
+      <c r="N24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="O24" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15">
+      <c r="A25" s="1" t="str">
+        <f t="shared" si="13"/>
+        <v>prevalence_incidental_90</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="1">
+        <v>85</v>
+      </c>
+      <c r="D25" s="1">
+        <f t="shared" si="14"/>
+        <v>95</v>
+      </c>
+      <c r="E25" s="1">
+        <f t="shared" si="10"/>
+        <v>90</v>
+      </c>
+      <c r="F25" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(F$1,bounds!$7:$7,0))</f>
+        <v>2</v>
+      </c>
+      <c r="G25" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(G$1,bounds!$7:$7,0))</f>
+        <v>418</v>
+      </c>
+      <c r="H25" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(H$1,bounds!$7:$7,0))</f>
+        <v>4.7846889952153108E-3</v>
+      </c>
+      <c r="I25" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(I$1,bounds!$7:$7,0))</f>
+        <v>1.313116453381476E-3</v>
+      </c>
+      <c r="J25" s="2">
+        <f>INDEX(bounds!$A$7:$L$1048576,MATCH(targets!$A25,bounds!$A$7:$A$1048576,0), MATCH(J$1,bounds!$7:$7,0))</f>
+        <v>1.7275523085785241E-2</v>
+      </c>
+      <c r="K25" s="2">
+        <v>3</v>
+      </c>
+      <c r="L25" s="2">
+        <f t="shared" si="11"/>
+        <v>-1E-3</v>
+      </c>
+      <c r="M25" s="2">
+        <f t="shared" si="12"/>
+        <v>4.2257191266925093E-2</v>
+      </c>
+      <c r="N25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="O25" s="1" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1831,15 +2077,16 @@
     <row r="8" spans="1:12">
       <c r="A8" s="1" t="str">
         <f>B8&amp;"_"&amp;E8</f>
-        <v>prevalence_preclin_71</v>
+        <v>prevalence_incidental_71</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C8" s="2">
         <v>66</v>
       </c>
       <c r="D8" s="2">
+        <f>C8+10</f>
         <v>76</v>
       </c>
       <c r="E8" s="1">
@@ -1872,20 +2119,21 @@
     <row r="9" spans="1:12">
       <c r="A9" s="1" t="str">
         <f t="shared" ref="A9:A13" si="4">B9&amp;"_"&amp;E9</f>
-        <v>prevalence_preclin_80</v>
+        <v>prevalence_incidental_81</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C9" s="2">
         <v>76</v>
       </c>
       <c r="D9" s="2">
-        <v>85</v>
+        <f t="shared" ref="D9:D10" si="5">C9+10</f>
+        <v>86</v>
       </c>
       <c r="E9" s="1">
         <f t="shared" si="0"/>
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G9" s="1">
         <v>1307</v>
@@ -1894,7 +2142,7 @@
         <v>2</v>
       </c>
       <c r="I9" s="1">
-        <f t="shared" ref="I9:I10" si="5">H9/G9</f>
+        <f t="shared" ref="I9:I10" si="6">H9/G9</f>
         <v>1.530221882172915E-3</v>
       </c>
       <c r="J9" s="1">
@@ -1913,20 +2161,21 @@
     <row r="10" spans="1:12">
       <c r="A10" s="1" t="str">
         <f t="shared" si="4"/>
-        <v>prevalence_preclin_92</v>
+        <v>prevalence_incidental_90</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C10" s="2">
         <v>85</v>
       </c>
       <c r="D10" s="2">
-        <v>100</v>
+        <f t="shared" si="5"/>
+        <v>95</v>
       </c>
       <c r="E10" s="1">
         <f t="shared" si="0"/>
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="G10" s="1">
         <v>418</v>
@@ -1935,7 +2184,7 @@
         <v>2</v>
       </c>
       <c r="I10" s="1">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>4.7846889952153108E-3</v>
       </c>
       <c r="J10" s="1">
@@ -1971,11 +2220,11 @@
         <v>21522.9</v>
       </c>
       <c r="I11" s="1">
-        <f t="shared" ref="I11:I13" si="6">H11/G11</f>
+        <f t="shared" ref="I11:I13" si="7">H11/G11</f>
         <v>0.77894736842105272</v>
       </c>
       <c r="J11" s="1">
-        <f t="shared" ref="J11:J13" si="7">$B$5^2/G11</f>
+        <f t="shared" ref="J11:J13" si="8">$B$5^2/G11</f>
         <v>1.3902839483887058E-4</v>
       </c>
       <c r="K11" s="1">
@@ -1999,7 +2248,7 @@
         <v>2</v>
       </c>
       <c r="G12" s="1">
-        <f t="shared" ref="G12:G13" si="8">29085*0.95</f>
+        <f t="shared" ref="G12:G13" si="9">29085*0.95</f>
         <v>27630.75</v>
       </c>
       <c r="H12" s="1">
@@ -2007,15 +2256,15 @@
         <v>5235.3</v>
       </c>
       <c r="I12" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>0.18947368421052632</v>
       </c>
       <c r="J12" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.3902839483887058E-4</v>
       </c>
       <c r="K12" s="1">
-        <f t="shared" ref="K12:K13" si="9">(I12+J12/2)/(J12+1)-$C$5/(J12+1)*SQRT(I12*(1-I12)/G12+J12/(4*G12))</f>
+        <f t="shared" ref="K12:K13" si="10">(I12+J12/2)/(J12+1)-$C$5/(J12+1)*SQRT(I12*(1-I12)/G12+J12/(4*G12))</f>
         <v>0.18034480649920773</v>
       </c>
       <c r="L12" s="1">
@@ -2035,7 +2284,7 @@
         <v>3</v>
       </c>
       <c r="G13" s="1">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>27630.75</v>
       </c>
       <c r="H13" s="1">
@@ -2043,15 +2292,15 @@
         <v>872.55</v>
       </c>
       <c r="I13" s="1">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3.1578947368421054E-2</v>
       </c>
       <c r="J13" s="1">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1.3902839483887058E-4</v>
       </c>
       <c r="K13" s="1">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>2.7549225740961719E-2</v>
       </c>
       <c r="L13" s="1">
@@ -2190,7 +2439,7 @@
     </row>
     <row r="25" spans="1:24">
       <c r="A25" s="1" t="str">
-        <f t="shared" ref="A25:A42" si="10">B25&amp;"_"&amp;E25</f>
+        <f t="shared" ref="A25:A42" si="11">B25&amp;"_"&amp;E25</f>
         <v>incidence_clin_2</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -2203,7 +2452,7 @@
         <v>5</v>
       </c>
       <c r="E25" s="1">
-        <f t="shared" ref="E25:E42" si="11">FLOOR(AVERAGE(C25,D25), 1)</f>
+        <f t="shared" ref="E25:E42" si="12">FLOOR(AVERAGE(C25,D25), 1)</f>
         <v>2</v>
       </c>
       <c r="F25" s="1">
@@ -2214,7 +2463,7 @@
         <v>10087170.893440001</v>
       </c>
       <c r="H25" s="1">
-        <f t="shared" ref="H25:H42" si="12">K25*G25/$B$21</f>
+        <f t="shared" ref="H25:H42" si="13">K25*G25/$B$21</f>
         <v>10.087170893440002</v>
       </c>
       <c r="I25" s="1">
@@ -2255,7 +2504,7 @@
     </row>
     <row r="26" spans="1:24">
       <c r="A26" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_7</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -2269,45 +2518,45 @@
         <v>10</v>
       </c>
       <c r="E26" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>7</v>
       </c>
       <c r="F26" s="1">
         <v>98204</v>
       </c>
       <c r="G26" s="1">
-        <f t="shared" ref="G26:G42" si="13">F26/$B$17*$B$18*($B$20-$B$19+1)</f>
+        <f t="shared" ref="G26:G42" si="14">F26/$B$17*$B$18*($B$20-$B$19+1)</f>
         <v>11734748.512359999</v>
       </c>
       <c r="H26" s="1">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>11.734748512359999</v>
       </c>
       <c r="I26" s="1">
-        <f t="shared" ref="I26:I42" si="14">MAX(0, K26-0.05)*G26/$B$21</f>
+        <f t="shared" ref="I26:I42" si="15">MAX(0, K26-0.05)*G26/$B$21</f>
         <v>5.8673742561799997</v>
       </c>
       <c r="J26" s="1">
-        <f t="shared" ref="J26:J42" si="15">(K26+0.05)*G26/$B$21</f>
+        <f t="shared" ref="J26:J42" si="16">(K26+0.05)*G26/$B$21</f>
         <v>17.602122768539999</v>
       </c>
       <c r="K26" s="1">
         <v>0.1</v>
       </c>
       <c r="M26" s="1">
-        <f t="shared" ref="M26:M42" si="16">IFERROR(0.5*_xlfn.CHISQ.INV($C$4/2,2*I26)/$G26*$B$21, 0)</f>
+        <f t="shared" ref="M26:M42" si="17">IFERROR(0.5*_xlfn.CHISQ.INV($C$4/2,2*I26)/$G26*$B$21, 0)</f>
         <v>4.254340947499706E-3</v>
       </c>
       <c r="N26" s="1">
-        <f t="shared" ref="N26:N42" si="17">IF(M26&lt;1, -0.001,M26)</f>
+        <f t="shared" ref="N26:N42" si="18">IF(M26&lt;1, -0.001,M26)</f>
         <v>-1E-3</v>
       </c>
       <c r="O26" s="1">
-        <f t="shared" ref="O26:O42" si="18">IFERROR(0.5*_xlfn.CHISQ.INV(1-$C$4/2,2*($J26+1))/$G26*$B$21, 0)</f>
+        <f t="shared" ref="O26:O42" si="19">IFERROR(0.5*_xlfn.CHISQ.INV(1-$C$4/2,2*($J26+1))/$G26*$B$21, 0)</f>
         <v>0.34176539057413913</v>
       </c>
       <c r="Q26" s="1">
-        <f t="shared" ref="Q26:Q42" si="19">K26/$B$21*(D26-C26)</f>
+        <f t="shared" ref="Q26:Q42" si="20">K26/$B$21*(D26-C26)</f>
         <v>4.9999999999999996E-6</v>
       </c>
       <c r="R26" s="1">
@@ -2317,7 +2566,7 @@
     </row>
     <row r="27" spans="1:24">
       <c r="A27" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_12</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -2327,49 +2576,49 @@
         <v>10</v>
       </c>
       <c r="D27" s="1">
-        <f t="shared" ref="D27:D41" si="20">C28</f>
+        <f t="shared" ref="D27:D41" si="21">C28</f>
         <v>15</v>
       </c>
       <c r="E27" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>12</v>
       </c>
       <c r="F27" s="1">
         <v>102304</v>
       </c>
       <c r="G27" s="1">
+        <f t="shared" si="14"/>
+        <v>12224672.231360001</v>
+      </c>
+      <c r="H27" s="1">
         <f t="shared" si="13"/>
-        <v>12224672.231360001</v>
-      </c>
-      <c r="H27" s="1">
-        <f t="shared" si="12"/>
         <v>0</v>
       </c>
       <c r="I27" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>0</v>
       </c>
       <c r="J27" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>6.1123361156800007</v>
       </c>
       <c r="K27" s="1">
         <v>0</v>
       </c>
       <c r="M27" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="N27" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-1E-3</v>
       </c>
       <c r="O27" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.18182240036888692</v>
       </c>
       <c r="Q27" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>0</v>
       </c>
       <c r="R27" s="1">
@@ -2379,7 +2628,7 @@
     </row>
     <row r="28" spans="1:24">
       <c r="A28" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_17</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -2389,49 +2638,49 @@
         <v>15</v>
       </c>
       <c r="D28" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>20</v>
       </c>
       <c r="E28" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>17</v>
       </c>
       <c r="F28" s="1">
         <v>93845</v>
       </c>
       <c r="G28" s="1">
+        <f t="shared" si="14"/>
+        <v>11213875.95355</v>
+      </c>
+      <c r="H28" s="1">
         <f t="shared" si="13"/>
-        <v>11213875.95355</v>
-      </c>
-      <c r="H28" s="1">
-        <f t="shared" si="12"/>
         <v>11.213875953550001</v>
       </c>
       <c r="I28" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>5.6069379767750007</v>
       </c>
       <c r="J28" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>16.820813930325002</v>
       </c>
       <c r="K28" s="1">
         <v>0.1</v>
       </c>
       <c r="M28" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>4.4519505398077797E-3</v>
       </c>
       <c r="N28" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-1E-3</v>
       </c>
       <c r="O28" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.34466310103500203</v>
       </c>
       <c r="Q28" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>4.9999999999999996E-6</v>
       </c>
       <c r="R28" s="1">
@@ -2441,7 +2690,7 @@
     </row>
     <row r="29" spans="1:24">
       <c r="A29" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_22</v>
       </c>
       <c r="B29" s="1" t="s">
@@ -2451,30 +2700,30 @@
         <v>20</v>
       </c>
       <c r="D29" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>25</v>
       </c>
       <c r="E29" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>22</v>
       </c>
       <c r="F29" s="1">
         <v>80561</v>
       </c>
       <c r="G29" s="1">
+        <f t="shared" si="14"/>
+        <v>9626523.1039899997</v>
+      </c>
+      <c r="H29" s="1">
         <f t="shared" si="13"/>
-        <v>9626523.1039899997</v>
-      </c>
-      <c r="H29" s="1">
-        <f t="shared" si="12"/>
         <v>28.879569311969998</v>
       </c>
       <c r="I29" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>24.066307759975</v>
       </c>
       <c r="J29" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>33.692830863964993</v>
       </c>
       <c r="K29" s="1">
@@ -2485,19 +2734,19 @@
         <v>7.0026509067945388E-3</v>
       </c>
       <c r="M29" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>9.7938196894199095E-2</v>
       </c>
       <c r="N29" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-1E-3</v>
       </c>
       <c r="O29" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.64601481946145045</v>
       </c>
       <c r="Q29" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1.5E-5</v>
       </c>
       <c r="R29" s="1">
@@ -2507,7 +2756,7 @@
     </row>
     <row r="30" spans="1:24">
       <c r="A30" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_27</v>
       </c>
       <c r="B30" s="1" t="s">
@@ -2517,49 +2766,49 @@
         <v>25</v>
       </c>
       <c r="D30" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>30</v>
       </c>
       <c r="E30" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>27</v>
       </c>
       <c r="F30" s="1">
         <v>66320</v>
       </c>
       <c r="G30" s="1">
+        <f t="shared" si="14"/>
+        <v>7924814.8888000008</v>
+      </c>
+      <c r="H30" s="1">
         <f t="shared" si="13"/>
-        <v>7924814.8888000008</v>
-      </c>
-      <c r="H30" s="1">
-        <f t="shared" si="12"/>
         <v>39.624074444000001</v>
       </c>
       <c r="I30" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>35.661666999600001</v>
       </c>
       <c r="J30" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>43.586481888400009</v>
       </c>
       <c r="K30" s="1">
         <v>0.5</v>
       </c>
       <c r="M30" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.21267471914061448</v>
       </c>
       <c r="N30" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-1E-3</v>
       </c>
       <c r="O30" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>0.94989916767749982</v>
       </c>
       <c r="Q30" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>2.5000000000000001E-5</v>
       </c>
       <c r="R30" s="1">
@@ -2569,7 +2818,7 @@
     </row>
     <row r="31" spans="1:24">
       <c r="A31" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_32</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -2579,49 +2828,49 @@
         <v>30</v>
       </c>
       <c r="D31" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>35</v>
       </c>
       <c r="E31" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>32</v>
       </c>
       <c r="F31" s="1">
         <v>56249</v>
       </c>
       <c r="G31" s="1">
+        <f t="shared" si="14"/>
+        <v>6721394.9439099999</v>
+      </c>
+      <c r="H31" s="1">
         <f t="shared" si="13"/>
-        <v>6721394.9439099999</v>
-      </c>
-      <c r="H31" s="1">
-        <f t="shared" si="12"/>
         <v>73.935344383010005</v>
       </c>
       <c r="I31" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>70.574646911054998</v>
       </c>
       <c r="J31" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>77.296041854965011</v>
       </c>
       <c r="K31" s="1">
         <v>1.1000000000000001</v>
       </c>
       <c r="M31" s="1">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v>0.63120633803390602</v>
       </c>
       <c r="N31" s="1">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v>-1E-3</v>
       </c>
       <c r="O31" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>1.7431061741782465</v>
       </c>
       <c r="Q31" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>5.5000000000000009E-5</v>
       </c>
       <c r="R31" s="1">
@@ -2631,7 +2880,7 @@
     </row>
     <row r="32" spans="1:24">
       <c r="A32" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_37</v>
       </c>
       <c r="B32" s="1" t="s">
@@ -2641,30 +2890,30 @@
         <v>35</v>
       </c>
       <c r="D32" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>40</v>
       </c>
       <c r="E32" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>37</v>
       </c>
       <c r="F32" s="1">
         <v>54656</v>
       </c>
       <c r="G32" s="1">
+        <f t="shared" si="14"/>
+        <v>6531041.6550400006</v>
+      </c>
+      <c r="H32" s="1">
         <f t="shared" si="13"/>
-        <v>6531041.6550400006</v>
-      </c>
-      <c r="H32" s="1">
-        <f t="shared" si="12"/>
         <v>143.68291641088004</v>
       </c>
       <c r="I32" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>140.41739558336002</v>
       </c>
       <c r="J32" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>146.94843723840003</v>
       </c>
       <c r="K32" s="1">
@@ -2675,19 +2924,19 @@
         <v>2.1957052888418878E-2</v>
       </c>
       <c r="M32" s="1">
-        <f t="shared" si="16"/>
-        <v>1.5096614770209527</v>
-      </c>
-      <c r="N32" s="1">
         <f t="shared" si="17"/>
         <v>1.5096614770209527</v>
       </c>
+      <c r="N32" s="1">
+        <f t="shared" si="18"/>
+        <v>1.5096614770209527</v>
+      </c>
       <c r="O32" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>3.0550947154719745</v>
       </c>
       <c r="Q32" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1.1000000000000002E-4</v>
       </c>
       <c r="R32" s="1">
@@ -2697,7 +2946,7 @@
     </row>
     <row r="33" spans="1:18">
       <c r="A33" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_42</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -2707,49 +2956,49 @@
         <v>40</v>
       </c>
       <c r="D33" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>45</v>
       </c>
       <c r="E33" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>42</v>
       </c>
       <c r="F33" s="1">
         <v>58958</v>
       </c>
       <c r="G33" s="1">
+        <f t="shared" si="14"/>
+        <v>7045103.0792200007</v>
+      </c>
+      <c r="H33" s="1">
         <f t="shared" si="13"/>
-        <v>7045103.0792200007</v>
-      </c>
-      <c r="H33" s="1">
-        <f t="shared" si="12"/>
         <v>302.93943240646001</v>
       </c>
       <c r="I33" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>299.41688086685002</v>
       </c>
       <c r="J33" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>306.46198394607001</v>
       </c>
       <c r="K33" s="1">
         <v>4.3</v>
       </c>
       <c r="M33" s="1">
-        <f t="shared" si="16"/>
-        <v>3.3552871864818119</v>
-      </c>
-      <c r="N33" s="1">
         <f t="shared" si="17"/>
         <v>3.3552871864818119</v>
       </c>
+      <c r="N33" s="1">
+        <f t="shared" si="18"/>
+        <v>3.3552871864818119</v>
+      </c>
       <c r="O33" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>5.3927965254376069</v>
       </c>
       <c r="Q33" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>2.1499999999999997E-4</v>
       </c>
       <c r="R33" s="1">
@@ -2759,7 +3008,7 @@
     </row>
     <row r="34" spans="1:18">
       <c r="A34" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_47</v>
       </c>
       <c r="B34" s="1" t="s">
@@ -2769,18 +3018,18 @@
         <v>45</v>
       </c>
       <c r="D34" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>50</v>
       </c>
       <c r="E34" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>47</v>
       </c>
       <c r="F34" s="1">
         <v>59622</v>
       </c>
       <c r="G34" s="1">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>7124446.8229799997</v>
       </c>
       <c r="H34" s="1">
@@ -2788,11 +3037,11 @@
         <v>676.82244818309994</v>
       </c>
       <c r="I34" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>673.26022477160996</v>
       </c>
       <c r="J34" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>680.38467159458992</v>
       </c>
       <c r="K34" s="1">
@@ -2803,19 +3052,19 @@
         <v>9.2660309853476744E-2</v>
       </c>
       <c r="M34" s="1">
-        <f t="shared" si="16"/>
-        <v>8.0953120007060804</v>
-      </c>
-      <c r="N34" s="1">
         <f t="shared" si="17"/>
         <v>8.0953120007060804</v>
       </c>
+      <c r="N34" s="1">
+        <f t="shared" si="18"/>
+        <v>8.0953120007060804</v>
+      </c>
       <c r="O34" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>11.050308439923784</v>
       </c>
       <c r="Q34" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>4.7500000000000005E-4</v>
       </c>
       <c r="R34" s="1">
@@ -2825,7 +3074,7 @@
     </row>
     <row r="35" spans="1:18">
       <c r="A35" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_52</v>
       </c>
       <c r="B35" s="1" t="s">
@@ -2835,49 +3084,49 @@
         <v>50</v>
       </c>
       <c r="D35" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>55</v>
       </c>
       <c r="E35" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>52</v>
       </c>
       <c r="F35" s="1">
         <v>54643</v>
       </c>
       <c r="G35" s="1">
+        <f t="shared" si="14"/>
+        <v>6529488.2383699995</v>
+      </c>
+      <c r="H35" s="1">
         <f t="shared" si="13"/>
-        <v>6529488.2383699995</v>
-      </c>
-      <c r="H35" s="1">
-        <f t="shared" si="12"/>
         <v>1207.9553240984499</v>
       </c>
       <c r="I35" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1204.6905799792648</v>
       </c>
       <c r="J35" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1211.2200682176351</v>
       </c>
       <c r="K35" s="1">
         <v>18.5</v>
       </c>
       <c r="M35" s="1">
-        <f t="shared" si="16"/>
-        <v>16.450899786160679</v>
-      </c>
-      <c r="N35" s="1">
         <f t="shared" si="17"/>
         <v>16.450899786160679</v>
       </c>
+      <c r="N35" s="1">
+        <f t="shared" si="18"/>
+        <v>16.450899786160679</v>
+      </c>
       <c r="O35" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>20.708865931030658</v>
       </c>
       <c r="Q35" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>9.2500000000000004E-4</v>
       </c>
       <c r="R35" s="1">
@@ -2887,7 +3136,7 @@
     </row>
     <row r="36" spans="1:18">
       <c r="A36" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_57</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -2897,30 +3146,30 @@
         <v>55</v>
       </c>
       <c r="D36" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>60</v>
       </c>
       <c r="E36" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>57</v>
       </c>
       <c r="F36" s="1">
         <v>49077</v>
       </c>
       <c r="G36" s="1">
+        <f t="shared" si="14"/>
+        <v>5864386.9164300002</v>
+      </c>
+      <c r="H36" s="1">
         <f t="shared" si="13"/>
-        <v>5864386.9164300002</v>
-      </c>
-      <c r="H36" s="1">
-        <f t="shared" si="12"/>
         <v>2011.48471233549</v>
       </c>
       <c r="I36" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2008.5525188772749</v>
       </c>
       <c r="J36" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2014.4169057937047</v>
       </c>
       <c r="K36" s="1">
@@ -2931,19 +3180,19 @@
         <v>0.23066375686826504</v>
       </c>
       <c r="M36" s="1">
-        <f t="shared" si="16"/>
-        <v>31.355881788353273</v>
-      </c>
-      <c r="N36" s="1">
         <f t="shared" si="17"/>
         <v>31.355881788353273</v>
       </c>
+      <c r="N36" s="1">
+        <f t="shared" si="18"/>
+        <v>31.355881788353273</v>
+      </c>
       <c r="O36" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>37.418662813000019</v>
       </c>
       <c r="Q36" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>1.7149999999999999E-3</v>
       </c>
       <c r="R36" s="1">
@@ -2953,7 +3202,7 @@
     </row>
     <row r="37" spans="1:18">
       <c r="A37" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_62</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -2963,49 +3212,49 @@
         <v>60</v>
       </c>
       <c r="D37" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>65</v>
       </c>
       <c r="E37" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>62</v>
       </c>
       <c r="F37" s="1">
         <v>42403</v>
       </c>
       <c r="G37" s="1">
+        <f t="shared" si="14"/>
+        <v>5066886.6967700003</v>
+      </c>
+      <c r="H37" s="1">
         <f t="shared" si="13"/>
-        <v>5066886.6967700003</v>
-      </c>
-      <c r="H37" s="1">
-        <f t="shared" si="12"/>
         <v>2680.3830625913301</v>
       </c>
       <c r="I37" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2677.8496192429452</v>
       </c>
       <c r="J37" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2682.9165059397151</v>
       </c>
       <c r="K37" s="1">
         <v>52.9</v>
       </c>
       <c r="M37" s="1">
-        <f t="shared" si="16"/>
-        <v>48.962568981583438</v>
-      </c>
-      <c r="N37" s="1">
         <f t="shared" si="17"/>
         <v>48.962568981583438</v>
       </c>
+      <c r="N37" s="1">
+        <f t="shared" si="18"/>
+        <v>48.962568981583438</v>
+      </c>
       <c r="O37" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>57.03248272374185</v>
       </c>
       <c r="Q37" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>2.6449999999999998E-3</v>
       </c>
       <c r="R37" s="1">
@@ -3015,7 +3264,7 @@
     </row>
     <row r="38" spans="1:18">
       <c r="A38" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_67</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -3025,30 +3274,30 @@
         <v>65</v>
       </c>
       <c r="D38" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>70</v>
       </c>
       <c r="E38" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>67</v>
       </c>
       <c r="F38" s="1">
         <v>34406</v>
       </c>
       <c r="G38" s="1">
+        <f t="shared" si="14"/>
+        <v>4111296.4575399999</v>
+      </c>
+      <c r="H38" s="1">
         <f t="shared" si="13"/>
-        <v>4111296.4575399999</v>
-      </c>
-      <c r="H38" s="1">
-        <f t="shared" si="12"/>
         <v>3404.15346684312</v>
       </c>
       <c r="I38" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3402.0978186143498</v>
       </c>
       <c r="J38" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>3406.2091150718898</v>
       </c>
       <c r="K38" s="1">
@@ -3059,19 +3308,19 @@
         <v>0.33905227084581235</v>
       </c>
       <c r="M38" s="1">
-        <f t="shared" si="16"/>
-        <v>77.342309223810418</v>
-      </c>
-      <c r="N38" s="1">
         <f t="shared" si="17"/>
         <v>77.342309223810418</v>
       </c>
+      <c r="N38" s="1">
+        <f t="shared" si="18"/>
+        <v>77.342309223810418</v>
+      </c>
       <c r="O38" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>88.507822558360061</v>
       </c>
       <c r="Q38" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>4.1399999999999996E-3</v>
       </c>
       <c r="R38" s="1">
@@ -3081,7 +3330,7 @@
     </row>
     <row r="39" spans="1:18">
       <c r="A39" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_72</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -3091,49 +3340,49 @@
         <v>70</v>
       </c>
       <c r="D39" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>75</v>
       </c>
       <c r="E39" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>72</v>
       </c>
       <c r="F39" s="1">
         <v>26789</v>
       </c>
       <c r="G39" s="1">
+        <f t="shared" si="14"/>
+        <v>3201113.7825100003</v>
+      </c>
+      <c r="H39" s="1">
         <f t="shared" si="13"/>
-        <v>3201113.7825100003</v>
-      </c>
-      <c r="H39" s="1">
-        <f t="shared" si="12"/>
         <v>3492.4151367184104</v>
       </c>
       <c r="I39" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>3490.8145798271553</v>
       </c>
       <c r="J39" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>3494.015693609665</v>
       </c>
       <c r="K39" s="1">
         <v>109.1</v>
       </c>
       <c r="M39" s="1">
-        <f t="shared" si="16"/>
-        <v>102.00634410001473</v>
-      </c>
-      <c r="N39" s="1">
         <f t="shared" si="17"/>
         <v>102.00634410001473</v>
       </c>
+      <c r="N39" s="1">
+        <f t="shared" si="18"/>
+        <v>102.00634410001473</v>
+      </c>
       <c r="O39" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>116.51359947428682</v>
       </c>
       <c r="Q39" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>5.4549999999999998E-3</v>
       </c>
       <c r="R39" s="1">
@@ -3143,7 +3392,7 @@
     </row>
     <row r="40" spans="1:18">
       <c r="A40" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_77</v>
       </c>
       <c r="B40" s="1" t="s">
@@ -3153,30 +3402,30 @@
         <v>75</v>
       </c>
       <c r="D40" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>80</v>
       </c>
       <c r="E40" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>77</v>
       </c>
       <c r="F40" s="1">
         <v>18871</v>
       </c>
       <c r="G40" s="1">
+        <f t="shared" si="14"/>
+        <v>2254963.5368899996</v>
+      </c>
+      <c r="H40" s="1">
         <f t="shared" si="13"/>
-        <v>2254963.5368899996</v>
-      </c>
-      <c r="H40" s="1">
-        <f t="shared" si="12"/>
         <v>2981.061795768579</v>
       </c>
       <c r="I40" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2979.9343140001338</v>
       </c>
       <c r="J40" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2982.1892775370247</v>
       </c>
       <c r="K40" s="1">
@@ -3187,19 +3436,19 @@
         <v>0.24514861979857369</v>
       </c>
       <c r="M40" s="1">
-        <f t="shared" si="16"/>
-        <v>122.92121750008623</v>
-      </c>
-      <c r="N40" s="1">
         <f t="shared" si="17"/>
         <v>122.92121750008623</v>
       </c>
+      <c r="N40" s="1">
+        <f t="shared" si="18"/>
+        <v>122.92121750008623</v>
+      </c>
       <c r="O40" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>141.91891919184286</v>
       </c>
       <c r="Q40" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>6.6099999999999996E-3</v>
       </c>
       <c r="R40" s="1">
@@ -3209,7 +3458,7 @@
     </row>
     <row r="41" spans="1:18">
       <c r="A41" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_82</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -3219,49 +3468,49 @@
         <v>80</v>
       </c>
       <c r="D41" s="1">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v>85</v>
       </c>
       <c r="E41" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>82</v>
       </c>
       <c r="F41" s="1">
         <v>11241</v>
       </c>
       <c r="G41" s="1">
+        <f t="shared" si="14"/>
+        <v>1343227.4451899999</v>
+      </c>
+      <c r="H41" s="1">
         <f t="shared" si="13"/>
-        <v>1343227.4451899999</v>
-      </c>
-      <c r="H41" s="1">
-        <f t="shared" si="12"/>
         <v>2005.43857566867</v>
       </c>
       <c r="I41" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>2004.7669619460751</v>
       </c>
       <c r="J41" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>2006.1101893912653</v>
       </c>
       <c r="K41" s="1">
         <v>149.30000000000001</v>
       </c>
       <c r="M41" s="1">
-        <f t="shared" si="16"/>
-        <v>136.61155641874043</v>
-      </c>
-      <c r="N41" s="1">
         <f t="shared" si="17"/>
         <v>136.61155641874043</v>
       </c>
+      <c r="N41" s="1">
+        <f t="shared" si="18"/>
+        <v>136.61155641874043</v>
+      </c>
       <c r="O41" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>162.74445396561978</v>
       </c>
       <c r="Q41" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>7.4650000000000011E-3</v>
       </c>
       <c r="R41" s="1">
@@ -3271,7 +3520,7 @@
     </row>
     <row r="42" spans="1:18">
       <c r="A42" s="1" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>incidence_clin_92</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -3284,26 +3533,26 @@
         <v>100</v>
       </c>
       <c r="E42" s="1">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>92</v>
       </c>
       <c r="F42" s="1">
         <v>7435</v>
       </c>
       <c r="G42" s="1">
+        <f t="shared" si="14"/>
+        <v>888434.84165000007</v>
+      </c>
+      <c r="H42" s="1">
         <f t="shared" si="13"/>
-        <v>888434.84165000007</v>
-      </c>
-      <c r="H42" s="1">
-        <f t="shared" si="12"/>
         <v>1258.9121706180499</v>
       </c>
       <c r="I42" s="1">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>1258.4679531972249</v>
       </c>
       <c r="J42" s="1">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v>1259.3563880388751</v>
       </c>
       <c r="K42" s="1">
@@ -3314,19 +3563,19 @@
         <v>6.1891217905532488E-2</v>
       </c>
       <c r="M42" s="1">
-        <f t="shared" si="16"/>
-        <v>126.59273939334641</v>
-      </c>
-      <c r="N42" s="1">
         <f t="shared" si="17"/>
         <v>126.59273939334641</v>
       </c>
+      <c r="N42" s="1">
+        <f t="shared" si="18"/>
+        <v>126.59273939334641</v>
+      </c>
       <c r="O42" s="1">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v>157.89999500379088</v>
       </c>
       <c r="Q42" s="1">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v>2.1254999999999996E-2</v>
       </c>
       <c r="R42" s="1">

</xml_diff>